<commit_message>
nikhil 05 march 816
</commit_message>
<xml_diff>
--- a/data/website stock.xlsx
+++ b/data/website stock.xlsx
@@ -116,7 +116,7 @@
     <t>1016 PATRIKA</t>
   </si>
   <si>
-    <t>1017 PATRIKA</t>
+    <t>1017 PATRIKA  (09.03 8000)</t>
   </si>
   <si>
     <t>1018 PATRIKA</t>
@@ -428,10 +428,10 @@
     <t>2101 PATRIKA (L)-DC</t>
   </si>
   <si>
-    <t>2102 PATRIKA *-* (M)</t>
-  </si>
-  <si>
-    <t>2103 PATRIKA (L)</t>
+    <t>2102 PATRIKA *-* (M) (09.03 1000)</t>
+  </si>
+  <si>
+    <t>2103 PATRIKA (L) (09.03 2000)</t>
   </si>
   <si>
     <t>2104 PATRIKA (DCU)</t>
@@ -440,7 +440,7 @@
     <t>2105 PATRIKA (DC)</t>
   </si>
   <si>
-    <t>2106 PATRIKA (L)</t>
+    <t>2106 PATRIKA (L) (09.03 1000)</t>
   </si>
   <si>
     <t>2107 PATRIKA *-* (M)</t>
@@ -449,7 +449,7 @@
     <t>2108 PATRIKA *-* (M) (DCU)</t>
   </si>
   <si>
-    <t>2109 PATRIKA (L)</t>
+    <t>2109 PATRIKA (L) (09.03 1000)</t>
   </si>
   <si>
     <t>2110 PATRIKA (DC)</t>
@@ -461,7 +461,7 @@
     <t>2112 PATRIKA (L)</t>
   </si>
   <si>
-    <t>2113 PATRIKA (L)</t>
+    <t>2113 PATRIKA (L) (09.03 400)</t>
   </si>
   <si>
     <t>2114 PATRIKA (L) (DCU)</t>
@@ -488,7 +488,7 @@
     <t>2121 PATRIKA (DC)</t>
   </si>
   <si>
-    <t>2122 PATRIKA</t>
+    <t>2122 PATRIKA (09.03 800)</t>
   </si>
   <si>
     <t>2123 PATRIKA (DCU)</t>
@@ -500,7 +500,7 @@
     <t>2125 PATRIKA *-* (M)</t>
   </si>
   <si>
-    <t>2126 PATRIKA *-* (M)</t>
+    <t>2126 PATRIKA *-* (M) (09.03 1000)</t>
   </si>
   <si>
     <t>2127 PATRIKA *-* (M) (DCU)</t>
@@ -515,7 +515,7 @@
     <t>2130 PATRIKA *-* (M) (DCU)</t>
   </si>
   <si>
-    <t>2131 PATRIKA *-* (M) (DCU)</t>
+    <t>2131 PATRIKA *-* (M) (DCU) (09.03 1000)</t>
   </si>
   <si>
     <t>2132 PATRIKA *-* (M) (DCU)</t>
@@ -524,7 +524,7 @@
     <t>2133 PATRIKA</t>
   </si>
   <si>
-    <t>2134 PATRIKA *-* (M)</t>
+    <t>2134 PATRIKA *-* (M) (09.03 1000)</t>
   </si>
   <si>
     <t>2135 PATRIKA *-* (M)</t>
@@ -839,7 +839,7 @@
     <t>5076 PATRIKA (JC)</t>
   </si>
   <si>
-    <t>5077 PATRIKA (1000-1500 11.03)</t>
+    <t>5077 PATRIKA (2500 11.03)</t>
   </si>
   <si>
     <t>5078 PATRIKA (DCU)</t>
@@ -860,7 +860,7 @@
     <t>5084 PATRIKA (05 march 4000)</t>
   </si>
   <si>
-    <t>5085 PATRIKA</t>
+    <t>5085 PATRIKA (09.03 2000)</t>
   </si>
   <si>
     <t>5086 PATRIKA (JC) *-* (M+D)</t>
@@ -1007,13 +1007,13 @@
     <t>5516 PATRIKA (JC) *-* (M)</t>
   </si>
   <si>
-    <t>5517 PATRIKA *-* (M) (Patti Aayegi) 2400 09.03</t>
+    <t>5517 PATRIKA *-* (M) (Patti Aayegi)</t>
   </si>
   <si>
     <t>5518 PATRIKA (JC) *-* (M)</t>
   </si>
   <si>
-    <t>5519 PATRIKA *-* (M)</t>
+    <t>5519 PATRIKA *-* (M) (09.03 2500)</t>
   </si>
   <si>
     <t>5520 PATRIKA</t>
@@ -1082,7 +1082,7 @@
     <t>5541 PATRIKA (JC)</t>
   </si>
   <si>
-    <t>5542 PATRIKA</t>
+    <t>5542 PATRIKA (09.03 2500)</t>
   </si>
   <si>
     <t>5543 PATRIKA</t>
@@ -1094,7 +1094,7 @@
     <t>5545 PATRIKA *-* (M) (DC)</t>
   </si>
   <si>
-    <t>5546 PATRIKA</t>
+    <t>5546 PATRIKA (09.03 3200)</t>
   </si>
   <si>
     <t>5547 PATRIKA *-* (M)</t>
@@ -1127,7 +1127,7 @@
     <t>5556 PATRIKA *-* (M)</t>
   </si>
   <si>
-    <t>5557 PATRIKA</t>
+    <t>5557 PATRIKA (09.03 2800)</t>
   </si>
   <si>
     <t>5558 PATRIKA *-* (M)</t>
@@ -1457,7 +1457,7 @@
     <t>6637 PATRIKA</t>
   </si>
   <si>
-    <t>6638 PATRIKA *-* (M)</t>
+    <t>6638 PATRIKA *-* (M) (09.03 1000)</t>
   </si>
   <si>
     <t>6639 PATRIKA</t>
@@ -1532,7 +1532,7 @@
     <t>6661 PATRIKA *-* (M)</t>
   </si>
   <si>
-    <t>6662 PATRIKA</t>
+    <t>6662 PATRIKA (09.03 1000)</t>
   </si>
   <si>
     <t>6663 PATRIKA</t>
@@ -1685,7 +1685,7 @@
     <t>7422 PATRIKA</t>
   </si>
   <si>
-    <t>7423 PATRIKA</t>
+    <t>7423 PATRIKA (09.03 2000)</t>
   </si>
   <si>
     <t>7424 PATRIKA *-* (F)</t>
@@ -2892,16 +2892,16 @@
         <v>13</v>
       </c>
       <c r="B11" s="24">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C11" s="25">
-        <v>153.5</v>
+        <v>150.5</v>
       </c>
       <c r="D11" s="26">
         <v>1.8</v>
       </c>
       <c r="E11" s="27">
-        <v>276.3</v>
+        <v>270.89999999999998</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2943,16 +2943,16 @@
         <v>16</v>
       </c>
       <c r="B14" s="24">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="C14" s="25">
-        <v>138</v>
+        <v>119</v>
       </c>
       <c r="D14" s="26">
         <v>2</v>
       </c>
       <c r="E14" s="27">
-        <v>276</v>
+        <v>238</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -2960,16 +2960,16 @@
         <v>17</v>
       </c>
       <c r="B15" s="24">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C15" s="25">
-        <v>14</v>
+        <v>7</v>
       </c>
       <c r="D15" s="26">
         <v>2</v>
       </c>
       <c r="E15" s="27">
-        <v>28</v>
+        <v>14</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -3107,16 +3107,16 @@
         <v>26</v>
       </c>
       <c r="B24" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C24" s="25">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="D24" s="26">
         <v>1.8</v>
       </c>
       <c r="E24" s="27">
-        <v>90</v>
+        <v>86.4</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -3124,16 +3124,16 @@
         <v>27</v>
       </c>
       <c r="B25" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C25" s="25">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D25" s="26">
         <v>1.65</v>
       </c>
       <c r="E25" s="27">
-        <v>92.4</v>
+        <v>85.8</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -3175,17 +3175,11 @@
         <v>30</v>
       </c>
       <c r="B28" s="24">
-        <v>51</v>
-      </c>
-      <c r="C28" s="25">
-        <v>4.5</v>
-      </c>
-      <c r="D28" s="26">
-        <v>2</v>
-      </c>
-      <c r="E28" s="27">
-        <v>9</v>
-      </c>
+        <v>53</v>
+      </c>
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
+      <c r="E28" s="28"/>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="23" t="s">
@@ -3288,16 +3282,16 @@
         <v>37</v>
       </c>
       <c r="B35" s="24">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C35" s="25">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="D35" s="26">
         <v>2.2999999999999998</v>
       </c>
       <c r="E35" s="27">
-        <v>144.9</v>
+        <v>135.69999999999999</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -3373,16 +3367,16 @@
         <v>42</v>
       </c>
       <c r="B40" s="24">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C40" s="25">
-        <v>35</v>
+        <v>29.5</v>
       </c>
       <c r="D40" s="26">
         <v>2.14</v>
       </c>
       <c r="E40" s="27">
-        <v>74.900000000000006</v>
+        <v>63.13</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -3424,16 +3418,16 @@
         <v>45</v>
       </c>
       <c r="B43" s="24">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C43" s="25">
-        <v>120.5</v>
+        <v>113.5</v>
       </c>
       <c r="D43" s="26">
         <v>2.4700000000000002</v>
       </c>
       <c r="E43" s="27">
-        <v>297.08</v>
+        <v>279.83</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -3492,16 +3486,16 @@
         <v>49</v>
       </c>
       <c r="B47" s="24">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C47" s="25">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="D47" s="26">
         <v>1.27</v>
       </c>
       <c r="E47" s="27">
-        <v>124.42</v>
+        <v>121.88</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
@@ -3509,16 +3503,16 @@
         <v>50</v>
       </c>
       <c r="B48" s="24">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C48" s="25">
-        <v>1.35</v>
+        <v>0.35</v>
       </c>
       <c r="D48" s="26">
-        <v>1.39</v>
+        <v>1.69</v>
       </c>
       <c r="E48" s="27">
-        <v>1.87</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -3560,16 +3554,16 @@
         <v>53</v>
       </c>
       <c r="B51" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C51" s="25">
-        <v>165.5</v>
+        <v>162.5</v>
       </c>
       <c r="D51" s="26">
         <v>1.8</v>
       </c>
       <c r="E51" s="27">
-        <v>297.89999999999998</v>
+        <v>292.5</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -3628,16 +3622,16 @@
         <v>57</v>
       </c>
       <c r="B55" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C55" s="25">
-        <v>242.65</v>
+        <v>242.15</v>
       </c>
       <c r="D55" s="26">
         <v>2.75</v>
       </c>
       <c r="E55" s="27">
-        <v>667.29</v>
+        <v>665.91</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -3724,16 +3718,16 @@
         <v>63</v>
       </c>
       <c r="B61" s="24">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C61" s="25">
-        <v>1008.5</v>
+        <v>1006.5</v>
       </c>
       <c r="D61" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E61" s="27">
-        <v>1149.02</v>
+        <v>1146.75</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -3758,16 +3752,16 @@
         <v>65</v>
       </c>
       <c r="B63" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C63" s="25">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="D63" s="26">
         <v>1.65</v>
       </c>
       <c r="E63" s="27">
-        <v>84.15</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.25">
@@ -3803,16 +3797,16 @@
         <v>68</v>
       </c>
       <c r="B66" s="24">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C66" s="25">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="D66" s="26">
         <v>1.65</v>
       </c>
       <c r="E66" s="27">
-        <v>99</v>
+        <v>84.15</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.25">
@@ -3865,16 +3859,16 @@
         <v>72</v>
       </c>
       <c r="B70" s="24">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C70" s="25">
-        <v>396</v>
+        <v>392.5</v>
       </c>
       <c r="D70" s="26">
         <v>1.4</v>
       </c>
       <c r="E70" s="27">
-        <v>554.4</v>
+        <v>549.5</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -3882,16 +3876,16 @@
         <v>73</v>
       </c>
       <c r="B71" s="24">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C71" s="25">
-        <v>14.5</v>
+        <v>1.5</v>
       </c>
       <c r="D71" s="26">
         <v>1.4</v>
       </c>
       <c r="E71" s="27">
-        <v>20.3</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -3916,16 +3910,16 @@
         <v>75</v>
       </c>
       <c r="B73" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C73" s="25">
-        <v>540</v>
+        <v>534</v>
       </c>
       <c r="D73" s="26">
         <v>1.4</v>
       </c>
       <c r="E73" s="27">
-        <v>756</v>
+        <v>747.6</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -3933,16 +3927,16 @@
         <v>76</v>
       </c>
       <c r="B74" s="24">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="C74" s="25">
-        <v>168.5</v>
+        <v>100</v>
       </c>
       <c r="D74" s="26">
         <v>1.2</v>
       </c>
       <c r="E74" s="27">
-        <v>202.2</v>
+        <v>120</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -4001,16 +3995,16 @@
         <v>80</v>
       </c>
       <c r="B78" s="24">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C78" s="25">
-        <v>328</v>
+        <v>322</v>
       </c>
       <c r="D78" s="26">
         <v>1.2</v>
       </c>
       <c r="E78" s="27">
-        <v>393.6</v>
+        <v>386.4</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -4103,16 +4097,16 @@
         <v>86</v>
       </c>
       <c r="B84" s="24">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="C84" s="25">
-        <v>1464.5</v>
+        <v>1428.5</v>
       </c>
       <c r="D84" s="26">
         <v>1.3</v>
       </c>
       <c r="E84" s="27">
-        <v>1903.85</v>
+        <v>1857.05</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -4120,16 +4114,16 @@
         <v>87</v>
       </c>
       <c r="B85" s="24">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C85" s="25">
-        <v>1415.5</v>
+        <v>1385.5</v>
       </c>
       <c r="D85" s="26">
         <v>1.3</v>
       </c>
       <c r="E85" s="27">
-        <v>1840.15</v>
+        <v>1801.15</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -4137,16 +4131,16 @@
         <v>88</v>
       </c>
       <c r="B86" s="24">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C86" s="25">
-        <v>1208</v>
+        <v>1206</v>
       </c>
       <c r="D86" s="26">
         <v>1.7</v>
       </c>
       <c r="E86" s="27">
-        <v>2053.6</v>
+        <v>2050.1999999999998</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -4154,16 +4148,16 @@
         <v>89</v>
       </c>
       <c r="B87" s="24">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C87" s="25">
-        <v>776</v>
+        <v>774</v>
       </c>
       <c r="D87" s="26">
         <v>1.7</v>
       </c>
       <c r="E87" s="27">
-        <v>1319.2</v>
+        <v>1315.8</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -4188,16 +4182,16 @@
         <v>91</v>
       </c>
       <c r="B89" s="24">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C89" s="25">
-        <v>245.5</v>
+        <v>233</v>
       </c>
       <c r="D89" s="26">
         <v>1.46</v>
       </c>
       <c r="E89" s="27">
-        <v>358.71</v>
+        <v>340.45</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -4239,16 +4233,16 @@
         <v>94</v>
       </c>
       <c r="B92" s="24">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C92" s="25">
-        <v>744</v>
+        <v>741</v>
       </c>
       <c r="D92" s="26">
         <v>1.81</v>
       </c>
       <c r="E92" s="27">
-        <v>1344.92</v>
+        <v>1339.5</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -4389,16 +4383,16 @@
         <v>104</v>
       </c>
       <c r="B102" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C102" s="25">
-        <v>277</v>
+        <v>269</v>
       </c>
       <c r="D102" s="26">
         <v>0.86</v>
       </c>
       <c r="E102" s="27">
-        <v>237.48</v>
+        <v>230.62</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.25">
@@ -4421,16 +4415,16 @@
         <v>106</v>
       </c>
       <c r="B104" s="24">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C104" s="25">
-        <v>165</v>
+        <v>155</v>
       </c>
       <c r="D104" s="26">
         <v>2.5</v>
       </c>
       <c r="E104" s="27">
-        <v>412.5</v>
+        <v>387.5</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.25">
@@ -4441,13 +4435,13 @@
         <v>20</v>
       </c>
       <c r="C105" s="25">
-        <v>315</v>
+        <v>319</v>
       </c>
       <c r="D105" s="26">
         <v>2.5</v>
       </c>
       <c r="E105" s="27">
-        <v>787.5</v>
+        <v>797.5</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
@@ -4472,16 +4466,16 @@
         <v>109</v>
       </c>
       <c r="B107" s="24">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C107" s="25">
-        <v>325.5</v>
+        <v>323.5</v>
       </c>
       <c r="D107" s="26">
         <v>2.5</v>
       </c>
       <c r="E107" s="27">
-        <v>813.75</v>
+        <v>808.75</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -4506,10 +4500,10 @@
         <v>111</v>
       </c>
       <c r="B109" s="24">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C109" s="25">
-        <v>111.5</v>
+        <v>108</v>
       </c>
       <c r="D109" s="29"/>
       <c r="E109" s="28"/>
@@ -4519,7 +4513,7 @@
         <v>112</v>
       </c>
       <c r="B110" s="24">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C110" s="25">
         <v>358.5</v>
@@ -4532,10 +4526,10 @@
         <v>113</v>
       </c>
       <c r="B111" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C111" s="25">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="D111" s="29"/>
       <c r="E111" s="28"/>
@@ -4558,10 +4552,10 @@
         <v>115</v>
       </c>
       <c r="B113" s="24">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C113" s="25">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="D113" s="29"/>
       <c r="E113" s="28"/>
@@ -4582,10 +4576,10 @@
         <v>117</v>
       </c>
       <c r="B115" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C115" s="25">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="D115" s="29"/>
       <c r="E115" s="28"/>
@@ -4664,10 +4658,10 @@
         <v>123</v>
       </c>
       <c r="B121" s="24">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="C121" s="25">
-        <v>0.11</v>
+        <v>0.1</v>
       </c>
       <c r="D121" s="29"/>
       <c r="E121" s="28"/>
@@ -4697,9 +4691,11 @@
         <v>126</v>
       </c>
       <c r="B124" s="24">
-        <v>272</v>
-      </c>
-      <c r="C124" s="28"/>
+        <v>273</v>
+      </c>
+      <c r="C124" s="25">
+        <v>-0.01</v>
+      </c>
       <c r="D124" s="29"/>
       <c r="E124" s="28"/>
     </row>
@@ -4734,10 +4730,10 @@
         <v>129</v>
       </c>
       <c r="B127" s="24">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="C127" s="25">
-        <v>0.76</v>
+        <v>0.75</v>
       </c>
       <c r="D127" s="29"/>
       <c r="E127" s="28"/>
@@ -4814,16 +4810,16 @@
         <v>135</v>
       </c>
       <c r="B133" s="24">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C133" s="25">
-        <v>10.5</v>
+        <v>10</v>
       </c>
       <c r="D133" s="26">
         <v>12.5</v>
       </c>
       <c r="E133" s="27">
-        <v>131.25</v>
+        <v>125</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.25">
@@ -5429,16 +5425,16 @@
         <v>172</v>
       </c>
       <c r="B170" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C170" s="25">
-        <v>181</v>
+        <v>171</v>
       </c>
       <c r="D170" s="26">
         <v>0.89</v>
       </c>
       <c r="E170" s="27">
-        <v>160.84</v>
+        <v>151.96</v>
       </c>
     </row>
     <row r="171" spans="1:5" x14ac:dyDescent="0.25">
@@ -5463,10 +5459,10 @@
         <v>174</v>
       </c>
       <c r="B172" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C172" s="25">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D172" s="29"/>
       <c r="E172" s="28"/>
@@ -5549,16 +5545,16 @@
         <v>180</v>
       </c>
       <c r="B178" s="24">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C178" s="25">
-        <v>64</v>
+        <v>60</v>
       </c>
       <c r="D178" s="26">
         <v>2.7</v>
       </c>
       <c r="E178" s="27">
-        <v>172.8</v>
+        <v>162</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
@@ -5750,16 +5746,16 @@
         <v>193</v>
       </c>
       <c r="B191" s="24">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C191" s="25">
-        <v>192.81</v>
+        <v>190.31</v>
       </c>
       <c r="D191" s="26">
         <v>2.65</v>
       </c>
       <c r="E191" s="27">
-        <v>510.95</v>
+        <v>504.32</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
@@ -5880,16 +5876,16 @@
         <v>201</v>
       </c>
       <c r="B199" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C199" s="25">
-        <v>16</v>
+        <v>13.5</v>
       </c>
       <c r="D199" s="26">
         <v>4.5</v>
       </c>
       <c r="E199" s="27">
-        <v>72</v>
+        <v>60.75</v>
       </c>
     </row>
     <row r="200" spans="1:5" x14ac:dyDescent="0.25">
@@ -5993,16 +5989,16 @@
         <v>208</v>
       </c>
       <c r="B206" s="24">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C206" s="25">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D206" s="26">
         <v>2.7</v>
       </c>
       <c r="E206" s="27">
-        <v>602.1</v>
+        <v>596.70000000000005</v>
       </c>
     </row>
     <row r="207" spans="1:5" x14ac:dyDescent="0.25">
@@ -6010,16 +6006,16 @@
         <v>209</v>
       </c>
       <c r="B207" s="24">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C207" s="25">
-        <v>35.5</v>
+        <v>32.5</v>
       </c>
       <c r="D207" s="26">
         <v>2.6</v>
       </c>
       <c r="E207" s="27">
-        <v>92.3</v>
+        <v>84.5</v>
       </c>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.25">
@@ -6129,16 +6125,16 @@
         <v>216</v>
       </c>
       <c r="B214" s="24">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="C214" s="25">
-        <v>356.5</v>
+        <v>355</v>
       </c>
       <c r="D214" s="26">
         <v>2.7</v>
       </c>
       <c r="E214" s="27">
-        <v>962.55</v>
+        <v>958.5</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
@@ -6146,16 +6142,16 @@
         <v>217</v>
       </c>
       <c r="B215" s="24">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C215" s="25">
-        <v>266</v>
+        <v>254</v>
       </c>
       <c r="D215" s="26">
         <v>2.7</v>
       </c>
       <c r="E215" s="27">
-        <v>718.2</v>
+        <v>685.8</v>
       </c>
     </row>
     <row r="216" spans="1:5" x14ac:dyDescent="0.25">
@@ -6197,16 +6193,16 @@
         <v>220</v>
       </c>
       <c r="B218" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C218" s="25">
-        <v>39.5</v>
+        <v>39</v>
       </c>
       <c r="D218" s="26">
         <v>3</v>
       </c>
       <c r="E218" s="27">
-        <v>118.5</v>
+        <v>117</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.25">
@@ -6248,16 +6244,16 @@
         <v>223</v>
       </c>
       <c r="B221" s="24">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C221" s="25">
-        <v>84.25</v>
+        <v>188.25</v>
       </c>
       <c r="D221" s="26">
         <v>3.25</v>
       </c>
       <c r="E221" s="27">
-        <v>273.81</v>
+        <v>611.80999999999995</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
@@ -6265,16 +6261,16 @@
         <v>224</v>
       </c>
       <c r="B222" s="24">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C222" s="25">
-        <v>96.5</v>
+        <v>92.5</v>
       </c>
       <c r="D222" s="26">
         <v>3.64</v>
       </c>
       <c r="E222" s="27">
-        <v>351.29</v>
+        <v>336.73</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
@@ -6282,16 +6278,16 @@
         <v>225</v>
       </c>
       <c r="B223" s="24">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C223" s="25">
-        <v>36.5</v>
+        <v>34</v>
       </c>
       <c r="D223" s="26">
         <v>2.7</v>
       </c>
       <c r="E223" s="27">
-        <v>98.55</v>
+        <v>91.8</v>
       </c>
     </row>
     <row r="224" spans="1:5" x14ac:dyDescent="0.25">
@@ -6418,16 +6414,16 @@
         <v>233</v>
       </c>
       <c r="B231" s="24">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C231" s="25">
-        <v>87</v>
+        <v>80</v>
       </c>
       <c r="D231" s="26">
         <v>3.5</v>
       </c>
       <c r="E231" s="27">
-        <v>304.5</v>
+        <v>280</v>
       </c>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.25">
@@ -6446,16 +6442,16 @@
         <v>235</v>
       </c>
       <c r="B233" s="24">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C233" s="25">
-        <v>73.38</v>
+        <v>71.38</v>
       </c>
       <c r="D233" s="26">
         <v>3.25</v>
       </c>
       <c r="E233" s="27">
-        <v>238.49</v>
+        <v>231.99</v>
       </c>
     </row>
     <row r="234" spans="1:5" x14ac:dyDescent="0.25">
@@ -6463,16 +6459,16 @@
         <v>236</v>
       </c>
       <c r="B234" s="24">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C234" s="25">
-        <v>37.5</v>
+        <v>34.5</v>
       </c>
       <c r="D234" s="26">
         <v>3.25</v>
       </c>
       <c r="E234" s="27">
-        <v>121.88</v>
+        <v>112.13</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
@@ -6605,16 +6601,16 @@
         <v>246</v>
       </c>
       <c r="B244" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C244" s="25">
-        <v>17</v>
+        <v>16.5</v>
       </c>
       <c r="D244" s="26">
         <v>5.75</v>
       </c>
       <c r="E244" s="27">
-        <v>97.75</v>
+        <v>94.88</v>
       </c>
     </row>
     <row r="245" spans="1:5" x14ac:dyDescent="0.25">
@@ -6622,16 +6618,16 @@
         <v>247</v>
       </c>
       <c r="B245" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C245" s="25">
-        <v>47</v>
+        <v>48.5</v>
       </c>
       <c r="D245" s="26">
         <v>4.8</v>
       </c>
       <c r="E245" s="27">
-        <v>225.6</v>
+        <v>232.8</v>
       </c>
     </row>
     <row r="246" spans="1:5" x14ac:dyDescent="0.25">
@@ -6656,16 +6652,16 @@
         <v>249</v>
       </c>
       <c r="B247" s="24">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C247" s="25">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="D247" s="26">
         <v>3</v>
       </c>
       <c r="E247" s="27">
-        <v>507</v>
+        <v>498</v>
       </c>
     </row>
     <row r="248" spans="1:5" x14ac:dyDescent="0.25">
@@ -6786,16 +6782,16 @@
         <v>257</v>
       </c>
       <c r="B255" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C255" s="25">
-        <v>57</v>
+        <v>53</v>
       </c>
       <c r="D255" s="26">
         <v>3.5</v>
       </c>
       <c r="E255" s="27">
-        <v>199.5</v>
+        <v>185.5</v>
       </c>
     </row>
     <row r="256" spans="1:5" x14ac:dyDescent="0.25">
@@ -6803,16 +6799,16 @@
         <v>258</v>
       </c>
       <c r="B256" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C256" s="25">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="D256" s="26">
         <v>4.25</v>
       </c>
       <c r="E256" s="27">
-        <v>51</v>
+        <v>29.75</v>
       </c>
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.25">
@@ -6921,16 +6917,16 @@
         <v>266</v>
       </c>
       <c r="B264" s="24">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="C264" s="25">
-        <v>25.5</v>
+        <v>23.5</v>
       </c>
       <c r="D264" s="26">
         <v>6.15</v>
       </c>
       <c r="E264" s="27">
-        <v>156.91</v>
+        <v>144.61000000000001</v>
       </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
@@ -6938,16 +6934,16 @@
         <v>267</v>
       </c>
       <c r="B265" s="24">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="C265" s="25">
-        <v>315</v>
+        <v>303</v>
       </c>
       <c r="D265" s="26">
         <v>4.28</v>
       </c>
       <c r="E265" s="27">
-        <v>1348.2</v>
+        <v>1296.8399999999999</v>
       </c>
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.25">
@@ -7003,13 +6999,13 @@
         <v>81</v>
       </c>
       <c r="C269" s="25">
-        <v>1</v>
+        <v>-8</v>
       </c>
       <c r="D269" s="26">
         <v>3.1</v>
       </c>
       <c r="E269" s="27">
-        <v>3.1</v>
+        <v>-24.8</v>
       </c>
     </row>
     <row r="270" spans="1:5" x14ac:dyDescent="0.25">
@@ -7062,16 +7058,16 @@
         <v>275</v>
       </c>
       <c r="B273" s="24">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C273" s="25">
-        <v>108.37</v>
+        <v>106.37</v>
       </c>
       <c r="D273" s="26">
         <v>4.25</v>
       </c>
       <c r="E273" s="27">
-        <v>460.57</v>
+        <v>452.07</v>
       </c>
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.25">
@@ -7186,16 +7182,16 @@
         <v>283</v>
       </c>
       <c r="B281" s="24">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C281" s="25">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D281" s="26">
         <v>4.8499999999999996</v>
       </c>
       <c r="E281" s="27">
-        <v>746.41</v>
+        <v>727.03</v>
       </c>
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.25">
@@ -7214,16 +7210,16 @@
         <v>285</v>
       </c>
       <c r="B283" s="24">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C283" s="25">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="D283" s="26">
         <v>4.7300000000000004</v>
       </c>
       <c r="E283" s="27">
-        <v>401.71</v>
+        <v>373.36</v>
       </c>
     </row>
     <row r="284" spans="1:5" x14ac:dyDescent="0.25">
@@ -7367,16 +7363,16 @@
         <v>294</v>
       </c>
       <c r="B292" s="24">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C292" s="25">
-        <v>109.5</v>
+        <v>109</v>
       </c>
       <c r="D292" s="26">
         <v>4.5</v>
       </c>
       <c r="E292" s="27">
-        <v>492.75</v>
+        <v>490.5</v>
       </c>
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.25">
@@ -7401,16 +7397,16 @@
         <v>296</v>
       </c>
       <c r="B294" s="24">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C294" s="25">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D294" s="26">
         <v>4.8899999999999997</v>
       </c>
       <c r="E294" s="27">
-        <v>479.02</v>
+        <v>464.36</v>
       </c>
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.25">
@@ -7455,13 +7451,13 @@
         <v>141</v>
       </c>
       <c r="C297" s="25">
-        <v>279.5</v>
+        <v>276.5</v>
       </c>
       <c r="D297" s="26">
         <v>6.07</v>
       </c>
       <c r="E297" s="27">
-        <v>1695.2</v>
+        <v>1677.15</v>
       </c>
     </row>
     <row r="298" spans="1:5" x14ac:dyDescent="0.25">
@@ -7486,16 +7482,16 @@
         <v>301</v>
       </c>
       <c r="B299" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C299" s="25">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D299" s="26">
         <v>4.2699999999999996</v>
       </c>
       <c r="E299" s="27">
-        <v>1037.19</v>
+        <v>1024.3900000000001</v>
       </c>
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.25">
@@ -7554,16 +7550,16 @@
         <v>305</v>
       </c>
       <c r="B303" s="24">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C303" s="25">
-        <v>245.25</v>
+        <v>243.25</v>
       </c>
       <c r="D303" s="26">
         <v>4.3</v>
       </c>
       <c r="E303" s="27">
-        <v>1054.06</v>
+        <v>1045.47</v>
       </c>
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.25">
@@ -7900,16 +7896,16 @@
         <v>327</v>
       </c>
       <c r="B325" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C325" s="25">
-        <v>4.5</v>
+        <v>23.5</v>
       </c>
       <c r="D325" s="26">
-        <v>7.63</v>
+        <v>7.45</v>
       </c>
       <c r="E325" s="27">
-        <v>34.33</v>
+        <v>174.97</v>
       </c>
     </row>
     <row r="326" spans="1:5" x14ac:dyDescent="0.25">
@@ -8034,16 +8030,16 @@
         <v>335</v>
       </c>
       <c r="B333" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C333" s="25">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D333" s="26">
         <v>7.97</v>
       </c>
       <c r="E333" s="27">
-        <v>119.57</v>
+        <v>79.709999999999994</v>
       </c>
     </row>
     <row r="334" spans="1:5" x14ac:dyDescent="0.25">
@@ -8113,16 +8109,16 @@
         <v>340</v>
       </c>
       <c r="B338" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C338" s="25">
-        <v>30.5</v>
+        <v>26.5</v>
       </c>
       <c r="D338" s="26">
         <v>9</v>
       </c>
       <c r="E338" s="27">
-        <v>274.5</v>
+        <v>238.5</v>
       </c>
     </row>
     <row r="339" spans="1:5" x14ac:dyDescent="0.25">
@@ -8158,16 +8154,16 @@
         <v>343</v>
       </c>
       <c r="B341" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C341" s="25">
-        <v>19.5</v>
+        <v>17.5</v>
       </c>
       <c r="D341" s="26">
         <v>9</v>
       </c>
       <c r="E341" s="27">
-        <v>175.5</v>
+        <v>157.5</v>
       </c>
     </row>
     <row r="342" spans="1:5" x14ac:dyDescent="0.25">
@@ -8337,16 +8333,16 @@
         <v>354</v>
       </c>
       <c r="B352" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C352" s="25">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D352" s="26">
         <v>6.4</v>
       </c>
       <c r="E352" s="27">
-        <v>57.6</v>
+        <v>51.2</v>
       </c>
     </row>
     <row r="353" spans="1:5" x14ac:dyDescent="0.25">
@@ -8499,16 +8495,16 @@
         <v>364</v>
       </c>
       <c r="B362" s="24">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C362" s="25">
-        <v>37.5</v>
+        <v>35</v>
       </c>
       <c r="D362" s="26">
         <v>7.76</v>
       </c>
       <c r="E362" s="27">
-        <v>290.94</v>
+        <v>271.54000000000002</v>
       </c>
     </row>
     <row r="363" spans="1:5" x14ac:dyDescent="0.25">
@@ -8638,13 +8634,13 @@
         <v>94</v>
       </c>
       <c r="C370" s="25">
-        <v>98.5</v>
+        <v>95.5</v>
       </c>
       <c r="D370" s="26">
         <v>6.6</v>
       </c>
       <c r="E370" s="27">
-        <v>650.1</v>
+        <v>630.29999999999995</v>
       </c>
     </row>
     <row r="371" spans="1:5" x14ac:dyDescent="0.25">
@@ -8720,16 +8716,16 @@
         <v>377</v>
       </c>
       <c r="B375" s="24">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="C375" s="25">
-        <v>45.83</v>
+        <v>38.83</v>
       </c>
       <c r="D375" s="26">
         <v>4.5</v>
       </c>
       <c r="E375" s="27">
-        <v>206.24</v>
+        <v>174.74</v>
       </c>
     </row>
     <row r="376" spans="1:5" x14ac:dyDescent="0.25">
@@ -8808,13 +8804,13 @@
         <v>14</v>
       </c>
       <c r="C380" s="25">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="D380" s="26">
         <v>9.5</v>
       </c>
       <c r="E380" s="27">
-        <v>137.75</v>
+        <v>133</v>
       </c>
     </row>
     <row r="381" spans="1:5" x14ac:dyDescent="0.25">
@@ -9006,13 +9002,13 @@
         <v>23</v>
       </c>
       <c r="C392" s="25">
-        <v>5.5</v>
+        <v>6.5</v>
       </c>
       <c r="D392" s="26">
         <v>3.6</v>
       </c>
       <c r="E392" s="27">
-        <v>19.8</v>
+        <v>23.4</v>
       </c>
     </row>
     <row r="393" spans="1:5" x14ac:dyDescent="0.25">
@@ -9020,16 +9016,16 @@
         <v>395</v>
       </c>
       <c r="B393" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C393" s="25">
-        <v>10</v>
+        <v>16.5</v>
       </c>
       <c r="D393" s="26">
-        <v>9.85</v>
+        <v>9.8800000000000008</v>
       </c>
       <c r="E393" s="27">
-        <v>98.48</v>
+        <v>162.94999999999999</v>
       </c>
     </row>
     <row r="394" spans="1:5" x14ac:dyDescent="0.25">
@@ -9103,16 +9099,16 @@
         <v>400</v>
       </c>
       <c r="B398" s="24">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C398" s="25">
-        <v>10.5</v>
+        <v>6.5</v>
       </c>
       <c r="D398" s="26">
         <v>6.65</v>
       </c>
       <c r="E398" s="27">
-        <v>69.83</v>
+        <v>43.23</v>
       </c>
     </row>
     <row r="399" spans="1:5" x14ac:dyDescent="0.25">
@@ -9326,16 +9322,16 @@
         <v>415</v>
       </c>
       <c r="B413" s="24">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C413" s="25">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D413" s="26">
         <v>5.2</v>
       </c>
       <c r="E413" s="27">
-        <v>312</v>
+        <v>306.8</v>
       </c>
     </row>
     <row r="414" spans="1:5" x14ac:dyDescent="0.25">
@@ -9378,13 +9374,13 @@
         <v>42</v>
       </c>
       <c r="C416" s="25">
-        <v>20.5</v>
+        <v>48</v>
       </c>
       <c r="D416" s="26">
         <v>5.3</v>
       </c>
       <c r="E416" s="27">
-        <v>108.65</v>
+        <v>254.4</v>
       </c>
     </row>
     <row r="417" spans="1:5" x14ac:dyDescent="0.25">
@@ -10182,9 +10178,15 @@
       <c r="B467" s="24">
         <v>15</v>
       </c>
-      <c r="C467" s="28"/>
-      <c r="D467" s="29"/>
-      <c r="E467" s="28"/>
+      <c r="C467" s="25">
+        <v>10</v>
+      </c>
+      <c r="D467" s="26">
+        <v>15.5</v>
+      </c>
+      <c r="E467" s="27">
+        <v>155</v>
+      </c>
     </row>
     <row r="468" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A468" s="23" t="s">
@@ -10385,16 +10387,16 @@
         <v>482</v>
       </c>
       <c r="B480" s="24">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C480" s="25">
-        <v>-2</v>
+        <v>-7</v>
       </c>
       <c r="D480" s="26">
         <v>10.32</v>
       </c>
       <c r="E480" s="27">
-        <v>-20.64</v>
+        <v>-72.25</v>
       </c>
     </row>
     <row r="481" spans="1:5" x14ac:dyDescent="0.25">
@@ -10737,16 +10739,16 @@
         <v>504</v>
       </c>
       <c r="B502" s="24">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C502" s="25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D502" s="26">
         <v>11.25</v>
       </c>
       <c r="E502" s="27">
-        <v>56.25</v>
+        <v>33.75</v>
       </c>
     </row>
     <row r="503" spans="1:5" x14ac:dyDescent="0.25">
@@ -10857,16 +10859,16 @@
         <v>512</v>
       </c>
       <c r="B510" s="24">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C510" s="25">
-        <v>12.5</v>
+        <v>9.5</v>
       </c>
       <c r="D510" s="26">
         <v>10.17</v>
       </c>
       <c r="E510" s="27">
-        <v>127.08</v>
+        <v>96.58</v>
       </c>
     </row>
     <row r="511" spans="1:5" x14ac:dyDescent="0.25">
@@ -11151,16 +11153,16 @@
         <v>530</v>
       </c>
       <c r="B528" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C528" s="25">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D528" s="26">
         <v>1.4</v>
       </c>
       <c r="E528" s="27">
-        <v>114.8</v>
+        <v>113.4</v>
       </c>
     </row>
     <row r="529" spans="1:5" x14ac:dyDescent="0.25">
@@ -11351,16 +11353,16 @@
         <v>542</v>
       </c>
       <c r="B540" s="24">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C540" s="25">
-        <v>15.5</v>
+        <v>13.5</v>
       </c>
       <c r="D540" s="26">
         <v>2.84</v>
       </c>
       <c r="E540" s="27">
-        <v>44.08</v>
+        <v>38.39</v>
       </c>
     </row>
     <row r="541" spans="1:5" x14ac:dyDescent="0.25">
@@ -11385,16 +11387,16 @@
         <v>544</v>
       </c>
       <c r="B542" s="24">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C542" s="25">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D542" s="26">
         <v>2</v>
       </c>
       <c r="E542" s="27">
-        <v>30</v>
+        <v>26</v>
       </c>
     </row>
     <row r="543" spans="1:5" x14ac:dyDescent="0.25">
@@ -11640,16 +11642,16 @@
         <v>559</v>
       </c>
       <c r="B557" s="24">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C557" s="25">
-        <v>50.2</v>
+        <v>44.7</v>
       </c>
       <c r="D557" s="26">
         <v>3.9</v>
       </c>
       <c r="E557" s="27">
-        <v>195.78</v>
+        <v>174.33</v>
       </c>
     </row>
     <row r="558" spans="1:5" x14ac:dyDescent="0.25">
@@ -11725,17 +11727,11 @@
         <v>564</v>
       </c>
       <c r="B562" s="24">
-        <v>19</v>
-      </c>
-      <c r="C562" s="25">
-        <v>2</v>
-      </c>
-      <c r="D562" s="26">
-        <v>3.6</v>
-      </c>
-      <c r="E562" s="27">
-        <v>7.2</v>
-      </c>
+        <v>20</v>
+      </c>
+      <c r="C562" s="28"/>
+      <c r="D562" s="29"/>
+      <c r="E562" s="28"/>
     </row>
     <row r="563" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A563" s="23" t="s">
@@ -11776,16 +11772,16 @@
         <v>567</v>
       </c>
       <c r="B565" s="24">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C565" s="25">
-        <v>75.25</v>
+        <v>74.25</v>
       </c>
       <c r="D565" s="26">
         <v>2.2999999999999998</v>
       </c>
       <c r="E565" s="27">
-        <v>173.08</v>
+        <v>170.78</v>
       </c>
     </row>
     <row r="566" spans="1:5" x14ac:dyDescent="0.25">
@@ -11827,16 +11823,16 @@
         <v>570</v>
       </c>
       <c r="B568" s="24">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C568" s="25">
-        <v>48</v>
+        <v>47.5</v>
       </c>
       <c r="D568" s="26">
         <v>3.5</v>
       </c>
       <c r="E568" s="27">
-        <v>168</v>
+        <v>166.25</v>
       </c>
     </row>
     <row r="569" spans="1:5" x14ac:dyDescent="0.25">
@@ -11963,16 +11959,16 @@
         <v>578</v>
       </c>
       <c r="B576" s="24">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C576" s="25">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D576" s="26">
         <v>2.71</v>
       </c>
       <c r="E576" s="27">
-        <v>21.69</v>
+        <v>18.98</v>
       </c>
     </row>
     <row r="577" spans="1:5" x14ac:dyDescent="0.25">
@@ -12014,16 +12010,16 @@
         <v>581</v>
       </c>
       <c r="B579" s="24">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C579" s="25">
-        <v>83.5</v>
+        <v>77</v>
       </c>
       <c r="D579" s="26">
         <v>1.4</v>
       </c>
       <c r="E579" s="27">
-        <v>116.9</v>
+        <v>107.8</v>
       </c>
     </row>
     <row r="580" spans="1:5" x14ac:dyDescent="0.25">
@@ -12031,16 +12027,16 @@
         <v>582</v>
       </c>
       <c r="B580" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C580" s="25">
-        <v>84.5</v>
+        <v>83.5</v>
       </c>
       <c r="D580" s="26">
         <v>1.8</v>
       </c>
       <c r="E580" s="27">
-        <v>152.1</v>
+        <v>150.30000000000001</v>
       </c>
     </row>
     <row r="581" spans="1:5" x14ac:dyDescent="0.25">
@@ -12172,10 +12168,10 @@
         <v>591</v>
       </c>
       <c r="B589" s="24">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="C589" s="25">
-        <v>266.5</v>
+        <v>258.5</v>
       </c>
       <c r="D589" s="29"/>
       <c r="E589" s="28"/>
@@ -12185,10 +12181,10 @@
         <v>592</v>
       </c>
       <c r="B590" s="24">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C590" s="25">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="D590" s="29"/>
       <c r="E590" s="28"/>
@@ -12198,10 +12194,10 @@
         <v>593</v>
       </c>
       <c r="B591" s="24">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C591" s="25">
-        <v>227.5</v>
+        <v>221.5</v>
       </c>
       <c r="D591" s="29"/>
       <c r="E591" s="28"/>
@@ -12211,10 +12207,10 @@
         <v>594</v>
       </c>
       <c r="B592" s="24">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C592" s="25">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D592" s="29"/>
       <c r="E592" s="28"/>
@@ -12227,7 +12223,7 @@
         <v>51</v>
       </c>
       <c r="C593" s="25">
-        <v>1</v>
+        <v>109</v>
       </c>
       <c r="D593" s="29"/>
       <c r="E593" s="28"/>
@@ -12237,16 +12233,16 @@
         <v>596</v>
       </c>
       <c r="B594" s="24">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C594" s="25">
-        <v>386</v>
+        <v>378</v>
       </c>
       <c r="D594" s="26">
         <v>0.87</v>
       </c>
       <c r="E594" s="27">
-        <v>335.82</v>
+        <v>328.86</v>
       </c>
     </row>
     <row r="595" spans="1:5" x14ac:dyDescent="0.25">
@@ -12370,10 +12366,10 @@
         <v>605</v>
       </c>
       <c r="B603" s="24">
+        <v>27</v>
+      </c>
+      <c r="C603" s="25">
         <v>26</v>
-      </c>
-      <c r="C603" s="25">
-        <v>66</v>
       </c>
       <c r="D603" s="29"/>
       <c r="E603" s="28"/>
@@ -12383,10 +12379,10 @@
         <v>606</v>
       </c>
       <c r="B604" s="24">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C604" s="25">
-        <v>95</v>
+        <v>53</v>
       </c>
       <c r="D604" s="29"/>
       <c r="E604" s="28"/>
@@ -12396,11 +12392,9 @@
         <v>607</v>
       </c>
       <c r="B605" s="24">
-        <v>31</v>
-      </c>
-      <c r="C605" s="25">
-        <v>23</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C605" s="28"/>
       <c r="D605" s="29"/>
       <c r="E605" s="28"/>
     </row>
@@ -12461,16 +12455,16 @@
         <v>612</v>
       </c>
       <c r="B610" s="24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C610" s="25">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D610" s="26">
         <v>0.73</v>
       </c>
       <c r="E610" s="27">
-        <v>43.07</v>
+        <v>38.69</v>
       </c>
     </row>
     <row r="611" spans="1:5" x14ac:dyDescent="0.25">
@@ -12478,16 +12472,16 @@
         <v>613</v>
       </c>
       <c r="B611" s="24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C611" s="25">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D611" s="26">
         <v>0.73</v>
       </c>
       <c r="E611" s="27">
-        <v>46.72</v>
+        <v>42.34</v>
       </c>
     </row>
     <row r="612" spans="1:5" x14ac:dyDescent="0.25">
@@ -12495,16 +12489,16 @@
         <v>614</v>
       </c>
       <c r="B612" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C612" s="25">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="D612" s="26">
         <v>0.85</v>
       </c>
       <c r="E612" s="27">
-        <v>22.95</v>
+        <v>14.45</v>
       </c>
     </row>
     <row r="613" spans="1:5" x14ac:dyDescent="0.25">
@@ -12512,16 +12506,16 @@
         <v>615</v>
       </c>
       <c r="B613" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C613" s="25">
-        <v>130</v>
+        <v>120</v>
       </c>
       <c r="D613" s="26">
         <v>0.85</v>
       </c>
       <c r="E613" s="27">
-        <v>110.5</v>
+        <v>102</v>
       </c>
     </row>
     <row r="614" spans="1:5" x14ac:dyDescent="0.25">
@@ -12612,16 +12606,16 @@
         <v>621</v>
       </c>
       <c r="B619" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C619" s="25">
-        <v>13</v>
+        <v>12.5</v>
       </c>
       <c r="D619" s="26">
         <v>5.5</v>
       </c>
       <c r="E619" s="27">
-        <v>71.5</v>
+        <v>68.75</v>
       </c>
     </row>
     <row r="620" spans="1:5" x14ac:dyDescent="0.25">
@@ -12731,16 +12725,16 @@
         <v>628</v>
       </c>
       <c r="B626" s="24">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C626" s="25">
-        <v>13.5</v>
+        <v>5.5</v>
       </c>
       <c r="D626" s="26">
         <v>6.5</v>
       </c>
       <c r="E626" s="27">
-        <v>87.75</v>
+        <v>35.75</v>
       </c>
     </row>
     <row r="627" spans="1:5" x14ac:dyDescent="0.25">
@@ -12765,16 +12759,16 @@
         <v>630</v>
       </c>
       <c r="B628" s="24">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C628" s="25">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="D628" s="26">
         <v>2.77</v>
       </c>
       <c r="E628" s="27">
-        <v>191.14</v>
+        <v>177.29</v>
       </c>
     </row>
     <row r="629" spans="1:5" x14ac:dyDescent="0.25">
@@ -12918,16 +12912,16 @@
         <v>639</v>
       </c>
       <c r="B637" s="24">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C637" s="25">
-        <v>151.5</v>
+        <v>148.5</v>
       </c>
       <c r="D637" s="26">
         <v>2.2799999999999998</v>
       </c>
       <c r="E637" s="27">
-        <v>345.42</v>
+        <v>338.58</v>
       </c>
     </row>
     <row r="638" spans="1:5" x14ac:dyDescent="0.25">
@@ -13116,16 +13110,16 @@
         <v>651</v>
       </c>
       <c r="B649" s="24">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C649" s="25">
-        <v>180.86</v>
+        <v>179.86</v>
       </c>
       <c r="D649" s="26">
         <v>1.7</v>
       </c>
       <c r="E649" s="27">
-        <v>307.45999999999998</v>
+        <v>305.76</v>
       </c>
     </row>
     <row r="650" spans="1:5" x14ac:dyDescent="0.25">
@@ -13235,16 +13229,16 @@
         <v>658</v>
       </c>
       <c r="B656" s="24">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C656" s="25">
-        <v>167.5</v>
+        <v>166.5</v>
       </c>
       <c r="D656" s="26">
         <v>2.85</v>
       </c>
       <c r="E656" s="27">
-        <v>477.38</v>
+        <v>474.53</v>
       </c>
     </row>
     <row r="657" spans="1:5" x14ac:dyDescent="0.25">
@@ -13331,16 +13325,16 @@
         <v>664</v>
       </c>
       <c r="B662" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C662" s="25">
-        <v>53.5</v>
+        <v>52</v>
       </c>
       <c r="D662" s="26">
         <v>5.73</v>
       </c>
       <c r="E662" s="27">
-        <v>306.66000000000003</v>
+        <v>298.06</v>
       </c>
     </row>
     <row r="663" spans="1:5" x14ac:dyDescent="0.25">
@@ -13501,16 +13495,16 @@
         <v>674</v>
       </c>
       <c r="B672" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C672" s="25">
-        <v>57.43</v>
+        <v>55.93</v>
       </c>
       <c r="D672" s="26">
         <v>3.6</v>
       </c>
       <c r="E672" s="27">
-        <v>206.75</v>
+        <v>201.35</v>
       </c>
     </row>
     <row r="673" spans="1:5" x14ac:dyDescent="0.25">
@@ -13569,7 +13563,7 @@
         <v>678</v>
       </c>
       <c r="B676" s="24">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C676" s="25">
         <v>58.5</v>
@@ -13654,16 +13648,16 @@
         <v>683</v>
       </c>
       <c r="B681" s="24">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C681" s="25">
-        <v>113.5</v>
+        <v>112</v>
       </c>
       <c r="D681" s="26">
         <v>2.25</v>
       </c>
       <c r="E681" s="27">
-        <v>255.38</v>
+        <v>252</v>
       </c>
     </row>
     <row r="682" spans="1:5" x14ac:dyDescent="0.25">
@@ -13671,16 +13665,16 @@
         <v>684</v>
       </c>
       <c r="B682" s="24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C682" s="25">
-        <v>12.5</v>
+        <v>10.5</v>
       </c>
       <c r="D682" s="26">
         <v>8.84</v>
       </c>
       <c r="E682" s="27">
-        <v>110.48</v>
+        <v>92.8</v>
       </c>
     </row>
     <row r="683" spans="1:5" x14ac:dyDescent="0.25">
@@ -13688,16 +13682,16 @@
         <v>685</v>
       </c>
       <c r="B683" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C683" s="25">
-        <v>51.5</v>
+        <v>51</v>
       </c>
       <c r="D683" s="26">
         <v>2.75</v>
       </c>
       <c r="E683" s="27">
-        <v>141.63</v>
+        <v>140.25</v>
       </c>
     </row>
     <row r="684" spans="1:5" x14ac:dyDescent="0.25">
@@ -13889,10 +13883,10 @@
         <v>698</v>
       </c>
       <c r="B696" s="24">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C696" s="25">
-        <v>63.34</v>
+        <v>59.34</v>
       </c>
       <c r="D696" s="29"/>
       <c r="E696" s="28"/>
@@ -13915,10 +13909,10 @@
         <v>700</v>
       </c>
       <c r="B698" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C698" s="25">
-        <v>94.5</v>
+        <v>84.5</v>
       </c>
       <c r="D698" s="29"/>
       <c r="E698" s="28"/>
@@ -13954,10 +13948,10 @@
         <v>703</v>
       </c>
       <c r="B701" s="24">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C701" s="25">
-        <v>64.5</v>
+        <v>62.5</v>
       </c>
       <c r="D701" s="29"/>
       <c r="E701" s="28"/>
@@ -13989,16 +13983,16 @@
         <v>706</v>
       </c>
       <c r="B704" s="24">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C704" s="25">
-        <v>168.5</v>
+        <v>163.5</v>
       </c>
       <c r="D704" s="26">
         <v>2.93</v>
       </c>
       <c r="E704" s="27">
-        <v>493.99</v>
+        <v>479.33</v>
       </c>
     </row>
     <row r="705" spans="1:5" x14ac:dyDescent="0.25">
@@ -14206,16 +14200,16 @@
         <v>723</v>
       </c>
       <c r="B721" s="24">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C721" s="25">
-        <v>68.5</v>
+        <v>70</v>
       </c>
       <c r="D721" s="26">
         <v>1.1599999999999999</v>
       </c>
       <c r="E721" s="27">
-        <v>79.459999999999994</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="722" spans="1:5" x14ac:dyDescent="0.25">
@@ -14260,10 +14254,10 @@
         <v>727</v>
       </c>
       <c r="B725" s="24">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C725" s="25">
-        <v>-98.15</v>
+        <v>-100.15</v>
       </c>
       <c r="D725" s="29"/>
       <c r="E725" s="28"/>
@@ -14352,16 +14346,16 @@
         <v>733</v>
       </c>
       <c r="B731" s="24">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C731" s="25">
-        <v>63.25</v>
+        <v>59.25</v>
       </c>
       <c r="D731" s="26">
         <v>2.5</v>
       </c>
       <c r="E731" s="27">
-        <v>158.13</v>
+        <v>148.13</v>
       </c>
     </row>
     <row r="732" spans="1:5" x14ac:dyDescent="0.25">
@@ -14431,10 +14425,10 @@
         <v>738</v>
       </c>
       <c r="B736" s="24">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C736" s="25">
-        <v>-517</v>
+        <v>-522.5</v>
       </c>
       <c r="D736" s="29"/>
       <c r="E736" s="28"/>
@@ -14445,11 +14439,11 @@
       </c>
       <c r="B737" s="31"/>
       <c r="C737" s="32">
-        <v>44922</v>
+        <v>44492.97</v>
       </c>
       <c r="D737" s="33"/>
       <c r="E737" s="34">
-        <v>108070.48</v>
+        <v>107563.74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nikhil 06.04 @ 447
</commit_message>
<xml_diff>
--- a/data/website stock.xlsx
+++ b/data/website stock.xlsx
@@ -35,7 +35,7 @@
     <t>Stock Group Summary</t>
   </si>
   <si>
-    <t>1-Jul-25 to 5-Apr-26</t>
+    <t>1-Jul-25 to 6-Apr-26</t>
   </si>
   <si>
     <t/>
@@ -173,7 +173,7 @@
     <t>1035 PATRIKA (DCU)</t>
   </si>
   <si>
-    <t>1101 PATRIKA (O.2591) AJ 16200</t>
+    <t>1101 PATRIKA (O.2591) DC</t>
   </si>
   <si>
     <t>1102 PATRIKA (P.2591)</t>
@@ -464,7 +464,7 @@
     <t>2106 PATRIKA (L) (DC)</t>
   </si>
   <si>
-    <t>2107 PATRIKA *-* (M) 500 04.04</t>
+    <t>2107 PATRIKA *-* (M)</t>
   </si>
   <si>
     <t>2108 PATRIKA *-* (M) (DCU)</t>
@@ -485,7 +485,7 @@
     <t>2113 PATRIKA (L)-(DC)</t>
   </si>
   <si>
-    <t>2114 PATRIKA (L) (DCU) 800 04.04</t>
+    <t>2114 PATRIKA (L) (DCU)</t>
   </si>
   <si>
     <t>2115 PATRIKA (L) (DCU)</t>
@@ -722,7 +722,7 @@
     <t>4295 PATRIKA</t>
   </si>
   <si>
-    <t>4296 PATRIKA (M)-(6 Apr-4800)</t>
+    <t>4296 PATRIKA (M)</t>
   </si>
   <si>
     <t>4297 PATRIKA</t>
@@ -734,7 +734,7 @@
     <t>4298 PATRIKA</t>
   </si>
   <si>
-    <t>4299 PATRIKA (4 APRIL)-DGN CHANGE</t>
+    <t>4299 PATRIKA DSGN CHNG</t>
   </si>
   <si>
     <t>4300 PATRIKA</t>
@@ -752,7 +752,7 @@
     <t>4304 PATRIKA</t>
   </si>
   <si>
-    <t>4305 PATRIKA -(9 Apr-3000)</t>
+    <t>4305 PATRIKA</t>
   </si>
   <si>
     <t>4306 PATRIKA (JC)</t>
@@ -824,7 +824,7 @@
     <t>5062 PATRIKA</t>
   </si>
   <si>
-    <t>5063 PATRIKA -(9 Apr-3000)</t>
+    <t>5063 PATRIKA</t>
   </si>
   <si>
     <t>5064 PATRIKA</t>
@@ -1799,7 +1799,7 @@
     <t>7451 PATRIKA</t>
   </si>
   <si>
-    <t>7452 PATRIKA-(6 Apr)</t>
+    <t>7452 PATRIKA</t>
   </si>
   <si>
     <t>7453 PATRIKA (ECO - 61) Blue</t>
@@ -1949,7 +1949,7 @@
     <t>9309 CARD - B  (DESIGN CHNG)</t>
   </si>
   <si>
-    <t>9309 CARDS *-* (T) (Dc) (2000 05.04)</t>
+    <t>9309 CARDS *-* (T) (Dc)</t>
   </si>
   <si>
     <t>9310 CARDS</t>
@@ -2940,16 +2940,16 @@
         <v>13</v>
       </c>
       <c r="B11" s="24">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="C11" s="25">
-        <v>31.5</v>
+        <v>93.5</v>
       </c>
       <c r="D11" s="26">
         <v>1.8</v>
       </c>
       <c r="E11" s="27">
-        <v>56.7</v>
+        <v>168.3</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -2960,13 +2960,13 @@
         <v>76</v>
       </c>
       <c r="C12" s="25">
-        <v>28</v>
+        <v>98</v>
       </c>
       <c r="D12" s="26">
         <v>1.95</v>
       </c>
       <c r="E12" s="27">
-        <v>54.6</v>
+        <v>191.1</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -2974,16 +2974,16 @@
         <v>15</v>
       </c>
       <c r="B13" s="24">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C13" s="25">
-        <v>37.5</v>
+        <v>105.5</v>
       </c>
       <c r="D13" s="26">
         <v>1.95</v>
       </c>
       <c r="E13" s="27">
-        <v>73.13</v>
+        <v>205.73</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -2991,16 +2991,16 @@
         <v>16</v>
       </c>
       <c r="B14" s="24">
-        <v>167</v>
+        <v>173</v>
       </c>
       <c r="C14" s="25">
-        <v>39.5</v>
+        <v>85.5</v>
       </c>
       <c r="D14" s="26">
         <v>2</v>
       </c>
       <c r="E14" s="27">
-        <v>79</v>
+        <v>171</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -3008,16 +3008,16 @@
         <v>17</v>
       </c>
       <c r="B15" s="24">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C15" s="25">
-        <v>4</v>
+        <v>57</v>
       </c>
       <c r="D15" s="26">
         <v>2</v>
       </c>
       <c r="E15" s="27">
-        <v>8</v>
+        <v>114</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -3042,16 +3042,16 @@
         <v>19</v>
       </c>
       <c r="B17" s="24">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C17" s="25">
-        <v>157</v>
+        <v>154.5</v>
       </c>
       <c r="D17" s="26">
         <v>2.1</v>
       </c>
       <c r="E17" s="27">
-        <v>329.7</v>
+        <v>324.45</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -3104,16 +3104,16 @@
         <v>23</v>
       </c>
       <c r="B21" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C21" s="25">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D21" s="26">
         <v>2.6</v>
       </c>
       <c r="E21" s="27">
-        <v>65</v>
+        <v>59.8</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3138,16 +3138,16 @@
         <v>25</v>
       </c>
       <c r="B23" s="24">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C23" s="25">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="D23" s="26">
         <v>1.8</v>
       </c>
       <c r="E23" s="27">
-        <v>90</v>
+        <v>84.6</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -3155,16 +3155,16 @@
         <v>26</v>
       </c>
       <c r="B24" s="24">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C24" s="25">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="D24" s="26">
         <v>1.8</v>
       </c>
       <c r="E24" s="27">
-        <v>24.3</v>
+        <v>22.5</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -3172,16 +3172,16 @@
         <v>27</v>
       </c>
       <c r="B25" s="24">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C25" s="25">
-        <v>29</v>
+        <v>18.5</v>
       </c>
       <c r="D25" s="26">
         <v>1.65</v>
       </c>
       <c r="E25" s="27">
-        <v>47.85</v>
+        <v>30.53</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -3206,16 +3206,16 @@
         <v>29</v>
       </c>
       <c r="B27" s="24">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C27" s="25">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D27" s="26">
         <v>2</v>
       </c>
       <c r="E27" s="27">
-        <v>106</v>
+        <v>104</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3225,25 +3225,31 @@
       <c r="B28" s="24">
         <v>82</v>
       </c>
-      <c r="C28" s="28"/>
-      <c r="D28" s="29"/>
-      <c r="E28" s="28"/>
+      <c r="C28" s="25">
+        <v>80</v>
+      </c>
+      <c r="D28" s="26">
+        <v>2</v>
+      </c>
+      <c r="E28" s="27">
+        <v>160</v>
+      </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="23" t="s">
         <v>31</v>
       </c>
       <c r="B29" s="24">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C29" s="25">
-        <v>19</v>
+        <v>16.5</v>
       </c>
       <c r="D29" s="26">
         <v>2.6</v>
       </c>
       <c r="E29" s="27">
-        <v>49.4</v>
+        <v>42.9</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -3268,16 +3274,16 @@
         <v>33</v>
       </c>
       <c r="B31" s="24">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C31" s="25">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D31" s="26">
         <v>2.85</v>
       </c>
       <c r="E31" s="27">
-        <v>225.15</v>
+        <v>222.3</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -3330,16 +3336,16 @@
         <v>37</v>
       </c>
       <c r="B35" s="24">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C35" s="25">
-        <v>9</v>
+        <v>1.5</v>
       </c>
       <c r="D35" s="26">
         <v>2.2999999999999998</v>
       </c>
       <c r="E35" s="27">
-        <v>20.7</v>
+        <v>3.45</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -3403,16 +3409,16 @@
         <v>42</v>
       </c>
       <c r="B40" s="24">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="C40" s="25">
-        <v>92.5</v>
+        <v>89</v>
       </c>
       <c r="D40" s="26">
         <v>2.14</v>
       </c>
       <c r="E40" s="27">
-        <v>197.95</v>
+        <v>190.46</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -3420,16 +3426,16 @@
         <v>43</v>
       </c>
       <c r="B41" s="24">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C41" s="25">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="D41" s="26">
         <v>2.14</v>
       </c>
       <c r="E41" s="27">
-        <v>47.08</v>
+        <v>40.659999999999997</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -3437,16 +3443,16 @@
         <v>44</v>
       </c>
       <c r="B42" s="24">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C42" s="25">
-        <v>30.5</v>
+        <v>27.5</v>
       </c>
       <c r="D42" s="26">
         <v>2.4500000000000002</v>
       </c>
       <c r="E42" s="27">
-        <v>74.83</v>
+        <v>67.47</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -3454,27 +3460,33 @@
         <v>45</v>
       </c>
       <c r="B43" s="24">
-        <v>191</v>
-      </c>
-      <c r="C43" s="28"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="28"/>
+        <v>194</v>
+      </c>
+      <c r="C43" s="25">
+        <v>63.5</v>
+      </c>
+      <c r="D43" s="26">
+        <v>2.4700000000000002</v>
+      </c>
+      <c r="E43" s="27">
+        <v>156.9</v>
+      </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A44" s="23" t="s">
         <v>46</v>
       </c>
       <c r="B44" s="24">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C44" s="25">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="D44" s="26">
         <v>2.72</v>
       </c>
       <c r="E44" s="27">
-        <v>40.75</v>
+        <v>32.6</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -3482,16 +3494,16 @@
         <v>47</v>
       </c>
       <c r="B45" s="24">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C45" s="25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D45" s="26">
         <v>2.66</v>
       </c>
       <c r="E45" s="27">
-        <v>13.3</v>
+        <v>7.98</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -3530,13 +3542,13 @@
         <v>146</v>
       </c>
       <c r="C48" s="25">
-        <v>54.5</v>
+        <v>324.5</v>
       </c>
       <c r="D48" s="26">
         <v>1.26</v>
       </c>
       <c r="E48" s="27">
-        <v>68.89</v>
+        <v>408.9</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -3578,16 +3590,16 @@
         <v>53</v>
       </c>
       <c r="B51" s="24">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="C51" s="25">
-        <v>198</v>
+        <v>180</v>
       </c>
       <c r="D51" s="26">
         <v>1.8</v>
       </c>
       <c r="E51" s="27">
-        <v>356.4</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -3595,16 +3607,16 @@
         <v>54</v>
       </c>
       <c r="B52" s="24">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="C52" s="25">
-        <v>83.5</v>
+        <v>73.5</v>
       </c>
       <c r="D52" s="26">
         <v>2.5</v>
       </c>
       <c r="E52" s="27">
-        <v>208.75</v>
+        <v>183.75</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -3612,16 +3624,16 @@
         <v>55</v>
       </c>
       <c r="B53" s="24">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C53" s="25">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="D53" s="26">
         <v>2.5</v>
       </c>
       <c r="E53" s="27">
-        <v>602.5</v>
+        <v>592.5</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -3629,7 +3641,7 @@
         <v>56</v>
       </c>
       <c r="B54" s="24">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C54" s="25">
         <v>76.5</v>
@@ -3646,16 +3658,16 @@
         <v>57</v>
       </c>
       <c r="B55" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C55" s="25">
-        <v>335.65</v>
+        <v>332.65</v>
       </c>
       <c r="D55" s="26">
         <v>2.75</v>
       </c>
       <c r="E55" s="27">
-        <v>923.03</v>
+        <v>914.78</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -3663,16 +3675,16 @@
         <v>58</v>
       </c>
       <c r="B56" s="24">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C56" s="25">
-        <v>86.5</v>
+        <v>79.5</v>
       </c>
       <c r="D56" s="26">
         <v>1.8</v>
       </c>
       <c r="E56" s="27">
-        <v>155.69999999999999</v>
+        <v>143.1</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -3680,16 +3692,16 @@
         <v>59</v>
       </c>
       <c r="B57" s="24">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C57" s="25">
-        <v>72.5</v>
+        <v>71</v>
       </c>
       <c r="D57" s="26">
         <v>1.9</v>
       </c>
       <c r="E57" s="27">
-        <v>137.75</v>
+        <v>134.9</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -3708,16 +3720,16 @@
         <v>61</v>
       </c>
       <c r="B59" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C59" s="25">
-        <v>24.75</v>
+        <v>22.25</v>
       </c>
       <c r="D59" s="26">
         <v>1.9</v>
       </c>
       <c r="E59" s="27">
-        <v>47.03</v>
+        <v>42.28</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -3725,16 +3737,16 @@
         <v>62</v>
       </c>
       <c r="B60" s="24">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C60" s="25">
-        <v>644.5</v>
+        <v>632.5</v>
       </c>
       <c r="D60" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E60" s="27">
-        <v>733.17</v>
+        <v>719.52</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -3742,16 +3754,16 @@
         <v>63</v>
       </c>
       <c r="B61" s="24">
-        <v>170</v>
+        <v>174</v>
       </c>
       <c r="C61" s="25">
-        <v>588.5</v>
+        <v>570.5</v>
       </c>
       <c r="D61" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E61" s="27">
-        <v>670.5</v>
+        <v>649.99</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -3804,16 +3816,16 @@
         <v>67</v>
       </c>
       <c r="B65" s="24">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C65" s="25">
-        <v>488.5</v>
+        <v>479.5</v>
       </c>
       <c r="D65" s="26">
         <v>1.65</v>
       </c>
       <c r="E65" s="27">
-        <v>806.03</v>
+        <v>791.18</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -3849,16 +3861,16 @@
         <v>70</v>
       </c>
       <c r="B68" s="24">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C68" s="25">
-        <v>375.5</v>
+        <v>367</v>
       </c>
       <c r="D68" s="26">
         <v>1.65</v>
       </c>
       <c r="E68" s="27">
-        <v>619.58000000000004</v>
+        <v>605.54999999999995</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -3877,16 +3889,16 @@
         <v>72</v>
       </c>
       <c r="B70" s="24">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="C70" s="25">
-        <v>429.5</v>
+        <v>423.5</v>
       </c>
       <c r="D70" s="26">
         <v>1.4</v>
       </c>
       <c r="E70" s="27">
-        <v>601.29999999999995</v>
+        <v>592.9</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -3894,16 +3906,16 @@
         <v>73</v>
       </c>
       <c r="B71" s="24">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="C71" s="25">
-        <v>659</v>
+        <v>656</v>
       </c>
       <c r="D71" s="26">
         <v>1.4</v>
       </c>
       <c r="E71" s="27">
-        <v>922.6</v>
+        <v>918.4</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -3928,16 +3940,16 @@
         <v>75</v>
       </c>
       <c r="B73" s="24">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="C73" s="25">
-        <v>441.5</v>
+        <v>440.5</v>
       </c>
       <c r="D73" s="26">
         <v>1.4</v>
       </c>
       <c r="E73" s="27">
-        <v>618.1</v>
+        <v>616.70000000000005</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -3945,16 +3957,16 @@
         <v>76</v>
       </c>
       <c r="B74" s="24">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="C74" s="25">
-        <v>176.5</v>
+        <v>173.5</v>
       </c>
       <c r="D74" s="26">
         <v>1.2</v>
       </c>
       <c r="E74" s="27">
-        <v>211.8</v>
+        <v>208.2</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -3962,16 +3974,16 @@
         <v>77</v>
       </c>
       <c r="B75" s="24">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="C75" s="25">
-        <v>306</v>
+        <v>290.5</v>
       </c>
       <c r="D75" s="26">
         <v>1.2</v>
       </c>
       <c r="E75" s="27">
-        <v>367.2</v>
+        <v>348.6</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -3979,16 +3991,16 @@
         <v>78</v>
       </c>
       <c r="B76" s="24">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="C76" s="25">
-        <v>406</v>
+        <v>394</v>
       </c>
       <c r="D76" s="26">
         <v>1.2</v>
       </c>
       <c r="E76" s="27">
-        <v>487.2</v>
+        <v>472.8</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -4013,16 +4025,16 @@
         <v>80</v>
       </c>
       <c r="B78" s="24">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="C78" s="25">
-        <v>364.5</v>
+        <v>343.5</v>
       </c>
       <c r="D78" s="26">
         <v>1.2</v>
       </c>
       <c r="E78" s="27">
-        <v>437.4</v>
+        <v>412.2</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -4030,16 +4042,16 @@
         <v>81</v>
       </c>
       <c r="B79" s="24">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C79" s="25">
-        <v>425</v>
+        <v>409</v>
       </c>
       <c r="D79" s="26">
         <v>1.2</v>
       </c>
       <c r="E79" s="27">
-        <v>510</v>
+        <v>490.8</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -4081,16 +4093,16 @@
         <v>84</v>
       </c>
       <c r="B82" s="24">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C82" s="25">
-        <v>316.5</v>
+        <v>308.5</v>
       </c>
       <c r="D82" s="26">
         <v>1.2</v>
       </c>
       <c r="E82" s="27">
-        <v>379.8</v>
+        <v>370.2</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -4115,16 +4127,16 @@
         <v>86</v>
       </c>
       <c r="B84" s="24">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="C84" s="25">
-        <v>449.5</v>
+        <v>430.5</v>
       </c>
       <c r="D84" s="26">
         <v>1.3</v>
       </c>
       <c r="E84" s="27">
-        <v>584.35</v>
+        <v>559.65</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -4132,16 +4144,16 @@
         <v>87</v>
       </c>
       <c r="B85" s="24">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="C85" s="25">
-        <v>901.5</v>
+        <v>882.5</v>
       </c>
       <c r="D85" s="26">
         <v>1.3</v>
       </c>
       <c r="E85" s="27">
-        <v>1171.95</v>
+        <v>1147.25</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -4200,16 +4212,16 @@
         <v>91</v>
       </c>
       <c r="B89" s="24">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C89" s="25">
-        <v>-63.5</v>
+        <v>-69.5</v>
       </c>
       <c r="D89" s="26">
         <v>1.47</v>
       </c>
       <c r="E89" s="27">
-        <v>-93.43</v>
+        <v>-102.26</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -4234,16 +4246,16 @@
         <v>93</v>
       </c>
       <c r="B91" s="24">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C91" s="25">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D91" s="26">
         <v>1.22</v>
       </c>
       <c r="E91" s="27">
-        <v>64.66</v>
+        <v>57.34</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -4268,16 +4280,16 @@
         <v>95</v>
       </c>
       <c r="B93" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C93" s="25">
-        <v>247.5</v>
+        <v>246.5</v>
       </c>
       <c r="D93" s="26">
         <v>2.27</v>
       </c>
       <c r="E93" s="27">
-        <v>560.85</v>
+        <v>558.59</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -4332,16 +4344,16 @@
         <v>99</v>
       </c>
       <c r="B97" s="24">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C97" s="25">
-        <v>174.5</v>
+        <v>171.5</v>
       </c>
       <c r="D97" s="26">
         <v>0.9</v>
       </c>
       <c r="E97" s="27">
-        <v>157.05000000000001</v>
+        <v>154.35</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -4366,16 +4378,16 @@
         <v>101</v>
       </c>
       <c r="B99" s="24">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="C99" s="25">
-        <v>244</v>
+        <v>215</v>
       </c>
       <c r="D99" s="26">
         <v>1.65</v>
       </c>
       <c r="E99" s="27">
-        <v>402.6</v>
+        <v>354.75</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -4475,16 +4487,16 @@
         <v>108</v>
       </c>
       <c r="B106" s="24">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C106" s="25">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D106" s="26">
         <v>2.5</v>
       </c>
       <c r="E106" s="27">
-        <v>145</v>
+        <v>140</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
@@ -4492,16 +4504,16 @@
         <v>109</v>
       </c>
       <c r="B107" s="24">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C107" s="25">
-        <v>111.5</v>
+        <v>102</v>
       </c>
       <c r="D107" s="26">
         <v>2.5</v>
       </c>
       <c r="E107" s="27">
-        <v>278.75</v>
+        <v>255</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -4509,16 +4521,16 @@
         <v>110</v>
       </c>
       <c r="B108" s="24">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C108" s="25">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D108" s="26">
         <v>2.5</v>
       </c>
       <c r="E108" s="27">
-        <v>230</v>
+        <v>227.5</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
@@ -4526,10 +4538,10 @@
         <v>111</v>
       </c>
       <c r="B109" s="24">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C109" s="25">
-        <v>42</v>
+        <v>33.5</v>
       </c>
       <c r="D109" s="29"/>
       <c r="E109" s="28"/>
@@ -4539,10 +4551,10 @@
         <v>112</v>
       </c>
       <c r="B110" s="24">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C110" s="25">
-        <v>75.5</v>
+        <v>69</v>
       </c>
       <c r="D110" s="29"/>
       <c r="E110" s="28"/>
@@ -4706,10 +4718,10 @@
         <v>125</v>
       </c>
       <c r="B123" s="24">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C123" s="25">
-        <v>-50</v>
+        <v>-56</v>
       </c>
       <c r="D123" s="29"/>
       <c r="E123" s="28"/>
@@ -4749,16 +4761,16 @@
         <v>128</v>
       </c>
       <c r="B126" s="24">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C126" s="25">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D126" s="26">
         <v>1.1499999999999999</v>
       </c>
       <c r="E126" s="27">
-        <v>24.15</v>
+        <v>18.399999999999999</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
@@ -4940,16 +4952,16 @@
         <v>143</v>
       </c>
       <c r="B141" s="24">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C141" s="25">
-        <v>13.5</v>
+        <v>10.5</v>
       </c>
       <c r="D141" s="26">
         <v>12.5</v>
       </c>
       <c r="E141" s="27">
-        <v>168.75</v>
+        <v>131.25</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
@@ -4988,13 +5000,13 @@
         <v>33</v>
       </c>
       <c r="C144" s="25">
-        <v>1.5</v>
+        <v>2.5</v>
       </c>
       <c r="D144" s="26">
         <v>12.5</v>
       </c>
       <c r="E144" s="27">
-        <v>18.75</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.25">
@@ -5075,16 +5087,16 @@
         <v>152</v>
       </c>
       <c r="B150" s="24">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C150" s="25">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="D150" s="26">
         <v>18.5</v>
       </c>
       <c r="E150" s="27">
-        <v>83.25</v>
+        <v>27.75</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
@@ -5092,16 +5104,16 @@
         <v>153</v>
       </c>
       <c r="B151" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C151" s="25">
-        <v>4.5</v>
+        <v>0.5</v>
       </c>
       <c r="D151" s="26">
         <v>18.5</v>
       </c>
       <c r="E151" s="27">
-        <v>83.25</v>
+        <v>9.25</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
@@ -5346,17 +5358,11 @@
         <v>169</v>
       </c>
       <c r="B167" s="24">
-        <v>22</v>
-      </c>
-      <c r="C167" s="25">
-        <v>5.5</v>
-      </c>
-      <c r="D167" s="26">
-        <v>11.5</v>
-      </c>
-      <c r="E167" s="27">
-        <v>63.25</v>
-      </c>
+        <v>24</v>
+      </c>
+      <c r="C167" s="28"/>
+      <c r="D167" s="29"/>
+      <c r="E167" s="28"/>
     </row>
     <row r="168" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A168" s="23" t="s">
@@ -5380,17 +5386,11 @@
         <v>171</v>
       </c>
       <c r="B169" s="24">
-        <v>28</v>
-      </c>
-      <c r="C169" s="25">
-        <v>-1</v>
-      </c>
-      <c r="D169" s="26">
-        <v>11.5</v>
-      </c>
-      <c r="E169" s="27">
-        <v>-11.5</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="C169" s="28"/>
+      <c r="D169" s="29"/>
+      <c r="E169" s="28"/>
     </row>
     <row r="170" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A170" s="23" t="s">
@@ -5498,16 +5498,16 @@
         <v>179</v>
       </c>
       <c r="B177" s="24">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C177" s="25">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="D177" s="26">
-        <v>0.91</v>
+        <v>0.92</v>
       </c>
       <c r="E177" s="27">
-        <v>45.44</v>
+        <v>92.38</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
@@ -5584,16 +5584,16 @@
         <v>185</v>
       </c>
       <c r="B183" s="24">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C183" s="25">
-        <v>26.5</v>
+        <v>25</v>
       </c>
       <c r="D183" s="26">
         <v>3.25</v>
       </c>
       <c r="E183" s="27">
-        <v>86.13</v>
+        <v>81.25</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
@@ -5678,16 +5678,16 @@
         <v>191</v>
       </c>
       <c r="B189" s="24">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C189" s="25">
-        <v>117.5</v>
+        <v>112.5</v>
       </c>
       <c r="D189" s="26">
         <v>2.8</v>
       </c>
       <c r="E189" s="27">
-        <v>329.21</v>
+        <v>315.2</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
@@ -5796,16 +5796,16 @@
         <v>199</v>
       </c>
       <c r="B197" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C197" s="25">
-        <v>7.5</v>
+        <v>6</v>
       </c>
       <c r="D197" s="26">
         <v>2.78</v>
       </c>
       <c r="E197" s="27">
-        <v>20.83</v>
+        <v>16.66</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
@@ -5813,16 +5813,16 @@
         <v>200</v>
       </c>
       <c r="B198" s="24">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C198" s="25">
-        <v>5.31</v>
+        <v>47.81</v>
       </c>
       <c r="D198" s="26">
         <v>2.65</v>
       </c>
       <c r="E198" s="27">
-        <v>14.07</v>
+        <v>126.7</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
@@ -5960,17 +5960,11 @@
         <v>209</v>
       </c>
       <c r="B207" s="24">
-        <v>72</v>
-      </c>
-      <c r="C207" s="25">
-        <v>1</v>
-      </c>
-      <c r="D207" s="26">
-        <v>4.5</v>
-      </c>
-      <c r="E207" s="27">
-        <v>4.5</v>
-      </c>
+        <v>73</v>
+      </c>
+      <c r="C207" s="28"/>
+      <c r="D207" s="29"/>
+      <c r="E207" s="28"/>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="23" t="s">
@@ -6050,16 +6044,16 @@
         <v>215</v>
       </c>
       <c r="B213" s="24">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C213" s="25">
-        <v>128</v>
+        <v>126.5</v>
       </c>
       <c r="D213" s="26">
         <v>2.7</v>
       </c>
       <c r="E213" s="27">
-        <v>345.6</v>
+        <v>341.55</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
@@ -6067,16 +6061,16 @@
         <v>216</v>
       </c>
       <c r="B214" s="24">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C214" s="25">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="D214" s="26">
         <v>2.6</v>
       </c>
       <c r="E214" s="27">
-        <v>166.4</v>
+        <v>161.19999999999999</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
@@ -6169,16 +6163,16 @@
         <v>222</v>
       </c>
       <c r="B220" s="24">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="C220" s="25">
-        <v>16</v>
+        <v>9.5</v>
       </c>
       <c r="D220" s="26">
         <v>3.93</v>
       </c>
       <c r="E220" s="27">
-        <v>62.91</v>
+        <v>37.35</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
@@ -6231,16 +6225,16 @@
         <v>226</v>
       </c>
       <c r="B224" s="24">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C224" s="25">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D224" s="26">
         <v>2.2999999999999998</v>
       </c>
       <c r="E224" s="27">
-        <v>121.9</v>
+        <v>108.1</v>
       </c>
     </row>
     <row r="225" spans="1:5" x14ac:dyDescent="0.25">
@@ -6248,16 +6242,16 @@
         <v>227</v>
       </c>
       <c r="B225" s="24">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C225" s="25">
-        <v>12.5</v>
+        <v>10.5</v>
       </c>
       <c r="D225" s="26">
         <v>4.5</v>
       </c>
       <c r="E225" s="27">
-        <v>56.25</v>
+        <v>47.25</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
@@ -6265,16 +6259,16 @@
         <v>228</v>
       </c>
       <c r="B226" s="24">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C226" s="25">
-        <v>53.5</v>
+        <v>52.5</v>
       </c>
       <c r="D226" s="26">
         <v>3</v>
       </c>
       <c r="E226" s="27">
-        <v>160.5</v>
+        <v>157.5</v>
       </c>
     </row>
     <row r="227" spans="1:5" x14ac:dyDescent="0.25">
@@ -6299,16 +6293,16 @@
         <v>230</v>
       </c>
       <c r="B228" s="24">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C228" s="25">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D228" s="26">
         <v>3.93</v>
       </c>
       <c r="E228" s="27">
-        <v>55.03</v>
+        <v>3.93</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.25">
@@ -6316,16 +6310,16 @@
         <v>231</v>
       </c>
       <c r="B229" s="24">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="C229" s="25">
-        <v>1.25</v>
+        <v>-1.75</v>
       </c>
       <c r="D229" s="26">
         <v>3.25</v>
       </c>
       <c r="E229" s="27">
-        <v>4.0599999999999996</v>
+        <v>-5.69</v>
       </c>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
@@ -6333,16 +6327,16 @@
         <v>232</v>
       </c>
       <c r="B230" s="24">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C230" s="25">
-        <v>34.75</v>
+        <v>32.75</v>
       </c>
       <c r="D230" s="26">
         <v>3.65</v>
       </c>
       <c r="E230" s="27">
-        <v>126.97</v>
+        <v>119.66</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.25">
@@ -6350,16 +6344,16 @@
         <v>233</v>
       </c>
       <c r="B231" s="24">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C231" s="25">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="D231" s="26">
         <v>2.7</v>
       </c>
       <c r="E231" s="27">
-        <v>54</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="232" spans="1:5" x14ac:dyDescent="0.25">
@@ -6395,27 +6389,33 @@
         <v>236</v>
       </c>
       <c r="B234" s="24">
-        <v>76</v>
-      </c>
-      <c r="C234" s="28"/>
-      <c r="D234" s="29"/>
-      <c r="E234" s="28"/>
+        <v>88</v>
+      </c>
+      <c r="C234" s="25">
+        <v>30</v>
+      </c>
+      <c r="D234" s="26">
+        <v>2.66</v>
+      </c>
+      <c r="E234" s="27">
+        <v>79.8</v>
+      </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A235" s="23" t="s">
         <v>237</v>
       </c>
       <c r="B235" s="24">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="C235" s="25">
-        <v>49.5</v>
+        <v>43</v>
       </c>
       <c r="D235" s="26">
         <v>4</v>
       </c>
       <c r="E235" s="27">
-        <v>198</v>
+        <v>172</v>
       </c>
     </row>
     <row r="236" spans="1:5" x14ac:dyDescent="0.25">
@@ -6423,16 +6423,16 @@
         <v>238</v>
       </c>
       <c r="B236" s="24">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C236" s="25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D236" s="26">
         <v>4</v>
       </c>
       <c r="E236" s="27">
-        <v>8</v>
+        <v>4</v>
       </c>
     </row>
     <row r="237" spans="1:5" x14ac:dyDescent="0.25">
@@ -6440,16 +6440,16 @@
         <v>239</v>
       </c>
       <c r="B237" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C237" s="25">
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="D237" s="26">
         <v>3.5</v>
       </c>
       <c r="E237" s="27">
-        <v>54.25</v>
+        <v>52.5</v>
       </c>
     </row>
     <row r="238" spans="1:5" x14ac:dyDescent="0.25">
@@ -6457,16 +6457,16 @@
         <v>240</v>
       </c>
       <c r="B238" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C238" s="25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D238" s="26">
         <v>3.33</v>
       </c>
       <c r="E238" s="27">
-        <v>9.99</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="239" spans="1:5" x14ac:dyDescent="0.25">
@@ -6474,16 +6474,16 @@
         <v>241</v>
       </c>
       <c r="B239" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C239" s="25">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D239" s="26">
         <v>3.96</v>
       </c>
       <c r="E239" s="27">
-        <v>312.58999999999997</v>
+        <v>308.64</v>
       </c>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.25">
@@ -6491,16 +6491,16 @@
         <v>242</v>
       </c>
       <c r="B240" s="24">
-        <v>159</v>
+        <v>168</v>
       </c>
       <c r="C240" s="25">
-        <v>41.5</v>
+        <v>21</v>
       </c>
       <c r="D240" s="26">
         <v>3.5</v>
       </c>
       <c r="E240" s="27">
-        <v>145.25</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.25">
@@ -6519,16 +6519,16 @@
         <v>244</v>
       </c>
       <c r="B242" s="24">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="C242" s="25">
-        <v>95.88</v>
+        <v>87.38</v>
       </c>
       <c r="D242" s="26">
         <v>3.25</v>
       </c>
       <c r="E242" s="27">
-        <v>311.61</v>
+        <v>283.99</v>
       </c>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.25">
@@ -6680,16 +6680,16 @@
         <v>255</v>
       </c>
       <c r="B253" s="24">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C253" s="25">
-        <v>4</v>
+        <v>-1.5</v>
       </c>
       <c r="D253" s="26">
         <v>5.75</v>
       </c>
       <c r="E253" s="27">
-        <v>23</v>
+        <v>-8.6199999999999992</v>
       </c>
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.25">
@@ -6697,17 +6697,11 @@
         <v>256</v>
       </c>
       <c r="B254" s="24">
-        <v>65</v>
-      </c>
-      <c r="C254" s="25">
-        <v>1.5</v>
-      </c>
-      <c r="D254" s="26">
-        <v>4.8</v>
-      </c>
-      <c r="E254" s="27">
-        <v>7.2</v>
-      </c>
+        <v>66</v>
+      </c>
+      <c r="C254" s="28"/>
+      <c r="D254" s="29"/>
+      <c r="E254" s="28"/>
     </row>
     <row r="255" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A255" s="23" t="s">
@@ -6731,16 +6725,16 @@
         <v>258</v>
       </c>
       <c r="B256" s="24">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C256" s="25">
-        <v>0.5</v>
+        <v>-0.5</v>
       </c>
       <c r="D256" s="26">
         <v>3</v>
       </c>
       <c r="E256" s="27">
-        <v>1.5</v>
+        <v>-1.5</v>
       </c>
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.25">
@@ -6748,16 +6742,16 @@
         <v>259</v>
       </c>
       <c r="B257" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C257" s="25">
-        <v>41.18</v>
+        <v>38.18</v>
       </c>
       <c r="D257" s="26">
         <v>3</v>
       </c>
       <c r="E257" s="27">
-        <v>123.54</v>
+        <v>114.54</v>
       </c>
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.25">
@@ -6765,16 +6759,16 @@
         <v>260</v>
       </c>
       <c r="B258" s="24">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="C258" s="25">
-        <v>35.5</v>
+        <v>31.5</v>
       </c>
       <c r="D258" s="26">
         <v>3.8</v>
       </c>
       <c r="E258" s="27">
-        <v>134.9</v>
+        <v>119.7</v>
       </c>
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.25">
@@ -6782,16 +6776,16 @@
         <v>261</v>
       </c>
       <c r="B259" s="24">
-        <v>306</v>
+        <v>311</v>
       </c>
       <c r="C259" s="25">
-        <v>143.5</v>
+        <v>131</v>
       </c>
       <c r="D259" s="26">
         <v>3.9</v>
       </c>
       <c r="E259" s="27">
-        <v>559.65</v>
+        <v>510.9</v>
       </c>
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.25">
@@ -6855,16 +6849,16 @@
         <v>266</v>
       </c>
       <c r="B264" s="24">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C264" s="25">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D264" s="26">
         <v>3.5</v>
       </c>
       <c r="E264" s="27">
-        <v>105</v>
+        <v>98</v>
       </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
@@ -6978,16 +6972,16 @@
         <v>275</v>
       </c>
       <c r="B273" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C273" s="25">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D273" s="26">
         <v>6.18</v>
       </c>
       <c r="E273" s="27">
-        <v>377.23</v>
+        <v>371.04</v>
       </c>
     </row>
     <row r="274" spans="1:5" x14ac:dyDescent="0.25">
@@ -6995,16 +6989,16 @@
         <v>276</v>
       </c>
       <c r="B274" s="24">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="C274" s="25">
-        <v>14</v>
+        <v>-6.5</v>
       </c>
       <c r="D274" s="26">
         <v>4.28</v>
       </c>
       <c r="E274" s="27">
-        <v>59.92</v>
+        <v>-27.82</v>
       </c>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.25">
@@ -7057,16 +7051,16 @@
         <v>280</v>
       </c>
       <c r="B278" s="24">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="C278" s="25">
-        <v>6</v>
+        <v>-2</v>
       </c>
       <c r="D278" s="26">
         <v>3.1</v>
       </c>
       <c r="E278" s="27">
-        <v>18.600000000000001</v>
+        <v>-6.2</v>
       </c>
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.25">
@@ -7085,16 +7079,16 @@
         <v>282</v>
       </c>
       <c r="B280" s="24">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C280" s="25">
-        <v>5.5</v>
+        <v>-4.5</v>
       </c>
       <c r="D280" s="26">
         <v>4.5</v>
       </c>
       <c r="E280" s="27">
-        <v>24.75</v>
+        <v>-20.25</v>
       </c>
     </row>
     <row r="281" spans="1:5" x14ac:dyDescent="0.25">
@@ -7119,16 +7113,16 @@
         <v>284</v>
       </c>
       <c r="B282" s="24">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="C282" s="25">
-        <v>17.37</v>
+        <v>6.37</v>
       </c>
       <c r="D282" s="26">
         <v>4.25</v>
       </c>
       <c r="E282" s="27">
-        <v>73.819999999999993</v>
+        <v>27.07</v>
       </c>
     </row>
     <row r="283" spans="1:5" x14ac:dyDescent="0.25">
@@ -7147,16 +7141,16 @@
         <v>286</v>
       </c>
       <c r="B284" s="24">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C284" s="25">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D284" s="26">
         <v>4.4000000000000004</v>
       </c>
       <c r="E284" s="27">
-        <v>48.42</v>
+        <v>39.619999999999997</v>
       </c>
     </row>
     <row r="285" spans="1:5" x14ac:dyDescent="0.25">
@@ -7164,16 +7158,16 @@
         <v>287</v>
       </c>
       <c r="B285" s="24">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C285" s="25">
-        <v>12.5</v>
+        <v>11.5</v>
       </c>
       <c r="D285" s="26">
         <v>4.28</v>
       </c>
       <c r="E285" s="27">
-        <v>53.5</v>
+        <v>49.22</v>
       </c>
     </row>
     <row r="286" spans="1:5" x14ac:dyDescent="0.25">
@@ -7237,16 +7231,16 @@
         <v>292</v>
       </c>
       <c r="B290" s="24">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C290" s="25">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D290" s="26">
         <v>4.8499999999999996</v>
       </c>
       <c r="E290" s="27">
-        <v>291.19</v>
+        <v>286.33</v>
       </c>
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.25">
@@ -7265,16 +7259,16 @@
         <v>294</v>
       </c>
       <c r="B292" s="24">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C292" s="25">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="D292" s="26">
         <v>4.75</v>
       </c>
       <c r="E292" s="27">
-        <v>85.45</v>
+        <v>23.74</v>
       </c>
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.25">
@@ -7299,16 +7293,16 @@
         <v>296</v>
       </c>
       <c r="B294" s="24">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C294" s="25">
-        <v>46.5</v>
+        <v>45.5</v>
       </c>
       <c r="D294" s="26">
         <v>5.16</v>
       </c>
       <c r="E294" s="27">
-        <v>239.94</v>
+        <v>234.78</v>
       </c>
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.25">
@@ -7333,16 +7327,16 @@
         <v>298</v>
       </c>
       <c r="B296" s="24">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C296" s="25">
-        <v>4</v>
+        <v>3.5</v>
       </c>
       <c r="D296" s="26">
         <v>5</v>
       </c>
       <c r="E296" s="27">
-        <v>20</v>
+        <v>17.5</v>
       </c>
     </row>
     <row r="297" spans="1:5" x14ac:dyDescent="0.25">
@@ -7367,16 +7361,16 @@
         <v>300</v>
       </c>
       <c r="B298" s="24">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C298" s="25">
-        <v>6.75</v>
+        <v>4.25</v>
       </c>
       <c r="D298" s="26">
         <v>5.97</v>
       </c>
       <c r="E298" s="27">
-        <v>40.299999999999997</v>
+        <v>25.37</v>
       </c>
     </row>
     <row r="299" spans="1:5" x14ac:dyDescent="0.25">
@@ -7418,16 +7412,16 @@
         <v>303</v>
       </c>
       <c r="B301" s="24">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C301" s="25">
-        <v>60.5</v>
+        <v>59.5</v>
       </c>
       <c r="D301" s="26">
         <v>4.5</v>
       </c>
       <c r="E301" s="27">
-        <v>272.25</v>
+        <v>267.75</v>
       </c>
     </row>
     <row r="302" spans="1:5" x14ac:dyDescent="0.25">
@@ -7435,16 +7429,16 @@
         <v>304</v>
       </c>
       <c r="B302" s="24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C302" s="25">
-        <v>9</v>
+        <v>8.5</v>
       </c>
       <c r="D302" s="26">
         <v>3.8</v>
       </c>
       <c r="E302" s="27">
-        <v>34.200000000000003</v>
+        <v>32.299999999999997</v>
       </c>
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.25">
@@ -7452,16 +7446,16 @@
         <v>305</v>
       </c>
       <c r="B303" s="24">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C303" s="25">
-        <v>29</v>
+        <v>18.5</v>
       </c>
       <c r="D303" s="26">
         <v>4.8899999999999997</v>
       </c>
       <c r="E303" s="27">
-        <v>141.69999999999999</v>
+        <v>90.39</v>
       </c>
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.25">
@@ -7486,16 +7480,16 @@
         <v>307</v>
       </c>
       <c r="B305" s="24">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C305" s="25">
-        <v>7.5</v>
+        <v>4.5</v>
       </c>
       <c r="D305" s="26">
         <v>3.15</v>
       </c>
       <c r="E305" s="27">
-        <v>23.63</v>
+        <v>14.18</v>
       </c>
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.25">
@@ -7503,16 +7497,16 @@
         <v>308</v>
       </c>
       <c r="B306" s="24">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="C306" s="25">
-        <v>79.5</v>
+        <v>70</v>
       </c>
       <c r="D306" s="26">
-        <v>6.19</v>
+        <v>6.21</v>
       </c>
       <c r="E306" s="27">
-        <v>492.13</v>
+        <v>434.97</v>
       </c>
     </row>
     <row r="307" spans="1:5" x14ac:dyDescent="0.25">
@@ -7520,16 +7514,16 @@
         <v>309</v>
       </c>
       <c r="B307" s="24">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C307" s="25">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="D307" s="26">
         <v>5.53</v>
       </c>
       <c r="E307" s="27">
-        <v>91.22</v>
+        <v>74.64</v>
       </c>
     </row>
     <row r="308" spans="1:5" x14ac:dyDescent="0.25">
@@ -7537,16 +7531,16 @@
         <v>310</v>
       </c>
       <c r="B308" s="24">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C308" s="25">
-        <v>188.5</v>
+        <v>181.5</v>
       </c>
       <c r="D308" s="26">
         <v>4.2699999999999996</v>
       </c>
       <c r="E308" s="27">
-        <v>804.69</v>
+        <v>774.81</v>
       </c>
     </row>
     <row r="309" spans="1:5" x14ac:dyDescent="0.25">
@@ -7582,16 +7576,16 @@
         <v>313</v>
       </c>
       <c r="B311" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C311" s="25">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="D311" s="26">
         <v>4.5</v>
       </c>
       <c r="E311" s="27">
-        <v>135</v>
+        <v>130.5</v>
       </c>
     </row>
     <row r="312" spans="1:5" x14ac:dyDescent="0.25">
@@ -7599,16 +7593,16 @@
         <v>314</v>
       </c>
       <c r="B312" s="24">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="C312" s="25">
-        <v>290.75</v>
+        <v>284.25</v>
       </c>
       <c r="D312" s="26">
         <v>4.3</v>
       </c>
       <c r="E312" s="27">
-        <v>1249.77</v>
+        <v>1221.83</v>
       </c>
     </row>
     <row r="313" spans="1:5" x14ac:dyDescent="0.25">
@@ -7647,13 +7641,13 @@
         <v>67</v>
       </c>
       <c r="C315" s="25">
-        <v>0.5</v>
+        <v>48.5</v>
       </c>
       <c r="D315" s="26">
-        <v>5.14</v>
+        <v>5.13</v>
       </c>
       <c r="E315" s="27">
-        <v>2.57</v>
+        <v>248.81</v>
       </c>
     </row>
     <row r="316" spans="1:5" x14ac:dyDescent="0.25">
@@ -7740,16 +7734,16 @@
         <v>323</v>
       </c>
       <c r="B321" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C321" s="25">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="D321" s="26">
-        <v>7.85</v>
+        <v>7.86</v>
       </c>
       <c r="E321" s="27">
-        <v>19.63</v>
+        <v>3.93</v>
       </c>
     </row>
     <row r="322" spans="1:5" x14ac:dyDescent="0.25">
@@ -7923,16 +7917,16 @@
         <v>336</v>
       </c>
       <c r="B334" s="24">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C334" s="25">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="D334" s="26">
         <v>7.3</v>
       </c>
       <c r="E334" s="27">
-        <v>138.72999999999999</v>
+        <v>116.83</v>
       </c>
     </row>
     <row r="335" spans="1:5" x14ac:dyDescent="0.25">
@@ -8002,16 +7996,16 @@
         <v>341</v>
       </c>
       <c r="B339" s="24">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C339" s="25">
-        <v>34.909999999999997</v>
+        <v>29.91</v>
       </c>
       <c r="D339" s="26">
         <v>4.28</v>
       </c>
       <c r="E339" s="27">
-        <v>149.41</v>
+        <v>128.01</v>
       </c>
     </row>
     <row r="340" spans="1:5" x14ac:dyDescent="0.25">
@@ -8019,16 +8013,16 @@
         <v>342</v>
       </c>
       <c r="B340" s="24">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C340" s="25">
-        <v>67.5</v>
+        <v>64</v>
       </c>
       <c r="D340" s="26">
         <v>4.28</v>
       </c>
       <c r="E340" s="27">
-        <v>288.89999999999998</v>
+        <v>273.92</v>
       </c>
     </row>
     <row r="341" spans="1:5" x14ac:dyDescent="0.25">
@@ -8126,16 +8120,16 @@
         <v>349</v>
       </c>
       <c r="B347" s="24">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="C347" s="25">
-        <v>11</v>
+        <v>1.5</v>
       </c>
       <c r="D347" s="26">
         <v>9</v>
       </c>
       <c r="E347" s="27">
-        <v>99</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="348" spans="1:5" x14ac:dyDescent="0.25">
@@ -8154,16 +8148,16 @@
         <v>351</v>
       </c>
       <c r="B349" s="24">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C349" s="25">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="D349" s="26">
         <v>9</v>
       </c>
       <c r="E349" s="27">
-        <v>40.5</v>
+        <v>13.5</v>
       </c>
     </row>
     <row r="350" spans="1:5" x14ac:dyDescent="0.25">
@@ -8327,33 +8321,27 @@
         <v>362</v>
       </c>
       <c r="B360" s="24">
-        <v>61</v>
-      </c>
-      <c r="C360" s="25">
-        <v>1</v>
-      </c>
-      <c r="D360" s="26">
-        <v>5.94</v>
-      </c>
-      <c r="E360" s="27">
-        <v>5.94</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C360" s="28"/>
+      <c r="D360" s="29"/>
+      <c r="E360" s="28"/>
     </row>
     <row r="361" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A361" s="23" t="s">
         <v>363</v>
       </c>
       <c r="B361" s="24">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C361" s="25">
-        <v>10</v>
+        <v>7.5</v>
       </c>
       <c r="D361" s="26">
         <v>6.4</v>
       </c>
       <c r="E361" s="27">
-        <v>64</v>
+        <v>48</v>
       </c>
     </row>
     <row r="362" spans="1:5" x14ac:dyDescent="0.25">
@@ -8372,16 +8360,16 @@
         <v>365</v>
       </c>
       <c r="B363" s="24">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C363" s="25">
-        <v>18.350000000000001</v>
+        <v>16.350000000000001</v>
       </c>
       <c r="D363" s="26">
         <v>4.75</v>
       </c>
       <c r="E363" s="27">
-        <v>87.16</v>
+        <v>77.66</v>
       </c>
     </row>
     <row r="364" spans="1:5" x14ac:dyDescent="0.25">
@@ -8438,16 +8426,16 @@
         <v>369</v>
       </c>
       <c r="B367" s="24">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C367" s="25">
-        <v>14.5</v>
+        <v>13</v>
       </c>
       <c r="D367" s="26">
         <v>8</v>
       </c>
       <c r="E367" s="27">
-        <v>115.97</v>
+        <v>103.97</v>
       </c>
     </row>
     <row r="368" spans="1:5" x14ac:dyDescent="0.25">
@@ -8590,16 +8578,16 @@
         <v>379</v>
       </c>
       <c r="B377" s="24">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C377" s="25">
-        <v>7</v>
+        <v>4.5</v>
       </c>
       <c r="D377" s="26">
         <v>7.13</v>
       </c>
       <c r="E377" s="27">
-        <v>49.91</v>
+        <v>32.090000000000003</v>
       </c>
     </row>
     <row r="378" spans="1:5" x14ac:dyDescent="0.25">
@@ -8624,16 +8612,16 @@
         <v>381</v>
       </c>
       <c r="B379" s="24">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C379" s="25">
-        <v>30.5</v>
+        <v>16.5</v>
       </c>
       <c r="D379" s="26">
         <v>6.6</v>
       </c>
       <c r="E379" s="27">
-        <v>201.3</v>
+        <v>108.9</v>
       </c>
     </row>
     <row r="380" spans="1:5" x14ac:dyDescent="0.25">
@@ -8692,16 +8680,16 @@
         <v>385</v>
       </c>
       <c r="B383" s="24">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C383" s="25">
-        <v>21.5</v>
+        <v>20.5</v>
       </c>
       <c r="D383" s="26">
         <v>7.31</v>
       </c>
       <c r="E383" s="27">
-        <v>157.27000000000001</v>
+        <v>149.94999999999999</v>
       </c>
     </row>
     <row r="384" spans="1:5" x14ac:dyDescent="0.25">
@@ -8777,16 +8765,16 @@
         <v>390</v>
       </c>
       <c r="B388" s="24">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C388" s="25">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="D388" s="26">
         <v>7</v>
       </c>
       <c r="E388" s="27">
-        <v>73.5</v>
+        <v>59.5</v>
       </c>
     </row>
     <row r="389" spans="1:5" x14ac:dyDescent="0.25">
@@ -8822,16 +8810,16 @@
         <v>393</v>
       </c>
       <c r="B391" s="24">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C391" s="25">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D391" s="26">
         <v>6</v>
       </c>
       <c r="E391" s="27">
-        <v>144</v>
+        <v>120</v>
       </c>
     </row>
     <row r="392" spans="1:5" x14ac:dyDescent="0.25">
@@ -9065,16 +9053,16 @@
         <v>408</v>
       </c>
       <c r="B406" s="24">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="C406" s="25">
-        <v>11.5</v>
+        <v>10.5</v>
       </c>
       <c r="D406" s="26">
         <v>8.5500000000000007</v>
       </c>
       <c r="E406" s="27">
-        <v>98.33</v>
+        <v>89.78</v>
       </c>
     </row>
     <row r="407" spans="1:5" x14ac:dyDescent="0.25">
@@ -9082,16 +9070,16 @@
         <v>409</v>
       </c>
       <c r="B407" s="24">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C407" s="25">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="D407" s="26">
         <v>6.65</v>
       </c>
       <c r="E407" s="27">
-        <v>93.1</v>
+        <v>86.45</v>
       </c>
     </row>
     <row r="408" spans="1:5" x14ac:dyDescent="0.25">
@@ -9172,17 +9160,11 @@
         <v>415</v>
       </c>
       <c r="B413" s="24">
-        <v>61</v>
-      </c>
-      <c r="C413" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="D413" s="26">
-        <v>7</v>
-      </c>
-      <c r="E413" s="27">
-        <v>3.5</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C413" s="28"/>
+      <c r="D413" s="29"/>
+      <c r="E413" s="28"/>
     </row>
     <row r="414" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A414" s="23" t="s">
@@ -9245,16 +9227,16 @@
         <v>420</v>
       </c>
       <c r="B418" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C418" s="25">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="D418" s="26">
         <v>7.13</v>
       </c>
       <c r="E418" s="27">
-        <v>64.17</v>
+        <v>42.78</v>
       </c>
     </row>
     <row r="419" spans="1:5" x14ac:dyDescent="0.25">
@@ -9279,16 +9261,16 @@
         <v>422</v>
       </c>
       <c r="B420" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C420" s="25">
-        <v>51.5</v>
+        <v>47.5</v>
       </c>
       <c r="D420" s="26">
         <v>5.7</v>
       </c>
       <c r="E420" s="27">
-        <v>293.55</v>
+        <v>270.75</v>
       </c>
     </row>
     <row r="421" spans="1:5" x14ac:dyDescent="0.25">
@@ -9369,16 +9351,16 @@
         <v>428</v>
       </c>
       <c r="B426" s="24">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C426" s="25">
-        <v>8</v>
+        <v>6.5</v>
       </c>
       <c r="D426" s="26">
         <v>4.9000000000000004</v>
       </c>
       <c r="E426" s="27">
-        <v>39.200000000000003</v>
+        <v>31.85</v>
       </c>
     </row>
     <row r="427" spans="1:5" x14ac:dyDescent="0.25">
@@ -9460,16 +9442,16 @@
         <v>435</v>
       </c>
       <c r="B433" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C433" s="25">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D433" s="26">
         <v>9</v>
       </c>
       <c r="E433" s="27">
-        <v>13.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="434" spans="1:5" x14ac:dyDescent="0.25">
@@ -9533,17 +9515,11 @@
         <v>440</v>
       </c>
       <c r="B438" s="24">
-        <v>21</v>
-      </c>
-      <c r="C438" s="25">
-        <v>1.5</v>
-      </c>
-      <c r="D438" s="26">
-        <v>6</v>
-      </c>
-      <c r="E438" s="27">
-        <v>9</v>
-      </c>
+        <v>22</v>
+      </c>
+      <c r="C438" s="28"/>
+      <c r="D438" s="29"/>
+      <c r="E438" s="28"/>
     </row>
     <row r="439" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A439" s="23" t="s">
@@ -9717,16 +9693,16 @@
         <v>452</v>
       </c>
       <c r="B450" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C450" s="25">
-        <v>9.5</v>
+        <v>9</v>
       </c>
       <c r="D450" s="26">
         <v>11.75</v>
       </c>
       <c r="E450" s="27">
-        <v>111.63</v>
+        <v>105.75</v>
       </c>
     </row>
     <row r="451" spans="1:5" x14ac:dyDescent="0.25">
@@ -10231,16 +10207,16 @@
         <v>486</v>
       </c>
       <c r="B484" s="24">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C484" s="25">
-        <v>9</v>
+        <v>7.5</v>
       </c>
       <c r="D484" s="26">
         <v>9.5</v>
       </c>
       <c r="E484" s="27">
-        <v>85.5</v>
+        <v>71.25</v>
       </c>
     </row>
     <row r="485" spans="1:5" x14ac:dyDescent="0.25">
@@ -10276,16 +10252,16 @@
         <v>489</v>
       </c>
       <c r="B487" s="24">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="C487" s="25">
-        <v>5.5</v>
+        <v>4</v>
       </c>
       <c r="D487" s="26">
         <v>25</v>
       </c>
       <c r="E487" s="27">
-        <v>137.5</v>
+        <v>100</v>
       </c>
     </row>
     <row r="488" spans="1:5" x14ac:dyDescent="0.25">
@@ -10349,16 +10325,16 @@
         <v>494</v>
       </c>
       <c r="B492" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C492" s="25">
-        <v>3.5</v>
+        <v>0.5</v>
       </c>
       <c r="D492" s="26">
         <v>11.4</v>
       </c>
       <c r="E492" s="27">
-        <v>39.9</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="493" spans="1:5" x14ac:dyDescent="0.25">
@@ -10377,16 +10353,16 @@
         <v>496</v>
       </c>
       <c r="B494" s="24">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C494" s="25">
-        <v>19</v>
+        <v>14.5</v>
       </c>
       <c r="D494" s="26">
         <v>13</v>
       </c>
       <c r="E494" s="27">
-        <v>247</v>
+        <v>188.5</v>
       </c>
     </row>
     <row r="495" spans="1:5" x14ac:dyDescent="0.25">
@@ -10899,16 +10875,16 @@
         <v>530</v>
       </c>
       <c r="B528" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C528" s="25">
-        <v>27.5</v>
+        <v>22.5</v>
       </c>
       <c r="D528" s="26">
         <v>3.8</v>
       </c>
       <c r="E528" s="27">
-        <v>104.5</v>
+        <v>85.5</v>
       </c>
     </row>
     <row r="529" spans="1:5" x14ac:dyDescent="0.25">
@@ -11095,7 +11071,7 @@
         <v>542</v>
       </c>
       <c r="B540" s="24">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C540" s="25">
         <v>30</v>
@@ -11461,16 +11437,16 @@
         <v>564</v>
       </c>
       <c r="B562" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C562" s="25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D562" s="26">
         <v>3.1</v>
       </c>
       <c r="E562" s="27">
-        <v>15.5</v>
+        <v>9.3000000000000007</v>
       </c>
     </row>
     <row r="563" spans="1:5" x14ac:dyDescent="0.25">
@@ -11529,16 +11505,16 @@
         <v>568</v>
       </c>
       <c r="B566" s="24">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="C566" s="25">
-        <v>55</v>
+        <v>41.5</v>
       </c>
       <c r="D566" s="26">
         <v>3.9</v>
       </c>
       <c r="E566" s="27">
-        <v>214.5</v>
+        <v>161.85</v>
       </c>
     </row>
     <row r="567" spans="1:5" x14ac:dyDescent="0.25">
@@ -11580,16 +11556,16 @@
         <v>571</v>
       </c>
       <c r="B569" s="24">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C569" s="25">
-        <v>10.5</v>
+        <v>8.5</v>
       </c>
       <c r="D569" s="26">
         <v>2.66</v>
       </c>
       <c r="E569" s="27">
-        <v>27.93</v>
+        <v>22.61</v>
       </c>
     </row>
     <row r="570" spans="1:5" x14ac:dyDescent="0.25">
@@ -11597,16 +11573,16 @@
         <v>572</v>
       </c>
       <c r="B570" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C570" s="25">
-        <v>11.5</v>
+        <v>10</v>
       </c>
       <c r="D570" s="26">
         <v>2.85</v>
       </c>
       <c r="E570" s="27">
-        <v>32.78</v>
+        <v>28.5</v>
       </c>
     </row>
     <row r="571" spans="1:5" x14ac:dyDescent="0.25">
@@ -11648,16 +11624,16 @@
         <v>575</v>
       </c>
       <c r="B573" s="24">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C573" s="25">
-        <v>5.5</v>
+        <v>1.5</v>
       </c>
       <c r="D573" s="26">
         <v>3.14</v>
       </c>
       <c r="E573" s="27">
-        <v>17.28</v>
+        <v>4.71</v>
       </c>
     </row>
     <row r="574" spans="1:5" x14ac:dyDescent="0.25">
@@ -11795,16 +11771,16 @@
         <v>584</v>
       </c>
       <c r="B582" s="24">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C582" s="25">
-        <v>33.5</v>
+        <v>32.5</v>
       </c>
       <c r="D582" s="26">
         <v>2.66</v>
       </c>
       <c r="E582" s="27">
-        <v>89.11</v>
+        <v>86.45</v>
       </c>
     </row>
     <row r="583" spans="1:5" x14ac:dyDescent="0.25">
@@ -11897,16 +11873,16 @@
         <v>590</v>
       </c>
       <c r="B588" s="24">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C588" s="25">
-        <v>-1</v>
+        <v>-2.5</v>
       </c>
       <c r="D588" s="26">
         <v>1.4</v>
       </c>
       <c r="E588" s="27">
-        <v>-1.4</v>
+        <v>-3.5</v>
       </c>
     </row>
     <row r="589" spans="1:5" x14ac:dyDescent="0.25">
@@ -11914,16 +11890,16 @@
         <v>591</v>
       </c>
       <c r="B589" s="24">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C589" s="25">
-        <v>0.5</v>
+        <v>118.5</v>
       </c>
       <c r="D589" s="26">
         <v>1.8</v>
       </c>
       <c r="E589" s="27">
-        <v>0.9</v>
+        <v>213.3</v>
       </c>
     </row>
     <row r="590" spans="1:5" x14ac:dyDescent="0.25">
@@ -11931,16 +11907,16 @@
         <v>592</v>
       </c>
       <c r="B590" s="24">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C590" s="25">
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="D590" s="26">
         <v>1.2</v>
       </c>
       <c r="E590" s="27">
-        <v>63.6</v>
+        <v>60</v>
       </c>
     </row>
     <row r="591" spans="1:5" x14ac:dyDescent="0.25">
@@ -12081,10 +12057,10 @@
         <v>602</v>
       </c>
       <c r="B600" s="24">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="C600" s="25">
-        <v>-134.5</v>
+        <v>-146.5</v>
       </c>
       <c r="D600" s="29"/>
       <c r="E600" s="28"/>
@@ -12094,10 +12070,10 @@
         <v>603</v>
       </c>
       <c r="B601" s="24">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C601" s="25">
-        <v>-68.5</v>
+        <v>-74.5</v>
       </c>
       <c r="D601" s="29"/>
       <c r="E601" s="28"/>
@@ -12120,10 +12096,10 @@
         <v>605</v>
       </c>
       <c r="B603" s="24">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C603" s="25">
-        <v>-15</v>
+        <v>-18</v>
       </c>
       <c r="D603" s="29"/>
       <c r="E603" s="28"/>
@@ -12146,16 +12122,16 @@
         <v>607</v>
       </c>
       <c r="B605" s="24">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="C605" s="25">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D605" s="26">
         <v>0.87</v>
       </c>
       <c r="E605" s="27">
-        <v>102.66</v>
+        <v>93.09</v>
       </c>
     </row>
     <row r="606" spans="1:5" x14ac:dyDescent="0.25">
@@ -12163,16 +12139,16 @@
         <v>608</v>
       </c>
       <c r="B606" s="24">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C606" s="25">
-        <v>410</v>
+        <v>388</v>
       </c>
       <c r="D606" s="26">
         <v>0.57999999999999996</v>
       </c>
       <c r="E606" s="27">
-        <v>237.8</v>
+        <v>225.04</v>
       </c>
     </row>
     <row r="607" spans="1:5" x14ac:dyDescent="0.25">
@@ -12180,16 +12156,16 @@
         <v>609</v>
       </c>
       <c r="B607" s="24">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C607" s="25">
-        <v>926.5</v>
+        <v>904</v>
       </c>
       <c r="D607" s="26">
         <v>0.85</v>
       </c>
       <c r="E607" s="27">
-        <v>787.53</v>
+        <v>768.4</v>
       </c>
     </row>
     <row r="608" spans="1:5" x14ac:dyDescent="0.25">
@@ -12208,16 +12184,16 @@
         <v>611</v>
       </c>
       <c r="B609" s="24">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C609" s="25">
-        <v>145.5</v>
+        <v>143.5</v>
       </c>
       <c r="D609" s="26">
         <v>0.85</v>
       </c>
       <c r="E609" s="27">
-        <v>123.68</v>
+        <v>121.98</v>
       </c>
     </row>
     <row r="610" spans="1:5" x14ac:dyDescent="0.25">
@@ -12294,10 +12270,10 @@
         <v>617</v>
       </c>
       <c r="B615" s="24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C615" s="25">
-        <v>-95</v>
+        <v>-105</v>
       </c>
       <c r="D615" s="29"/>
       <c r="E615" s="28"/>
@@ -12683,16 +12659,16 @@
         <v>642</v>
       </c>
       <c r="B640" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C640" s="25">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="D640" s="26">
         <v>5.75</v>
       </c>
       <c r="E640" s="27">
-        <v>14.38</v>
+        <v>8.6300000000000008</v>
       </c>
     </row>
     <row r="641" spans="1:5" x14ac:dyDescent="0.25">
@@ -12700,16 +12676,16 @@
         <v>643</v>
       </c>
       <c r="B641" s="24">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="C641" s="25">
-        <v>6.35</v>
+        <v>-1.65</v>
       </c>
       <c r="D641" s="26">
         <v>4</v>
       </c>
       <c r="E641" s="27">
-        <v>25.4</v>
+        <v>-6.6</v>
       </c>
     </row>
     <row r="642" spans="1:5" x14ac:dyDescent="0.25">
@@ -12751,16 +12727,16 @@
         <v>646</v>
       </c>
       <c r="B644" s="24">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="C644" s="25">
-        <v>-0.5</v>
+        <v>11</v>
       </c>
       <c r="D644" s="26">
-        <v>2.78</v>
+        <v>2.77</v>
       </c>
       <c r="E644" s="27">
-        <v>-1.39</v>
+        <v>30.43</v>
       </c>
     </row>
     <row r="645" spans="1:5" x14ac:dyDescent="0.25">
@@ -12768,16 +12744,16 @@
         <v>647</v>
       </c>
       <c r="B645" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C645" s="25">
-        <v>1.5</v>
+        <v>-0.5</v>
       </c>
       <c r="D645" s="26">
-        <v>2.73</v>
+        <v>2.72</v>
       </c>
       <c r="E645" s="27">
-        <v>4.09</v>
+        <v>-1.36</v>
       </c>
     </row>
     <row r="646" spans="1:5" x14ac:dyDescent="0.25">
@@ -12796,16 +12772,16 @@
         <v>649</v>
       </c>
       <c r="B647" s="24">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C647" s="25">
-        <v>9</v>
+        <v>10.5</v>
       </c>
       <c r="D647" s="26">
         <v>2.76</v>
       </c>
       <c r="E647" s="27">
-        <v>24.83</v>
+        <v>28.95</v>
       </c>
     </row>
     <row r="648" spans="1:5" x14ac:dyDescent="0.25">
@@ -12813,16 +12789,16 @@
         <v>650</v>
       </c>
       <c r="B648" s="24">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C648" s="25">
-        <v>6.5</v>
+        <v>2</v>
       </c>
       <c r="D648" s="26">
         <v>4</v>
       </c>
       <c r="E648" s="27">
-        <v>26</v>
+        <v>8</v>
       </c>
     </row>
     <row r="649" spans="1:5" x14ac:dyDescent="0.25">
@@ -12892,16 +12868,16 @@
         <v>655</v>
       </c>
       <c r="B653" s="24">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C653" s="25">
-        <v>64</v>
+        <v>49</v>
       </c>
       <c r="D653" s="26">
         <v>2.2799999999999998</v>
       </c>
       <c r="E653" s="27">
-        <v>145.91999999999999</v>
+        <v>111.72</v>
       </c>
     </row>
     <row r="654" spans="1:5" x14ac:dyDescent="0.25">
@@ -12971,16 +12947,16 @@
         <v>660</v>
       </c>
       <c r="B658" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C658" s="25">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="D658" s="26">
         <v>4.6500000000000004</v>
       </c>
       <c r="E658" s="27">
-        <v>76.73</v>
+        <v>62.78</v>
       </c>
     </row>
     <row r="659" spans="1:5" x14ac:dyDescent="0.25">
@@ -13022,16 +12998,16 @@
         <v>663</v>
       </c>
       <c r="B661" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C661" s="25">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="D661" s="26">
         <v>3.5</v>
       </c>
       <c r="E661" s="27">
-        <v>24.5</v>
+        <v>22.75</v>
       </c>
     </row>
     <row r="662" spans="1:5" x14ac:dyDescent="0.25">
@@ -13084,16 +13060,16 @@
         <v>667</v>
       </c>
       <c r="B665" s="24">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="C665" s="25">
-        <v>157.86000000000001</v>
+        <v>153.86000000000001</v>
       </c>
       <c r="D665" s="26">
         <v>1.7</v>
       </c>
       <c r="E665" s="27">
-        <v>268.36</v>
+        <v>261.56</v>
       </c>
     </row>
     <row r="666" spans="1:5" x14ac:dyDescent="0.25">
@@ -13101,16 +13077,16 @@
         <v>668</v>
       </c>
       <c r="B666" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C666" s="25">
-        <v>28.5</v>
+        <v>26.5</v>
       </c>
       <c r="D666" s="26">
         <v>3.33</v>
       </c>
       <c r="E666" s="27">
-        <v>94.91</v>
+        <v>88.25</v>
       </c>
     </row>
     <row r="667" spans="1:5" x14ac:dyDescent="0.25">
@@ -13203,16 +13179,16 @@
         <v>674</v>
       </c>
       <c r="B672" s="24">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="C672" s="25">
-        <v>37.5</v>
+        <v>37</v>
       </c>
       <c r="D672" s="26">
         <v>2.85</v>
       </c>
       <c r="E672" s="27">
-        <v>106.88</v>
+        <v>105.45</v>
       </c>
     </row>
     <row r="673" spans="1:5" x14ac:dyDescent="0.25">
@@ -13287,16 +13263,16 @@
         <v>680</v>
       </c>
       <c r="B678" s="24">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C678" s="25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D678" s="26">
         <v>5.73</v>
       </c>
       <c r="E678" s="27">
-        <v>143.30000000000001</v>
+        <v>137.56</v>
       </c>
     </row>
     <row r="679" spans="1:5" x14ac:dyDescent="0.25">
@@ -13422,16 +13398,16 @@
         <v>689</v>
       </c>
       <c r="B687" s="24">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="C687" s="25">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="D687" s="26">
         <v>3.1</v>
       </c>
       <c r="E687" s="27">
-        <v>412.3</v>
+        <v>403</v>
       </c>
     </row>
     <row r="688" spans="1:5" x14ac:dyDescent="0.25">
@@ -13439,16 +13415,16 @@
         <v>690</v>
       </c>
       <c r="B688" s="24">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C688" s="25">
-        <v>8.93</v>
+        <v>5.93</v>
       </c>
       <c r="D688" s="26">
         <v>3.6</v>
       </c>
       <c r="E688" s="27">
-        <v>32.15</v>
+        <v>21.35</v>
       </c>
     </row>
     <row r="689" spans="1:5" x14ac:dyDescent="0.25">
@@ -13490,16 +13466,16 @@
         <v>693</v>
       </c>
       <c r="B691" s="24">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C691" s="25">
-        <v>-24.5</v>
+        <v>-26.5</v>
       </c>
       <c r="D691" s="26">
         <v>3.75</v>
       </c>
       <c r="E691" s="27">
-        <v>-91.88</v>
+        <v>-99.38</v>
       </c>
     </row>
     <row r="692" spans="1:5" x14ac:dyDescent="0.25">
@@ -13586,16 +13562,16 @@
         <v>699</v>
       </c>
       <c r="B697" s="24">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C697" s="25">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="D697" s="26">
         <v>2.25</v>
       </c>
       <c r="E697" s="27">
-        <v>72</v>
+        <v>65.25</v>
       </c>
     </row>
     <row r="698" spans="1:5" x14ac:dyDescent="0.25">
@@ -13620,16 +13596,16 @@
         <v>701</v>
       </c>
       <c r="B699" s="24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C699" s="25">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="D699" s="26">
         <v>2.75</v>
       </c>
       <c r="E699" s="27">
-        <v>45.38</v>
+        <v>37.130000000000003</v>
       </c>
     </row>
     <row r="700" spans="1:5" x14ac:dyDescent="0.25">
@@ -13654,16 +13630,16 @@
         <v>703</v>
       </c>
       <c r="B701" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C701" s="25">
-        <v>22</v>
+        <v>16</v>
       </c>
       <c r="D701" s="26">
         <v>2.75</v>
       </c>
       <c r="E701" s="27">
-        <v>60.5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="702" spans="1:5" x14ac:dyDescent="0.25">
@@ -13808,10 +13784,10 @@
         <v>713</v>
       </c>
       <c r="B711" s="24">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="C711" s="25">
-        <v>8.5</v>
+        <v>3.5</v>
       </c>
       <c r="D711" s="29"/>
       <c r="E711" s="28"/>
@@ -13860,10 +13836,10 @@
         <v>717</v>
       </c>
       <c r="B715" s="24">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C715" s="25">
-        <v>3.5</v>
+        <v>-3</v>
       </c>
       <c r="D715" s="29"/>
       <c r="E715" s="28"/>
@@ -13873,10 +13849,10 @@
         <v>718</v>
       </c>
       <c r="B716" s="24">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C716" s="25">
-        <v>-84.5</v>
+        <v>-85.5</v>
       </c>
       <c r="D716" s="29"/>
       <c r="E716" s="28"/>
@@ -13886,10 +13862,10 @@
         <v>719</v>
       </c>
       <c r="B717" s="24">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C717" s="25">
-        <v>-48.5</v>
+        <v>-52.5</v>
       </c>
       <c r="D717" s="29"/>
       <c r="E717" s="28"/>
@@ -13899,10 +13875,10 @@
         <v>720</v>
       </c>
       <c r="B718" s="24">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C718" s="25">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="D718" s="29"/>
       <c r="E718" s="28"/>
@@ -13921,16 +13897,16 @@
         <v>722</v>
       </c>
       <c r="B720" s="24">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="C720" s="25">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D720" s="26">
         <v>2.93</v>
       </c>
       <c r="E720" s="27">
-        <v>134.86000000000001</v>
+        <v>126.06</v>
       </c>
     </row>
     <row r="721" spans="1:5" x14ac:dyDescent="0.25">
@@ -14369,10 +14345,10 @@
         <v>754</v>
       </c>
       <c r="B752" s="24">
-        <v>294</v>
+        <v>300</v>
       </c>
       <c r="C752" s="25">
-        <v>-879.7</v>
+        <v>-895.7</v>
       </c>
       <c r="D752" s="29"/>
       <c r="E752" s="28"/>
@@ -14383,11 +14359,11 @@
       </c>
       <c r="B753" s="31"/>
       <c r="C753" s="32">
-        <v>27081.34</v>
+        <v>27196.84</v>
       </c>
       <c r="D753" s="33"/>
       <c r="E753" s="34">
-        <v>61220.97</v>
+        <v>60534.55</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nikhil 07 april @ 1238 night
</commit_message>
<xml_diff>
--- a/data/website stock.xlsx
+++ b/data/website stock.xlsx
@@ -257,7 +257,7 @@
     <t>1127 PATRIKA (Eco-52)</t>
   </si>
   <si>
-    <t>1128 PATRIKA (Eco-55)</t>
+    <t>1128 PATRIKA (Eco-55) MAAL NHI MIL RHA</t>
   </si>
   <si>
     <t>1129 PATRIKA (Eco-56)</t>
@@ -908,7 +908,7 @@
     <t>5091 PATRIKA (JC)</t>
   </si>
   <si>
-    <t>5092 PATRIKA</t>
+    <t>5092 PATRIKA (10.04 6000</t>
   </si>
   <si>
     <t>5093 PATRIKA</t>
@@ -1838,7 +1838,7 @@
     <t>9222 CARDS - RED (9205)</t>
   </si>
   <si>
-    <t>9223 CARDS (9206-B) -GOLDEN</t>
+    <t>9223 CARDS (9206-B) -GOLDEN (Not Avlbl)</t>
   </si>
   <si>
     <t>9224 CARDS - RED (DESIGN CHAGE) 9208</t>
@@ -2991,16 +2991,16 @@
         <v>16</v>
       </c>
       <c r="B14" s="24">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="C14" s="25">
-        <v>85.5</v>
+        <v>113</v>
       </c>
       <c r="D14" s="26">
         <v>2</v>
       </c>
       <c r="E14" s="27">
-        <v>171</v>
+        <v>226</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -3008,17 +3008,11 @@
         <v>17</v>
       </c>
       <c r="B15" s="24">
-        <v>115</v>
-      </c>
-      <c r="C15" s="25">
-        <v>57</v>
-      </c>
-      <c r="D15" s="26">
-        <v>2</v>
-      </c>
-      <c r="E15" s="27">
-        <v>114</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="C15" s="28"/>
+      <c r="D15" s="29"/>
+      <c r="E15" s="28"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" s="23" t="s">
@@ -3042,16 +3036,16 @@
         <v>19</v>
       </c>
       <c r="B17" s="24">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C17" s="25">
-        <v>154.5</v>
+        <v>139.5</v>
       </c>
       <c r="D17" s="26">
         <v>2.1</v>
       </c>
       <c r="E17" s="27">
-        <v>324.45</v>
+        <v>292.95</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -3172,16 +3166,16 @@
         <v>27</v>
       </c>
       <c r="B25" s="24">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="C25" s="25">
-        <v>18.5</v>
+        <v>5</v>
       </c>
       <c r="D25" s="26">
         <v>1.65</v>
       </c>
       <c r="E25" s="27">
-        <v>30.53</v>
+        <v>8.25</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -3206,16 +3200,16 @@
         <v>29</v>
       </c>
       <c r="B27" s="24">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C27" s="25">
-        <v>52</v>
+        <v>50.5</v>
       </c>
       <c r="D27" s="26">
         <v>2</v>
       </c>
       <c r="E27" s="27">
-        <v>104</v>
+        <v>101</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3223,16 +3217,16 @@
         <v>30</v>
       </c>
       <c r="B28" s="24">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C28" s="25">
-        <v>80</v>
+        <v>76</v>
       </c>
       <c r="D28" s="26">
         <v>2</v>
       </c>
       <c r="E28" s="27">
-        <v>160</v>
+        <v>152</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -3240,16 +3234,16 @@
         <v>31</v>
       </c>
       <c r="B29" s="24">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C29" s="25">
-        <v>16.5</v>
+        <v>13.5</v>
       </c>
       <c r="D29" s="26">
         <v>2.6</v>
       </c>
       <c r="E29" s="27">
-        <v>42.9</v>
+        <v>35.1</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
@@ -3274,16 +3268,16 @@
         <v>33</v>
       </c>
       <c r="B31" s="24">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C31" s="25">
-        <v>78</v>
+        <v>74.5</v>
       </c>
       <c r="D31" s="26">
         <v>2.85</v>
       </c>
       <c r="E31" s="27">
-        <v>222.3</v>
+        <v>212.33</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -3336,17 +3330,11 @@
         <v>37</v>
       </c>
       <c r="B35" s="24">
-        <v>107</v>
-      </c>
-      <c r="C35" s="25">
-        <v>1.5</v>
-      </c>
-      <c r="D35" s="26">
-        <v>2.2999999999999998</v>
-      </c>
-      <c r="E35" s="27">
-        <v>3.45</v>
-      </c>
+        <v>106</v>
+      </c>
+      <c r="C35" s="28"/>
+      <c r="D35" s="29"/>
+      <c r="E35" s="28"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" s="23" t="s">
@@ -3409,16 +3397,16 @@
         <v>42</v>
       </c>
       <c r="B40" s="24">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C40" s="25">
-        <v>89</v>
+        <v>82</v>
       </c>
       <c r="D40" s="26">
         <v>2.14</v>
       </c>
       <c r="E40" s="27">
-        <v>190.46</v>
+        <v>175.48</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -3426,16 +3414,16 @@
         <v>43</v>
       </c>
       <c r="B41" s="24">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C41" s="25">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D41" s="26">
         <v>2.14</v>
       </c>
       <c r="E41" s="27">
-        <v>40.659999999999997</v>
+        <v>36.380000000000003</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -3477,16 +3465,16 @@
         <v>46</v>
       </c>
       <c r="B44" s="24">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C44" s="25">
-        <v>12</v>
+        <v>10.5</v>
       </c>
       <c r="D44" s="26">
         <v>2.72</v>
       </c>
       <c r="E44" s="27">
-        <v>32.6</v>
+        <v>28.52</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -3494,16 +3482,16 @@
         <v>47</v>
       </c>
       <c r="B45" s="24">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C45" s="25">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D45" s="26">
         <v>2.66</v>
       </c>
       <c r="E45" s="27">
-        <v>7.98</v>
+        <v>10.64</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -3539,16 +3527,16 @@
         <v>50</v>
       </c>
       <c r="B48" s="24">
-        <v>146</v>
+        <v>154</v>
       </c>
       <c r="C48" s="25">
-        <v>324.5</v>
+        <v>291</v>
       </c>
       <c r="D48" s="26">
         <v>1.26</v>
       </c>
       <c r="E48" s="27">
-        <v>408.9</v>
+        <v>366.69</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -3556,16 +3544,16 @@
         <v>51</v>
       </c>
       <c r="B49" s="24">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C49" s="25">
-        <v>106</v>
+        <v>98</v>
       </c>
       <c r="D49" s="26">
         <v>1.4</v>
       </c>
       <c r="E49" s="27">
-        <v>148.4</v>
+        <v>137.19999999999999</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -3590,16 +3578,16 @@
         <v>53</v>
       </c>
       <c r="B51" s="24">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C51" s="25">
-        <v>180</v>
+        <v>172</v>
       </c>
       <c r="D51" s="26">
         <v>1.8</v>
       </c>
       <c r="E51" s="27">
-        <v>324</v>
+        <v>309.60000000000002</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -3607,16 +3595,16 @@
         <v>54</v>
       </c>
       <c r="B52" s="24">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C52" s="25">
-        <v>73.5</v>
+        <v>72.5</v>
       </c>
       <c r="D52" s="26">
         <v>2.5</v>
       </c>
       <c r="E52" s="27">
-        <v>183.75</v>
+        <v>181.25</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -3624,16 +3612,16 @@
         <v>55</v>
       </c>
       <c r="B53" s="24">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C53" s="25">
-        <v>237</v>
+        <v>236.5</v>
       </c>
       <c r="D53" s="26">
         <v>2.5</v>
       </c>
       <c r="E53" s="27">
-        <v>592.5</v>
+        <v>591.25</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -3641,16 +3629,16 @@
         <v>56</v>
       </c>
       <c r="B54" s="24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C54" s="25">
-        <v>76.5</v>
+        <v>67.5</v>
       </c>
       <c r="D54" s="26">
         <v>2.75</v>
       </c>
       <c r="E54" s="27">
-        <v>210.38</v>
+        <v>185.63</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -3661,13 +3649,13 @@
         <v>44</v>
       </c>
       <c r="C55" s="25">
-        <v>332.65</v>
+        <v>182.65</v>
       </c>
       <c r="D55" s="26">
         <v>2.75</v>
       </c>
       <c r="E55" s="27">
-        <v>914.78</v>
+        <v>502.29</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -3675,16 +3663,16 @@
         <v>58</v>
       </c>
       <c r="B56" s="24">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C56" s="25">
-        <v>79.5</v>
+        <v>74.5</v>
       </c>
       <c r="D56" s="26">
         <v>1.8</v>
       </c>
       <c r="E56" s="27">
-        <v>143.1</v>
+        <v>134.1</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -3720,16 +3708,16 @@
         <v>61</v>
       </c>
       <c r="B59" s="24">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C59" s="25">
-        <v>22.25</v>
+        <v>17.25</v>
       </c>
       <c r="D59" s="26">
         <v>1.9</v>
       </c>
       <c r="E59" s="27">
-        <v>42.28</v>
+        <v>32.78</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -3737,16 +3725,16 @@
         <v>62</v>
       </c>
       <c r="B60" s="24">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C60" s="25">
-        <v>632.5</v>
+        <v>622.5</v>
       </c>
       <c r="D60" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E60" s="27">
-        <v>719.52</v>
+        <v>708.14</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.25">
@@ -3754,16 +3742,16 @@
         <v>63</v>
       </c>
       <c r="B61" s="24">
-        <v>174</v>
+        <v>178</v>
       </c>
       <c r="C61" s="25">
-        <v>570.5</v>
+        <v>545.5</v>
       </c>
       <c r="D61" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E61" s="27">
-        <v>649.99</v>
+        <v>621.51</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -3816,16 +3804,16 @@
         <v>67</v>
       </c>
       <c r="B65" s="24">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C65" s="25">
-        <v>479.5</v>
+        <v>475.5</v>
       </c>
       <c r="D65" s="26">
         <v>1.65</v>
       </c>
       <c r="E65" s="27">
-        <v>791.18</v>
+        <v>784.58</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -3861,16 +3849,16 @@
         <v>70</v>
       </c>
       <c r="B68" s="24">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="C68" s="25">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="D68" s="26">
         <v>1.65</v>
       </c>
       <c r="E68" s="27">
-        <v>605.54999999999995</v>
+        <v>590.70000000000005</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -3889,16 +3877,16 @@
         <v>72</v>
       </c>
       <c r="B70" s="24">
-        <v>168</v>
+        <v>172</v>
       </c>
       <c r="C70" s="25">
-        <v>423.5</v>
+        <v>401.5</v>
       </c>
       <c r="D70" s="26">
         <v>1.4</v>
       </c>
       <c r="E70" s="27">
-        <v>592.9</v>
+        <v>562.1</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -3906,16 +3894,16 @@
         <v>73</v>
       </c>
       <c r="B71" s="24">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="C71" s="25">
-        <v>656</v>
+        <v>622</v>
       </c>
       <c r="D71" s="26">
         <v>1.4</v>
       </c>
       <c r="E71" s="27">
-        <v>918.4</v>
+        <v>870.8</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -3923,16 +3911,16 @@
         <v>74</v>
       </c>
       <c r="B72" s="24">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C72" s="25">
-        <v>469</v>
+        <v>459.5</v>
       </c>
       <c r="D72" s="26">
         <v>1.4</v>
       </c>
       <c r="E72" s="27">
-        <v>656.6</v>
+        <v>643.29999999999995</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -3940,16 +3928,16 @@
         <v>75</v>
       </c>
       <c r="B73" s="24">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="C73" s="25">
-        <v>440.5</v>
+        <v>430.5</v>
       </c>
       <c r="D73" s="26">
         <v>1.4</v>
       </c>
       <c r="E73" s="27">
-        <v>616.70000000000005</v>
+        <v>602.70000000000005</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -3957,16 +3945,16 @@
         <v>76</v>
       </c>
       <c r="B74" s="24">
-        <v>164</v>
+        <v>168</v>
       </c>
       <c r="C74" s="25">
-        <v>173.5</v>
+        <v>156</v>
       </c>
       <c r="D74" s="26">
         <v>1.2</v>
       </c>
       <c r="E74" s="27">
-        <v>208.2</v>
+        <v>187.2</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -3974,16 +3962,16 @@
         <v>77</v>
       </c>
       <c r="B75" s="24">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="C75" s="25">
-        <v>290.5</v>
+        <v>280.5</v>
       </c>
       <c r="D75" s="26">
         <v>1.2</v>
       </c>
       <c r="E75" s="27">
-        <v>348.6</v>
+        <v>336.6</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
@@ -3991,16 +3979,16 @@
         <v>78</v>
       </c>
       <c r="B76" s="24">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C76" s="25">
-        <v>394</v>
+        <v>393</v>
       </c>
       <c r="D76" s="26">
         <v>1.2</v>
       </c>
       <c r="E76" s="27">
-        <v>472.8</v>
+        <v>471.6</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -4025,16 +4013,16 @@
         <v>80</v>
       </c>
       <c r="B78" s="24">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="C78" s="25">
-        <v>343.5</v>
+        <v>313.5</v>
       </c>
       <c r="D78" s="26">
         <v>1.2</v>
       </c>
       <c r="E78" s="27">
-        <v>412.2</v>
+        <v>376.2</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -4042,16 +4030,16 @@
         <v>81</v>
       </c>
       <c r="B79" s="24">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C79" s="25">
-        <v>409</v>
+        <v>361</v>
       </c>
       <c r="D79" s="26">
         <v>1.2</v>
       </c>
       <c r="E79" s="27">
-        <v>490.8</v>
+        <v>433.2</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -4059,16 +4047,16 @@
         <v>82</v>
       </c>
       <c r="B80" s="24">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C80" s="25">
-        <v>363.5</v>
+        <v>327.5</v>
       </c>
       <c r="D80" s="26">
         <v>1.2</v>
       </c>
       <c r="E80" s="27">
-        <v>436.2</v>
+        <v>393</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -4127,16 +4115,16 @@
         <v>86</v>
       </c>
       <c r="B84" s="24">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="C84" s="25">
-        <v>430.5</v>
+        <v>426.5</v>
       </c>
       <c r="D84" s="26">
         <v>1.3</v>
       </c>
       <c r="E84" s="27">
-        <v>559.65</v>
+        <v>554.45000000000005</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -4144,16 +4132,16 @@
         <v>87</v>
       </c>
       <c r="B85" s="24">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="C85" s="25">
-        <v>882.5</v>
+        <v>872.5</v>
       </c>
       <c r="D85" s="26">
         <v>1.3</v>
       </c>
       <c r="E85" s="27">
-        <v>1147.25</v>
+        <v>1134.25</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -4161,16 +4149,16 @@
         <v>88</v>
       </c>
       <c r="B86" s="24">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C86" s="25">
-        <v>919</v>
+        <v>903</v>
       </c>
       <c r="D86" s="26">
         <v>1.7</v>
       </c>
       <c r="E86" s="27">
-        <v>1562.3</v>
+        <v>1535.1</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -4212,16 +4200,16 @@
         <v>91</v>
       </c>
       <c r="B89" s="24">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C89" s="25">
-        <v>-69.5</v>
+        <v>-77.5</v>
       </c>
       <c r="D89" s="26">
         <v>1.47</v>
       </c>
       <c r="E89" s="27">
-        <v>-102.26</v>
+        <v>-114.03</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -4229,16 +4217,16 @@
         <v>92</v>
       </c>
       <c r="B90" s="24">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C90" s="25">
-        <v>93.2</v>
+        <v>90.7</v>
       </c>
       <c r="D90" s="26">
         <v>1.28</v>
       </c>
       <c r="E90" s="27">
-        <v>119.55</v>
+        <v>116.34</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -4263,16 +4251,16 @@
         <v>94</v>
       </c>
       <c r="B92" s="24">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C92" s="25">
-        <v>753.5</v>
+        <v>747</v>
       </c>
       <c r="D92" s="26">
         <v>1.83</v>
       </c>
       <c r="E92" s="27">
-        <v>1377.75</v>
+        <v>1365.87</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -4280,16 +4268,16 @@
         <v>95</v>
       </c>
       <c r="B93" s="24">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C93" s="25">
-        <v>246.5</v>
+        <v>241.5</v>
       </c>
       <c r="D93" s="26">
         <v>2.27</v>
       </c>
       <c r="E93" s="27">
-        <v>558.59</v>
+        <v>547.26</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.25">
@@ -4310,16 +4298,16 @@
         <v>97</v>
       </c>
       <c r="B95" s="24">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C95" s="25">
-        <v>110.5</v>
+        <v>107.5</v>
       </c>
       <c r="D95" s="26">
         <v>0.9</v>
       </c>
       <c r="E95" s="27">
-        <v>99.45</v>
+        <v>96.75</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -4344,16 +4332,16 @@
         <v>99</v>
       </c>
       <c r="B97" s="24">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C97" s="25">
-        <v>171.5</v>
+        <v>168</v>
       </c>
       <c r="D97" s="26">
         <v>0.9</v>
       </c>
       <c r="E97" s="27">
-        <v>154.35</v>
+        <v>151.19999999999999</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -4378,16 +4366,16 @@
         <v>101</v>
       </c>
       <c r="B99" s="24">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="C99" s="25">
-        <v>215</v>
+        <v>203</v>
       </c>
       <c r="D99" s="26">
         <v>1.65</v>
       </c>
       <c r="E99" s="27">
-        <v>354.75</v>
+        <v>334.95</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -4487,16 +4475,16 @@
         <v>108</v>
       </c>
       <c r="B106" s="24">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C106" s="25">
-        <v>56</v>
+        <v>39</v>
       </c>
       <c r="D106" s="26">
         <v>2.5</v>
       </c>
       <c r="E106" s="27">
-        <v>140</v>
+        <v>97.5</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.25">
@@ -4504,16 +4492,16 @@
         <v>109</v>
       </c>
       <c r="B107" s="24">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C107" s="25">
-        <v>102</v>
+        <v>98.5</v>
       </c>
       <c r="D107" s="26">
         <v>2.5</v>
       </c>
       <c r="E107" s="27">
-        <v>255</v>
+        <v>246.25</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -4538,10 +4526,10 @@
         <v>111</v>
       </c>
       <c r="B109" s="24">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="C109" s="25">
-        <v>33.5</v>
+        <v>12.5</v>
       </c>
       <c r="D109" s="29"/>
       <c r="E109" s="28"/>
@@ -4551,10 +4539,10 @@
         <v>112</v>
       </c>
       <c r="B110" s="24">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C110" s="25">
-        <v>69</v>
+        <v>59</v>
       </c>
       <c r="D110" s="29"/>
       <c r="E110" s="28"/>
@@ -4564,11 +4552,9 @@
         <v>113</v>
       </c>
       <c r="B111" s="24">
-        <v>25</v>
-      </c>
-      <c r="C111" s="25">
-        <v>14</v>
-      </c>
+        <v>26</v>
+      </c>
+      <c r="C111" s="28"/>
       <c r="D111" s="29"/>
       <c r="E111" s="28"/>
     </row>
@@ -4627,10 +4613,10 @@
         <v>118</v>
       </c>
       <c r="B116" s="24">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C116" s="25">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="D116" s="29"/>
       <c r="E116" s="28"/>
@@ -4653,10 +4639,10 @@
         <v>120</v>
       </c>
       <c r="B118" s="24">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C118" s="25">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="D118" s="29"/>
       <c r="E118" s="28"/>
@@ -4679,10 +4665,10 @@
         <v>122</v>
       </c>
       <c r="B120" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C120" s="25">
-        <v>-44</v>
+        <v>-56</v>
       </c>
       <c r="D120" s="29"/>
       <c r="E120" s="28"/>
@@ -4692,10 +4678,10 @@
         <v>123</v>
       </c>
       <c r="B121" s="24">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C121" s="25">
-        <v>-20</v>
+        <v>-30</v>
       </c>
       <c r="D121" s="29"/>
       <c r="E121" s="28"/>
@@ -4761,16 +4747,16 @@
         <v>128</v>
       </c>
       <c r="B126" s="24">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C126" s="25">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="D126" s="26">
         <v>1.1499999999999999</v>
       </c>
       <c r="E126" s="27">
-        <v>18.399999999999999</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
@@ -4943,9 +4929,15 @@
       <c r="B140" s="24">
         <v>81</v>
       </c>
-      <c r="C140" s="28"/>
-      <c r="D140" s="29"/>
-      <c r="E140" s="28"/>
+      <c r="C140" s="25">
+        <v>1</v>
+      </c>
+      <c r="D140" s="26">
+        <v>12.5</v>
+      </c>
+      <c r="E140" s="27">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A141" s="23" t="s">
@@ -5070,16 +5062,16 @@
         <v>151</v>
       </c>
       <c r="B149" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C149" s="25">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="D149" s="26">
         <v>18.5</v>
       </c>
       <c r="E149" s="27">
-        <v>111</v>
+        <v>55.5</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.25">
@@ -5087,16 +5079,16 @@
         <v>152</v>
       </c>
       <c r="B150" s="24">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C150" s="25">
-        <v>1.5</v>
+        <v>3.5</v>
       </c>
       <c r="D150" s="26">
         <v>18.5</v>
       </c>
       <c r="E150" s="27">
-        <v>27.75</v>
+        <v>64.75</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
@@ -5104,16 +5096,16 @@
         <v>153</v>
       </c>
       <c r="B151" s="24">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C151" s="25">
-        <v>0.5</v>
+        <v>4.5</v>
       </c>
       <c r="D151" s="26">
         <v>18.5</v>
       </c>
       <c r="E151" s="27">
-        <v>9.25</v>
+        <v>83.25</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.25">
@@ -5138,16 +5130,16 @@
         <v>155</v>
       </c>
       <c r="B153" s="24">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C153" s="25">
-        <v>1.27</v>
+        <v>3.27</v>
       </c>
       <c r="D153" s="26">
         <v>18.5</v>
       </c>
       <c r="E153" s="27">
-        <v>23.5</v>
+        <v>60.5</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.25">
@@ -5290,16 +5282,16 @@
         <v>165</v>
       </c>
       <c r="B163" s="24">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C163" s="25">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="D163" s="26">
         <v>11.5</v>
       </c>
       <c r="E163" s="27">
-        <v>17.25</v>
+        <v>11.5</v>
       </c>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
@@ -5584,16 +5576,16 @@
         <v>185</v>
       </c>
       <c r="B183" s="24">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C183" s="25">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D183" s="26">
         <v>3.25</v>
       </c>
       <c r="E183" s="27">
-        <v>81.25</v>
+        <v>78</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
@@ -5678,16 +5670,16 @@
         <v>191</v>
       </c>
       <c r="B189" s="24">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C189" s="25">
-        <v>112.5</v>
+        <v>109.5</v>
       </c>
       <c r="D189" s="26">
         <v>2.8</v>
       </c>
       <c r="E189" s="27">
-        <v>315.2</v>
+        <v>306.79000000000002</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
@@ -5729,16 +5721,16 @@
         <v>194</v>
       </c>
       <c r="B192" s="24">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C192" s="25">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="D192" s="26">
         <v>3.33</v>
       </c>
       <c r="E192" s="27">
-        <v>26.64</v>
+        <v>3.33</v>
       </c>
     </row>
     <row r="193" spans="1:5" x14ac:dyDescent="0.25">
@@ -5813,16 +5805,16 @@
         <v>200</v>
       </c>
       <c r="B198" s="24">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C198" s="25">
-        <v>47.81</v>
+        <v>49.31</v>
       </c>
       <c r="D198" s="26">
         <v>2.65</v>
       </c>
       <c r="E198" s="27">
-        <v>126.7</v>
+        <v>130.66999999999999</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
@@ -5909,16 +5901,16 @@
         <v>206</v>
       </c>
       <c r="B204" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C204" s="25">
-        <v>17.5</v>
+        <v>16.5</v>
       </c>
       <c r="D204" s="26">
         <v>3.14</v>
       </c>
       <c r="E204" s="27">
-        <v>54.95</v>
+        <v>51.81</v>
       </c>
     </row>
     <row r="205" spans="1:5" x14ac:dyDescent="0.25">
@@ -5999,16 +5991,16 @@
         <v>212</v>
       </c>
       <c r="B210" s="24">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C210" s="25">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D210" s="26">
         <v>4.5</v>
       </c>
       <c r="E210" s="27">
-        <v>58.5</v>
+        <v>54</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.25">
@@ -6044,16 +6036,16 @@
         <v>215</v>
       </c>
       <c r="B213" s="24">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C213" s="25">
-        <v>126.5</v>
+        <v>124</v>
       </c>
       <c r="D213" s="26">
         <v>2.7</v>
       </c>
       <c r="E213" s="27">
-        <v>341.55</v>
+        <v>334.8</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
@@ -6061,16 +6053,16 @@
         <v>216</v>
       </c>
       <c r="B214" s="24">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="C214" s="25">
-        <v>62</v>
+        <v>53.5</v>
       </c>
       <c r="D214" s="26">
         <v>2.6</v>
       </c>
       <c r="E214" s="27">
-        <v>161.19999999999999</v>
+        <v>139.1</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
@@ -6095,16 +6087,16 @@
         <v>218</v>
       </c>
       <c r="B216" s="24">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C216" s="25">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="D216" s="26">
         <v>2.6</v>
       </c>
       <c r="E216" s="27">
-        <v>6.5</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="217" spans="1:5" x14ac:dyDescent="0.25">
@@ -6163,16 +6155,16 @@
         <v>222</v>
       </c>
       <c r="B220" s="24">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="C220" s="25">
-        <v>9.5</v>
+        <v>13.5</v>
       </c>
       <c r="D220" s="26">
         <v>3.93</v>
       </c>
       <c r="E220" s="27">
-        <v>37.35</v>
+        <v>53.08</v>
       </c>
     </row>
     <row r="221" spans="1:5" x14ac:dyDescent="0.25">
@@ -6180,11 +6172,17 @@
         <v>223</v>
       </c>
       <c r="B221" s="24">
-        <v>34</v>
-      </c>
-      <c r="C221" s="28"/>
-      <c r="D221" s="29"/>
-      <c r="E221" s="28"/>
+        <v>33</v>
+      </c>
+      <c r="C221" s="25">
+        <v>2</v>
+      </c>
+      <c r="D221" s="26">
+        <v>4.5</v>
+      </c>
+      <c r="E221" s="27">
+        <v>9</v>
+      </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A222" s="23" t="s">
@@ -6242,16 +6240,16 @@
         <v>227</v>
       </c>
       <c r="B225" s="24">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C225" s="25">
-        <v>10.5</v>
+        <v>11.5</v>
       </c>
       <c r="D225" s="26">
         <v>4.5</v>
       </c>
       <c r="E225" s="27">
-        <v>47.25</v>
+        <v>51.75</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
@@ -6276,16 +6274,16 @@
         <v>229</v>
       </c>
       <c r="B227" s="24">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C227" s="25">
-        <v>52.5</v>
+        <v>51.5</v>
       </c>
       <c r="D227" s="26">
         <v>3</v>
       </c>
       <c r="E227" s="27">
-        <v>157.5</v>
+        <v>154.5</v>
       </c>
     </row>
     <row r="228" spans="1:5" x14ac:dyDescent="0.25">
@@ -6310,16 +6308,16 @@
         <v>231</v>
       </c>
       <c r="B229" s="24">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C229" s="25">
-        <v>-1.75</v>
+        <v>3.25</v>
       </c>
       <c r="D229" s="26">
         <v>3.25</v>
       </c>
       <c r="E229" s="27">
-        <v>-5.69</v>
+        <v>10.56</v>
       </c>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
@@ -6327,16 +6325,16 @@
         <v>232</v>
       </c>
       <c r="B230" s="24">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C230" s="25">
-        <v>32.75</v>
+        <v>30.75</v>
       </c>
       <c r="D230" s="26">
         <v>3.65</v>
       </c>
       <c r="E230" s="27">
-        <v>119.66</v>
+        <v>112.36</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.25">
@@ -6389,16 +6387,16 @@
         <v>236</v>
       </c>
       <c r="B234" s="24">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C234" s="25">
-        <v>30</v>
+        <v>25.5</v>
       </c>
       <c r="D234" s="26">
         <v>2.66</v>
       </c>
       <c r="E234" s="27">
-        <v>79.8</v>
+        <v>67.83</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
@@ -6474,16 +6472,16 @@
         <v>241</v>
       </c>
       <c r="B239" s="24">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C239" s="25">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D239" s="26">
         <v>3.96</v>
       </c>
       <c r="E239" s="27">
-        <v>308.64</v>
+        <v>304.68</v>
       </c>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.25">
@@ -6491,16 +6489,16 @@
         <v>242</v>
       </c>
       <c r="B240" s="24">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="C240" s="25">
-        <v>21</v>
+        <v>19.5</v>
       </c>
       <c r="D240" s="26">
         <v>3.5</v>
       </c>
       <c r="E240" s="27">
-        <v>73.5</v>
+        <v>68.25</v>
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.25">
@@ -6522,13 +6520,13 @@
         <v>134</v>
       </c>
       <c r="C242" s="25">
-        <v>87.38</v>
+        <v>88.38</v>
       </c>
       <c r="D242" s="26">
         <v>3.25</v>
       </c>
       <c r="E242" s="27">
-        <v>283.99</v>
+        <v>287.24</v>
       </c>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.25">
@@ -6663,16 +6661,16 @@
         <v>254</v>
       </c>
       <c r="B252" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C252" s="25">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="D252" s="26">
         <v>8.25</v>
       </c>
       <c r="E252" s="27">
-        <v>123.75</v>
+        <v>82.5</v>
       </c>
     </row>
     <row r="253" spans="1:5" x14ac:dyDescent="0.25">
@@ -6680,16 +6678,16 @@
         <v>255</v>
       </c>
       <c r="B253" s="24">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C253" s="25">
-        <v>-1.5</v>
+        <v>1</v>
       </c>
       <c r="D253" s="26">
         <v>5.75</v>
       </c>
       <c r="E253" s="27">
-        <v>-8.6199999999999992</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="254" spans="1:5" x14ac:dyDescent="0.25">
@@ -6725,16 +6723,16 @@
         <v>258</v>
       </c>
       <c r="B256" s="24">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C256" s="25">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="D256" s="26">
         <v>3</v>
       </c>
       <c r="E256" s="27">
-        <v>-1.5</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="257" spans="1:5" x14ac:dyDescent="0.25">
@@ -6742,16 +6740,16 @@
         <v>259</v>
       </c>
       <c r="B257" s="24">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C257" s="25">
-        <v>38.18</v>
+        <v>37.18</v>
       </c>
       <c r="D257" s="26">
         <v>3</v>
       </c>
       <c r="E257" s="27">
-        <v>114.54</v>
+        <v>111.54</v>
       </c>
     </row>
     <row r="258" spans="1:5" x14ac:dyDescent="0.25">
@@ -6759,16 +6757,16 @@
         <v>260</v>
       </c>
       <c r="B258" s="24">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C258" s="25">
-        <v>31.5</v>
+        <v>32.5</v>
       </c>
       <c r="D258" s="26">
         <v>3.8</v>
       </c>
       <c r="E258" s="27">
-        <v>119.7</v>
+        <v>123.5</v>
       </c>
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.25">
@@ -6776,16 +6774,16 @@
         <v>261</v>
       </c>
       <c r="B259" s="24">
-        <v>311</v>
+        <v>316</v>
       </c>
       <c r="C259" s="25">
-        <v>131</v>
+        <v>101</v>
       </c>
       <c r="D259" s="26">
         <v>3.9</v>
       </c>
       <c r="E259" s="27">
-        <v>510.9</v>
+        <v>393.9</v>
       </c>
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.25">
@@ -6849,16 +6847,16 @@
         <v>266</v>
       </c>
       <c r="B264" s="24">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C264" s="25">
-        <v>28</v>
+        <v>25.5</v>
       </c>
       <c r="D264" s="26">
         <v>3.5</v>
       </c>
       <c r="E264" s="27">
-        <v>98</v>
+        <v>89.25</v>
       </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
@@ -6992,13 +6990,13 @@
         <v>421</v>
       </c>
       <c r="C274" s="25">
-        <v>-6.5</v>
+        <v>-5.5</v>
       </c>
       <c r="D274" s="26">
         <v>4.28</v>
       </c>
       <c r="E274" s="27">
-        <v>-27.82</v>
+        <v>-23.54</v>
       </c>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.25">
@@ -7051,16 +7049,16 @@
         <v>280</v>
       </c>
       <c r="B278" s="24">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="C278" s="25">
-        <v>-2</v>
+        <v>1</v>
       </c>
       <c r="D278" s="26">
         <v>3.1</v>
       </c>
       <c r="E278" s="27">
-        <v>-6.2</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.25">
@@ -7079,16 +7077,16 @@
         <v>282</v>
       </c>
       <c r="B280" s="24">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C280" s="25">
-        <v>-4.5</v>
+        <v>0.5</v>
       </c>
       <c r="D280" s="26">
         <v>4.5</v>
       </c>
       <c r="E280" s="27">
-        <v>-20.25</v>
+        <v>2.25</v>
       </c>
     </row>
     <row r="281" spans="1:5" x14ac:dyDescent="0.25">
@@ -7099,13 +7097,13 @@
         <v>59</v>
       </c>
       <c r="C281" s="25">
-        <v>11.5</v>
+        <v>15.5</v>
       </c>
       <c r="D281" s="26">
         <v>6.25</v>
       </c>
       <c r="E281" s="27">
-        <v>71.88</v>
+        <v>96.88</v>
       </c>
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.25">
@@ -7141,16 +7139,16 @@
         <v>286</v>
       </c>
       <c r="B284" s="24">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C284" s="25">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="D284" s="26">
         <v>4.4000000000000004</v>
       </c>
       <c r="E284" s="27">
-        <v>39.619999999999997</v>
+        <v>22.01</v>
       </c>
     </row>
     <row r="285" spans="1:5" x14ac:dyDescent="0.25">
@@ -7197,16 +7195,16 @@
         <v>290</v>
       </c>
       <c r="B288" s="24">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C288" s="25">
-        <v>3.5</v>
+        <v>0.5</v>
       </c>
       <c r="D288" s="26">
         <v>6.5</v>
       </c>
       <c r="E288" s="27">
-        <v>22.75</v>
+        <v>3.25</v>
       </c>
     </row>
     <row r="289" spans="1:5" x14ac:dyDescent="0.25">
@@ -7231,16 +7229,16 @@
         <v>292</v>
       </c>
       <c r="B290" s="24">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="C290" s="25">
-        <v>59</v>
+        <v>50.5</v>
       </c>
       <c r="D290" s="26">
         <v>4.8499999999999996</v>
       </c>
       <c r="E290" s="27">
-        <v>286.33</v>
+        <v>245.08</v>
       </c>
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.25">
@@ -7259,16 +7257,16 @@
         <v>294</v>
       </c>
       <c r="B292" s="24">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C292" s="25">
-        <v>5</v>
+        <v>1.5</v>
       </c>
       <c r="D292" s="26">
         <v>4.75</v>
       </c>
       <c r="E292" s="27">
-        <v>23.74</v>
+        <v>7.12</v>
       </c>
     </row>
     <row r="293" spans="1:5" x14ac:dyDescent="0.25">
@@ -7293,16 +7291,16 @@
         <v>296</v>
       </c>
       <c r="B294" s="24">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C294" s="25">
-        <v>45.5</v>
+        <v>46.5</v>
       </c>
       <c r="D294" s="26">
         <v>5.16</v>
       </c>
       <c r="E294" s="27">
-        <v>234.78</v>
+        <v>239.94</v>
       </c>
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.25">
@@ -7378,16 +7376,16 @@
         <v>301</v>
       </c>
       <c r="B299" s="24">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C299" s="25">
-        <v>24.5</v>
+        <v>20.5</v>
       </c>
       <c r="D299" s="26">
         <v>4.66</v>
       </c>
       <c r="E299" s="27">
-        <v>114.16</v>
+        <v>95.52</v>
       </c>
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.25">
@@ -7429,16 +7427,16 @@
         <v>304</v>
       </c>
       <c r="B302" s="24">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C302" s="25">
-        <v>8.5</v>
+        <v>4.5</v>
       </c>
       <c r="D302" s="26">
         <v>3.8</v>
       </c>
       <c r="E302" s="27">
-        <v>32.299999999999997</v>
+        <v>17.100000000000001</v>
       </c>
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.25">
@@ -7446,16 +7444,16 @@
         <v>305</v>
       </c>
       <c r="B303" s="24">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C303" s="25">
-        <v>18.5</v>
+        <v>7.5</v>
       </c>
       <c r="D303" s="26">
         <v>4.8899999999999997</v>
       </c>
       <c r="E303" s="27">
-        <v>90.39</v>
+        <v>36.65</v>
       </c>
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.25">
@@ -7480,16 +7478,16 @@
         <v>307</v>
       </c>
       <c r="B305" s="24">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C305" s="25">
-        <v>4.5</v>
+        <v>3.5</v>
       </c>
       <c r="D305" s="26">
         <v>3.15</v>
       </c>
       <c r="E305" s="27">
-        <v>14.18</v>
+        <v>11.03</v>
       </c>
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.25">
@@ -7497,16 +7495,16 @@
         <v>308</v>
       </c>
       <c r="B306" s="24">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="C306" s="25">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="D306" s="26">
-        <v>6.21</v>
+        <v>6.22</v>
       </c>
       <c r="E306" s="27">
-        <v>434.97</v>
+        <v>422.94</v>
       </c>
     </row>
     <row r="307" spans="1:5" x14ac:dyDescent="0.25">
@@ -7717,16 +7715,16 @@
         <v>322</v>
       </c>
       <c r="B320" s="24">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C320" s="25">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="D320" s="26">
         <v>7.75</v>
       </c>
       <c r="E320" s="27">
-        <v>54.25</v>
+        <v>19.38</v>
       </c>
     </row>
     <row r="321" spans="1:5" x14ac:dyDescent="0.25">
@@ -7883,16 +7881,16 @@
         <v>334</v>
       </c>
       <c r="B332" s="24">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C332" s="25">
-        <v>7.5</v>
+        <v>5.5</v>
       </c>
       <c r="D332" s="26">
         <v>5.25</v>
       </c>
       <c r="E332" s="27">
-        <v>39.380000000000003</v>
+        <v>28.88</v>
       </c>
     </row>
     <row r="333" spans="1:5" x14ac:dyDescent="0.25">
@@ -7951,16 +7949,16 @@
         <v>338</v>
       </c>
       <c r="B336" s="24">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C336" s="25">
-        <v>6.5</v>
+        <v>3.5</v>
       </c>
       <c r="D336" s="26">
         <v>10</v>
       </c>
       <c r="E336" s="27">
-        <v>65</v>
+        <v>35</v>
       </c>
     </row>
     <row r="337" spans="1:5" x14ac:dyDescent="0.25">
@@ -7996,16 +7994,16 @@
         <v>341</v>
       </c>
       <c r="B339" s="24">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C339" s="25">
-        <v>29.91</v>
+        <v>34.909999999999997</v>
       </c>
       <c r="D339" s="26">
         <v>4.28</v>
       </c>
       <c r="E339" s="27">
-        <v>128.01</v>
+        <v>149.41</v>
       </c>
     </row>
     <row r="340" spans="1:5" x14ac:dyDescent="0.25">
@@ -8013,16 +8011,16 @@
         <v>342</v>
       </c>
       <c r="B340" s="24">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C340" s="25">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D340" s="26">
         <v>4.28</v>
       </c>
       <c r="E340" s="27">
-        <v>273.92</v>
+        <v>282.48</v>
       </c>
     </row>
     <row r="341" spans="1:5" x14ac:dyDescent="0.25">
@@ -8086,16 +8084,16 @@
         <v>347</v>
       </c>
       <c r="B345" s="24">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C345" s="25">
-        <v>20.5</v>
+        <v>18.5</v>
       </c>
       <c r="D345" s="26">
         <v>9</v>
       </c>
       <c r="E345" s="27">
-        <v>184.5</v>
+        <v>166.5</v>
       </c>
     </row>
     <row r="346" spans="1:5" x14ac:dyDescent="0.25">
@@ -8123,13 +8121,13 @@
         <v>72</v>
       </c>
       <c r="C347" s="25">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D347" s="26">
         <v>9</v>
       </c>
       <c r="E347" s="27">
-        <v>13.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="348" spans="1:5" x14ac:dyDescent="0.25">
@@ -8363,13 +8361,13 @@
         <v>79</v>
       </c>
       <c r="C363" s="25">
-        <v>16.350000000000001</v>
+        <v>9.35</v>
       </c>
       <c r="D363" s="26">
         <v>4.75</v>
       </c>
       <c r="E363" s="27">
-        <v>77.66</v>
+        <v>44.41</v>
       </c>
     </row>
     <row r="364" spans="1:5" x14ac:dyDescent="0.25">
@@ -8409,16 +8407,16 @@
         <v>368</v>
       </c>
       <c r="B366" s="24">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C366" s="25">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D366" s="26">
         <v>10.5</v>
       </c>
       <c r="E366" s="27">
-        <v>252</v>
+        <v>210</v>
       </c>
     </row>
     <row r="367" spans="1:5" x14ac:dyDescent="0.25">
@@ -8426,16 +8424,16 @@
         <v>369</v>
       </c>
       <c r="B367" s="24">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C367" s="25">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D367" s="26">
         <v>8</v>
       </c>
       <c r="E367" s="27">
-        <v>103.97</v>
+        <v>95.97</v>
       </c>
     </row>
     <row r="368" spans="1:5" x14ac:dyDescent="0.25">
@@ -8488,16 +8486,16 @@
         <v>373</v>
       </c>
       <c r="B371" s="24">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C371" s="25">
-        <v>30.5</v>
+        <v>25.5</v>
       </c>
       <c r="D371" s="26">
         <v>7.77</v>
       </c>
       <c r="E371" s="27">
-        <v>236.88</v>
+        <v>198.05</v>
       </c>
     </row>
     <row r="372" spans="1:5" x14ac:dyDescent="0.25">
@@ -8505,16 +8503,16 @@
         <v>374</v>
       </c>
       <c r="B372" s="24">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C372" s="25">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D372" s="26">
         <v>7.13</v>
       </c>
       <c r="E372" s="27">
-        <v>206.77</v>
+        <v>192.51</v>
       </c>
     </row>
     <row r="373" spans="1:5" x14ac:dyDescent="0.25">
@@ -8547,13 +8545,13 @@
         <v>43</v>
       </c>
       <c r="C375" s="25">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="D375" s="26">
         <v>7.2</v>
       </c>
       <c r="E375" s="27">
-        <v>3.6</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="376" spans="1:5" x14ac:dyDescent="0.25">
@@ -8578,16 +8576,16 @@
         <v>379</v>
       </c>
       <c r="B377" s="24">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C377" s="25">
-        <v>4.5</v>
+        <v>4</v>
       </c>
       <c r="D377" s="26">
         <v>7.13</v>
       </c>
       <c r="E377" s="27">
-        <v>32.090000000000003</v>
+        <v>28.52</v>
       </c>
     </row>
     <row r="378" spans="1:5" x14ac:dyDescent="0.25">
@@ -8612,16 +8610,16 @@
         <v>381</v>
       </c>
       <c r="B379" s="24">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="C379" s="25">
-        <v>16.5</v>
+        <v>12</v>
       </c>
       <c r="D379" s="26">
         <v>6.6</v>
       </c>
       <c r="E379" s="27">
-        <v>108.9</v>
+        <v>79.2</v>
       </c>
     </row>
     <row r="380" spans="1:5" x14ac:dyDescent="0.25">
@@ -8680,16 +8678,16 @@
         <v>385</v>
       </c>
       <c r="B383" s="24">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C383" s="25">
-        <v>20.5</v>
+        <v>17.5</v>
       </c>
       <c r="D383" s="26">
         <v>7.31</v>
       </c>
       <c r="E383" s="27">
-        <v>149.94999999999999</v>
+        <v>128.01</v>
       </c>
     </row>
     <row r="384" spans="1:5" x14ac:dyDescent="0.25">
@@ -8765,16 +8763,16 @@
         <v>390</v>
       </c>
       <c r="B388" s="24">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C388" s="25">
-        <v>8.5</v>
+        <v>5.5</v>
       </c>
       <c r="D388" s="26">
         <v>7</v>
       </c>
       <c r="E388" s="27">
-        <v>59.5</v>
+        <v>38.5</v>
       </c>
     </row>
     <row r="389" spans="1:5" x14ac:dyDescent="0.25">
@@ -8793,16 +8791,16 @@
         <v>392</v>
       </c>
       <c r="B390" s="24">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C390" s="25">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="D390" s="26">
         <v>3.6</v>
       </c>
       <c r="E390" s="27">
-        <v>16.2</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="391" spans="1:5" x14ac:dyDescent="0.25">
@@ -8813,13 +8811,13 @@
         <v>57</v>
       </c>
       <c r="C391" s="25">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D391" s="26">
         <v>6</v>
       </c>
       <c r="E391" s="27">
-        <v>120</v>
+        <v>126</v>
       </c>
     </row>
     <row r="392" spans="1:5" x14ac:dyDescent="0.25">
@@ -9053,16 +9051,16 @@
         <v>408</v>
       </c>
       <c r="B406" s="24">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C406" s="25">
-        <v>10.5</v>
+        <v>6.5</v>
       </c>
       <c r="D406" s="26">
         <v>8.5500000000000007</v>
       </c>
       <c r="E406" s="27">
-        <v>89.78</v>
+        <v>55.58</v>
       </c>
     </row>
     <row r="407" spans="1:5" x14ac:dyDescent="0.25">
@@ -9261,16 +9259,16 @@
         <v>422</v>
       </c>
       <c r="B420" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C420" s="25">
-        <v>47.5</v>
+        <v>47</v>
       </c>
       <c r="D420" s="26">
         <v>5.7</v>
       </c>
       <c r="E420" s="27">
-        <v>270.75</v>
+        <v>267.89999999999998</v>
       </c>
     </row>
     <row r="421" spans="1:5" x14ac:dyDescent="0.25">
@@ -9963,16 +9961,16 @@
         <v>470</v>
       </c>
       <c r="B468" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C468" s="25">
-        <v>2.5</v>
+        <v>1.5</v>
       </c>
       <c r="D468" s="26">
         <v>22.5</v>
       </c>
       <c r="E468" s="27">
-        <v>56.25</v>
+        <v>33.75</v>
       </c>
     </row>
     <row r="469" spans="1:5" x14ac:dyDescent="0.25">
@@ -10207,16 +10205,16 @@
         <v>486</v>
       </c>
       <c r="B484" s="24">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C484" s="25">
-        <v>7.5</v>
+        <v>12.5</v>
       </c>
       <c r="D484" s="26">
         <v>9.5</v>
       </c>
       <c r="E484" s="27">
-        <v>71.25</v>
+        <v>118.75</v>
       </c>
     </row>
     <row r="485" spans="1:5" x14ac:dyDescent="0.25">
@@ -10353,16 +10351,16 @@
         <v>496</v>
       </c>
       <c r="B494" s="24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C494" s="25">
-        <v>14.5</v>
+        <v>13.5</v>
       </c>
       <c r="D494" s="26">
         <v>13</v>
       </c>
       <c r="E494" s="27">
-        <v>188.5</v>
+        <v>175.5</v>
       </c>
     </row>
     <row r="495" spans="1:5" x14ac:dyDescent="0.25">
@@ -10443,16 +10441,16 @@
         <v>502</v>
       </c>
       <c r="B500" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C500" s="25">
-        <v>5</v>
+        <v>3.5</v>
       </c>
       <c r="D500" s="26">
         <v>10.45</v>
       </c>
       <c r="E500" s="27">
-        <v>52.25</v>
+        <v>36.58</v>
       </c>
     </row>
     <row r="501" spans="1:5" x14ac:dyDescent="0.25">
@@ -10792,16 +10790,16 @@
         <v>525</v>
       </c>
       <c r="B523" s="24">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C523" s="25">
-        <v>8.5</v>
+        <v>10</v>
       </c>
       <c r="D523" s="26">
         <v>12.8</v>
       </c>
       <c r="E523" s="27">
-        <v>108.8</v>
+        <v>128</v>
       </c>
     </row>
     <row r="524" spans="1:5" x14ac:dyDescent="0.25">
@@ -11074,13 +11072,13 @@
         <v>25</v>
       </c>
       <c r="C540" s="25">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="D540" s="26">
         <v>2</v>
       </c>
       <c r="E540" s="27">
-        <v>60</v>
+        <v>52</v>
       </c>
     </row>
     <row r="541" spans="1:5" x14ac:dyDescent="0.25">
@@ -11171,16 +11169,16 @@
         <v>548</v>
       </c>
       <c r="B546" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C546" s="25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D546" s="26">
         <v>3.5</v>
       </c>
       <c r="E546" s="27">
-        <v>17.5</v>
+        <v>14</v>
       </c>
     </row>
     <row r="547" spans="1:5" x14ac:dyDescent="0.25">
@@ -11222,16 +11220,16 @@
         <v>551</v>
       </c>
       <c r="B549" s="24">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C549" s="25">
-        <v>56.5</v>
+        <v>55.5</v>
       </c>
       <c r="D549" s="26">
         <v>2.82</v>
       </c>
       <c r="E549" s="27">
-        <v>159.13</v>
+        <v>156.32</v>
       </c>
     </row>
     <row r="550" spans="1:5" x14ac:dyDescent="0.25">
@@ -11403,16 +11401,16 @@
         <v>562</v>
       </c>
       <c r="B560" s="24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C560" s="25">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="D560" s="26">
         <v>4.75</v>
       </c>
       <c r="E560" s="27">
-        <v>26.13</v>
+        <v>21.38</v>
       </c>
     </row>
     <row r="561" spans="1:5" x14ac:dyDescent="0.25">
@@ -11505,16 +11503,16 @@
         <v>568</v>
       </c>
       <c r="B566" s="24">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="C566" s="25">
-        <v>41.5</v>
+        <v>39.5</v>
       </c>
       <c r="D566" s="26">
         <v>3.9</v>
       </c>
       <c r="E566" s="27">
-        <v>161.85</v>
+        <v>154.05000000000001</v>
       </c>
     </row>
     <row r="567" spans="1:5" x14ac:dyDescent="0.25">
@@ -11556,16 +11554,16 @@
         <v>571</v>
       </c>
       <c r="B569" s="24">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C569" s="25">
-        <v>8.5</v>
+        <v>9.5</v>
       </c>
       <c r="D569" s="26">
         <v>2.66</v>
       </c>
       <c r="E569" s="27">
-        <v>22.61</v>
+        <v>25.27</v>
       </c>
     </row>
     <row r="570" spans="1:5" x14ac:dyDescent="0.25">
@@ -11627,13 +11625,13 @@
         <v>68</v>
       </c>
       <c r="C573" s="25">
-        <v>1.5</v>
+        <v>4.5</v>
       </c>
       <c r="D573" s="26">
         <v>3.14</v>
       </c>
       <c r="E573" s="27">
-        <v>4.71</v>
+        <v>14.14</v>
       </c>
     </row>
     <row r="574" spans="1:5" x14ac:dyDescent="0.25">
@@ -11641,16 +11639,16 @@
         <v>576</v>
       </c>
       <c r="B574" s="24">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C574" s="25">
-        <v>46.25</v>
+        <v>44.75</v>
       </c>
       <c r="D574" s="26">
         <v>2.2999999999999998</v>
       </c>
       <c r="E574" s="27">
-        <v>106.38</v>
+        <v>102.93</v>
       </c>
     </row>
     <row r="575" spans="1:5" x14ac:dyDescent="0.25">
@@ -11771,16 +11769,16 @@
         <v>584</v>
       </c>
       <c r="B582" s="24">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C582" s="25">
-        <v>32.5</v>
+        <v>31.5</v>
       </c>
       <c r="D582" s="26">
         <v>2.66</v>
       </c>
       <c r="E582" s="27">
-        <v>86.45</v>
+        <v>83.79</v>
       </c>
     </row>
     <row r="583" spans="1:5" x14ac:dyDescent="0.25">
@@ -11907,16 +11905,16 @@
         <v>592</v>
       </c>
       <c r="B590" s="24">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C590" s="25">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="D590" s="26">
         <v>1.2</v>
       </c>
       <c r="E590" s="27">
-        <v>60</v>
+        <v>63.6</v>
       </c>
     </row>
     <row r="591" spans="1:5" x14ac:dyDescent="0.25">
@@ -12040,16 +12038,16 @@
         <v>601</v>
       </c>
       <c r="B599" s="24">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C599" s="25">
-        <v>243.5</v>
+        <v>239.5</v>
       </c>
       <c r="D599" s="26">
         <v>1.5</v>
       </c>
       <c r="E599" s="27">
-        <v>365.25</v>
+        <v>359.25</v>
       </c>
     </row>
     <row r="600" spans="1:5" x14ac:dyDescent="0.25">
@@ -12057,10 +12055,10 @@
         <v>602</v>
       </c>
       <c r="B600" s="24">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C600" s="25">
-        <v>-146.5</v>
+        <v>-222.5</v>
       </c>
       <c r="D600" s="29"/>
       <c r="E600" s="28"/>
@@ -12070,10 +12068,10 @@
         <v>603</v>
       </c>
       <c r="B601" s="24">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="C601" s="25">
-        <v>-74.5</v>
+        <v>-80.5</v>
       </c>
       <c r="D601" s="29"/>
       <c r="E601" s="28"/>
@@ -12085,9 +12083,7 @@
       <c r="B602" s="24">
         <v>173</v>
       </c>
-      <c r="C602" s="25">
-        <v>11</v>
-      </c>
+      <c r="C602" s="28"/>
       <c r="D602" s="29"/>
       <c r="E602" s="28"/>
     </row>
@@ -12096,10 +12092,10 @@
         <v>605</v>
       </c>
       <c r="B603" s="24">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C603" s="25">
-        <v>-18</v>
+        <v>-24</v>
       </c>
       <c r="D603" s="29"/>
       <c r="E603" s="28"/>
@@ -12122,16 +12118,16 @@
         <v>607</v>
       </c>
       <c r="B605" s="24">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="C605" s="25">
-        <v>107</v>
+        <v>92.5</v>
       </c>
       <c r="D605" s="26">
         <v>0.87</v>
       </c>
       <c r="E605" s="27">
-        <v>93.09</v>
+        <v>80.48</v>
       </c>
     </row>
     <row r="606" spans="1:5" x14ac:dyDescent="0.25">
@@ -12139,16 +12135,16 @@
         <v>608</v>
       </c>
       <c r="B606" s="24">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="C606" s="25">
-        <v>388</v>
+        <v>378</v>
       </c>
       <c r="D606" s="26">
         <v>0.57999999999999996</v>
       </c>
       <c r="E606" s="27">
-        <v>225.04</v>
+        <v>219.24</v>
       </c>
     </row>
     <row r="607" spans="1:5" x14ac:dyDescent="0.25">
@@ -12156,16 +12152,16 @@
         <v>609</v>
       </c>
       <c r="B607" s="24">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="C607" s="25">
-        <v>904</v>
+        <v>896</v>
       </c>
       <c r="D607" s="26">
         <v>0.85</v>
       </c>
       <c r="E607" s="27">
-        <v>768.4</v>
+        <v>761.6</v>
       </c>
     </row>
     <row r="608" spans="1:5" x14ac:dyDescent="0.25">
@@ -12184,16 +12180,16 @@
         <v>611</v>
       </c>
       <c r="B609" s="24">
-        <v>200</v>
+        <v>204</v>
       </c>
       <c r="C609" s="25">
-        <v>143.5</v>
+        <v>132.5</v>
       </c>
       <c r="D609" s="26">
         <v>0.85</v>
       </c>
       <c r="E609" s="27">
-        <v>121.98</v>
+        <v>112.63</v>
       </c>
     </row>
     <row r="610" spans="1:5" x14ac:dyDescent="0.25">
@@ -12642,16 +12638,16 @@
         <v>641</v>
       </c>
       <c r="B639" s="24">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C639" s="25">
-        <v>20.5</v>
+        <v>13.5</v>
       </c>
       <c r="D639" s="26">
         <v>3.5</v>
       </c>
       <c r="E639" s="27">
-        <v>71.75</v>
+        <v>47.25</v>
       </c>
     </row>
     <row r="640" spans="1:5" x14ac:dyDescent="0.25">
@@ -12676,16 +12672,16 @@
         <v>643</v>
       </c>
       <c r="B641" s="24">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C641" s="25">
-        <v>-1.65</v>
+        <v>4.3499999999999996</v>
       </c>
       <c r="D641" s="26">
         <v>4</v>
       </c>
       <c r="E641" s="27">
-        <v>-6.6</v>
+        <v>17.399999999999999</v>
       </c>
     </row>
     <row r="642" spans="1:5" x14ac:dyDescent="0.25">
@@ -12727,17 +12723,11 @@
         <v>646</v>
       </c>
       <c r="B644" s="24">
-        <v>125</v>
-      </c>
-      <c r="C644" s="25">
-        <v>11</v>
-      </c>
-      <c r="D644" s="26">
-        <v>2.77</v>
-      </c>
-      <c r="E644" s="27">
-        <v>30.43</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="C644" s="28"/>
+      <c r="D644" s="29"/>
+      <c r="E644" s="28"/>
     </row>
     <row r="645" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A645" s="23" t="s">
@@ -12792,13 +12782,13 @@
         <v>62</v>
       </c>
       <c r="C648" s="25">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D648" s="26">
         <v>4</v>
       </c>
       <c r="E648" s="27">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="649" spans="1:5" x14ac:dyDescent="0.25">
@@ -12868,16 +12858,16 @@
         <v>655</v>
       </c>
       <c r="B653" s="24">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="C653" s="25">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="D653" s="26">
         <v>2.2799999999999998</v>
       </c>
       <c r="E653" s="27">
-        <v>111.72</v>
+        <v>107.16</v>
       </c>
     </row>
     <row r="654" spans="1:5" x14ac:dyDescent="0.25">
@@ -12947,16 +12937,16 @@
         <v>660</v>
       </c>
       <c r="B658" s="24">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C658" s="25">
-        <v>13.5</v>
+        <v>15.5</v>
       </c>
       <c r="D658" s="26">
         <v>4.6500000000000004</v>
       </c>
       <c r="E658" s="27">
-        <v>62.78</v>
+        <v>72.08</v>
       </c>
     </row>
     <row r="659" spans="1:5" x14ac:dyDescent="0.25">
@@ -12998,16 +12988,16 @@
         <v>663</v>
       </c>
       <c r="B661" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C661" s="25">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="D661" s="26">
         <v>3.5</v>
       </c>
       <c r="E661" s="27">
-        <v>22.75</v>
+        <v>19.25</v>
       </c>
     </row>
     <row r="662" spans="1:5" x14ac:dyDescent="0.25">
@@ -13026,16 +13016,16 @@
         <v>665</v>
       </c>
       <c r="B663" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C663" s="25">
-        <v>4.5</v>
+        <v>2.5</v>
       </c>
       <c r="D663" s="26">
         <v>5.45</v>
       </c>
       <c r="E663" s="27">
-        <v>24.53</v>
+        <v>13.63</v>
       </c>
     </row>
     <row r="664" spans="1:5" x14ac:dyDescent="0.25">
@@ -13077,16 +13067,16 @@
         <v>668</v>
       </c>
       <c r="B666" s="24">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C666" s="25">
-        <v>26.5</v>
+        <v>25.5</v>
       </c>
       <c r="D666" s="26">
         <v>3.33</v>
       </c>
       <c r="E666" s="27">
-        <v>88.25</v>
+        <v>84.92</v>
       </c>
     </row>
     <row r="667" spans="1:5" x14ac:dyDescent="0.25">
@@ -13114,13 +13104,13 @@
         <v>43</v>
       </c>
       <c r="C668" s="25">
-        <v>1</v>
+        <v>2.5</v>
       </c>
       <c r="D668" s="26">
         <v>3.5</v>
       </c>
       <c r="E668" s="27">
-        <v>3.5</v>
+        <v>8.75</v>
       </c>
     </row>
     <row r="669" spans="1:5" x14ac:dyDescent="0.25">
@@ -13145,16 +13135,16 @@
         <v>672</v>
       </c>
       <c r="B670" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C670" s="25">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="D670" s="26">
         <v>8.75</v>
       </c>
       <c r="E670" s="27">
-        <v>48.13</v>
+        <v>26.25</v>
       </c>
     </row>
     <row r="671" spans="1:5" x14ac:dyDescent="0.25">
@@ -13162,16 +13152,16 @@
         <v>673</v>
       </c>
       <c r="B671" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C671" s="25">
-        <v>7.5</v>
+        <v>5</v>
       </c>
       <c r="D671" s="26">
         <v>6.25</v>
       </c>
       <c r="E671" s="27">
-        <v>46.88</v>
+        <v>31.25</v>
       </c>
     </row>
     <row r="672" spans="1:5" x14ac:dyDescent="0.25">
@@ -13179,16 +13169,16 @@
         <v>674</v>
       </c>
       <c r="B672" s="24">
-        <v>208</v>
+        <v>212</v>
       </c>
       <c r="C672" s="25">
-        <v>37</v>
+        <v>31.5</v>
       </c>
       <c r="D672" s="26">
         <v>2.85</v>
       </c>
       <c r="E672" s="27">
-        <v>105.45</v>
+        <v>89.78</v>
       </c>
     </row>
     <row r="673" spans="1:5" x14ac:dyDescent="0.25">
@@ -13246,16 +13236,16 @@
         <v>679</v>
       </c>
       <c r="B677" s="24">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="C677" s="25">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D677" s="26">
         <v>3.1</v>
       </c>
       <c r="E677" s="27">
-        <v>102.3</v>
+        <v>86.8</v>
       </c>
     </row>
     <row r="678" spans="1:5" x14ac:dyDescent="0.25">
@@ -13263,16 +13253,16 @@
         <v>680</v>
       </c>
       <c r="B678" s="24">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="C678" s="25">
-        <v>24</v>
+        <v>22.5</v>
       </c>
       <c r="D678" s="26">
         <v>5.73</v>
       </c>
       <c r="E678" s="27">
-        <v>137.56</v>
+        <v>128.97</v>
       </c>
     </row>
     <row r="679" spans="1:5" x14ac:dyDescent="0.25">
@@ -13297,16 +13287,16 @@
         <v>682</v>
       </c>
       <c r="B680" s="24">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C680" s="25">
-        <v>19</v>
+        <v>8.5</v>
       </c>
       <c r="D680" s="26">
         <v>4.8</v>
       </c>
       <c r="E680" s="27">
-        <v>91.2</v>
+        <v>40.799999999999997</v>
       </c>
     </row>
     <row r="681" spans="1:5" x14ac:dyDescent="0.25">
@@ -13398,16 +13388,16 @@
         <v>689</v>
       </c>
       <c r="B687" s="24">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C687" s="25">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="D687" s="26">
         <v>3.1</v>
       </c>
       <c r="E687" s="27">
-        <v>403</v>
+        <v>387.5</v>
       </c>
     </row>
     <row r="688" spans="1:5" x14ac:dyDescent="0.25">
@@ -13466,16 +13456,16 @@
         <v>693</v>
       </c>
       <c r="B691" s="24">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C691" s="25">
-        <v>-26.5</v>
+        <v>-9.5</v>
       </c>
       <c r="D691" s="26">
         <v>3.75</v>
       </c>
       <c r="E691" s="27">
-        <v>-99.38</v>
+        <v>-35.630000000000003</v>
       </c>
     </row>
     <row r="692" spans="1:5" x14ac:dyDescent="0.25">
@@ -13562,16 +13552,16 @@
         <v>699</v>
       </c>
       <c r="B697" s="24">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C697" s="25">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="D697" s="26">
         <v>2.25</v>
       </c>
       <c r="E697" s="27">
-        <v>65.25</v>
+        <v>72</v>
       </c>
     </row>
     <row r="698" spans="1:5" x14ac:dyDescent="0.25">
@@ -13596,16 +13586,16 @@
         <v>701</v>
       </c>
       <c r="B699" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C699" s="25">
-        <v>13.5</v>
+        <v>10.5</v>
       </c>
       <c r="D699" s="26">
         <v>2.75</v>
       </c>
       <c r="E699" s="27">
-        <v>37.130000000000003</v>
+        <v>28.88</v>
       </c>
     </row>
     <row r="700" spans="1:5" x14ac:dyDescent="0.25">
@@ -13630,16 +13620,16 @@
         <v>703</v>
       </c>
       <c r="B701" s="24">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C701" s="25">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="D701" s="26">
         <v>2.75</v>
       </c>
       <c r="E701" s="27">
-        <v>44</v>
+        <v>33</v>
       </c>
     </row>
     <row r="702" spans="1:5" x14ac:dyDescent="0.25">
@@ -13826,7 +13816,7 @@
         <v>77</v>
       </c>
       <c r="C714" s="25">
-        <v>-4</v>
+        <v>-5.5</v>
       </c>
       <c r="D714" s="29"/>
       <c r="E714" s="28"/>
@@ -13836,10 +13826,10 @@
         <v>717</v>
       </c>
       <c r="B715" s="24">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C715" s="25">
-        <v>-3</v>
+        <v>2</v>
       </c>
       <c r="D715" s="29"/>
       <c r="E715" s="28"/>
@@ -13875,10 +13865,10 @@
         <v>720</v>
       </c>
       <c r="B718" s="24">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C718" s="25">
-        <v>5.5</v>
+        <v>3.5</v>
       </c>
       <c r="D718" s="29"/>
       <c r="E718" s="28"/>
@@ -13900,13 +13890,13 @@
         <v>78</v>
       </c>
       <c r="C720" s="25">
-        <v>43</v>
+        <v>45.5</v>
       </c>
       <c r="D720" s="26">
         <v>2.93</v>
       </c>
       <c r="E720" s="27">
-        <v>126.06</v>
+        <v>133.38999999999999</v>
       </c>
     </row>
     <row r="721" spans="1:5" x14ac:dyDescent="0.25">
@@ -14345,10 +14335,10 @@
         <v>754</v>
       </c>
       <c r="B752" s="24">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="C752" s="25">
-        <v>-895.7</v>
+        <v>-898.2</v>
       </c>
       <c r="D752" s="29"/>
       <c r="E752" s="28"/>
@@ -14359,11 +14349,11 @@
       </c>
       <c r="B753" s="31"/>
       <c r="C753" s="32">
-        <v>27196.84</v>
+        <v>26131.84</v>
       </c>
       <c r="D753" s="33"/>
       <c r="E753" s="34">
-        <v>60534.55</v>
+        <v>58616.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
NIkhil 0904 @ 925
</commit_message>
<xml_diff>
--- a/data/website stock.xlsx
+++ b/data/website stock.xlsx
@@ -140,7 +140,7 @@
     <t>1024 PATRIKA</t>
   </si>
   <si>
-    <t>1025 PATRIKA-(10 Apr)</t>
+    <t>1025 PATRIKA</t>
   </si>
   <si>
     <t>1026 PATRIKA (JC)</t>
@@ -698,7 +698,7 @@
     <t>4287 PATRIKA</t>
   </si>
   <si>
-    <t>4288 PATRIKA (TIME LAGEGA)-(10 Apr)</t>
+    <t>4288 PATRIKA Design Change</t>
   </si>
   <si>
     <t>4289 PATRIKA (TIME LAGEGA)-(10 Apr)</t>
@@ -716,7 +716,7 @@
     <t>4293 PATRIKA</t>
   </si>
   <si>
-    <t>4294 PATRIKA-(9 Apr)</t>
+    <t>4294 PATRIKA</t>
   </si>
   <si>
     <t>4295 PATRIKA</t>
@@ -875,7 +875,7 @@
     <t>5079 PATRIKA</t>
   </si>
   <si>
-    <t>5080 PATRIKA (2800-10)</t>
+    <t>5080 PATRIKA</t>
   </si>
   <si>
     <t>5081 PATRIKA</t>
@@ -956,7 +956,7 @@
     <t>5108 PATRIKA (DCU)</t>
   </si>
   <si>
-    <t>5109 PATRIKA (800) SATURDAY</t>
+    <t>5109 PATRIKA</t>
   </si>
   <si>
     <t>5110 PATRIKA (JC)</t>
@@ -1721,7 +1721,7 @@
     <t>7425 PATRIKA</t>
   </si>
   <si>
-    <t>7426 PATRIKA (F/G) *-*</t>
+    <t>7426 PATRIKA (F/G) *-* (Dc)</t>
   </si>
   <si>
     <t>7427 PATRIKA</t>
@@ -2991,16 +2991,16 @@
         <v>16</v>
       </c>
       <c r="B14" s="24">
-        <v>184</v>
+        <v>190</v>
       </c>
       <c r="C14" s="25">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="D14" s="26">
         <v>2</v>
       </c>
       <c r="E14" s="27">
-        <v>200</v>
+        <v>164</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -3036,16 +3036,16 @@
         <v>19</v>
       </c>
       <c r="B17" s="24">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="C17" s="25">
-        <v>131</v>
+        <v>114.5</v>
       </c>
       <c r="D17" s="26">
         <v>2.1</v>
       </c>
       <c r="E17" s="27">
-        <v>275.10000000000002</v>
+        <v>240.45</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -3126,16 +3126,16 @@
         <v>25</v>
       </c>
       <c r="B23" s="24">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="C23" s="25">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D23" s="26">
         <v>1.8</v>
       </c>
       <c r="E23" s="27">
-        <v>82.8</v>
+        <v>77.400000000000006</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -3194,16 +3194,16 @@
         <v>29</v>
       </c>
       <c r="B27" s="24">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="C27" s="25">
-        <v>22</v>
+        <v>12</v>
       </c>
       <c r="D27" s="26">
         <v>2</v>
       </c>
       <c r="E27" s="27">
-        <v>44</v>
+        <v>24</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3211,16 +3211,16 @@
         <v>30</v>
       </c>
       <c r="B28" s="24">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C28" s="25">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="D28" s="26">
         <v>2</v>
       </c>
       <c r="E28" s="27">
-        <v>372</v>
+        <v>366</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -3262,16 +3262,16 @@
         <v>33</v>
       </c>
       <c r="B31" s="24">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C31" s="25">
-        <v>33.5</v>
+        <v>30.5</v>
       </c>
       <c r="D31" s="26">
         <v>2.85</v>
       </c>
       <c r="E31" s="27">
-        <v>95.48</v>
+        <v>86.93</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -3279,16 +3279,16 @@
         <v>34</v>
       </c>
       <c r="B32" s="24">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C32" s="25">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D32" s="26">
         <v>2.8</v>
       </c>
       <c r="E32" s="27">
-        <v>92.4</v>
+        <v>81.2</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
@@ -3307,16 +3307,16 @@
         <v>36</v>
       </c>
       <c r="B34" s="24">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C34" s="25">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D34" s="26">
         <v>2.5</v>
       </c>
       <c r="E34" s="27">
-        <v>50</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -3341,11 +3341,17 @@
         <v>38</v>
       </c>
       <c r="B36" s="24">
-        <v>91</v>
-      </c>
-      <c r="C36" s="28"/>
-      <c r="D36" s="29"/>
-      <c r="E36" s="28"/>
+        <v>95</v>
+      </c>
+      <c r="C36" s="25">
+        <v>48</v>
+      </c>
+      <c r="D36" s="26">
+        <v>2.2999999999999998</v>
+      </c>
+      <c r="E36" s="27">
+        <v>110.4</v>
+      </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" s="23" t="s">
@@ -3391,16 +3397,16 @@
         <v>42</v>
       </c>
       <c r="B40" s="24">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C40" s="25">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="D40" s="26">
         <v>2.14</v>
       </c>
       <c r="E40" s="27">
-        <v>166.92</v>
+        <v>162.63999999999999</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -3408,16 +3414,16 @@
         <v>43</v>
       </c>
       <c r="B41" s="24">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C41" s="25">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D41" s="26">
         <v>2.14</v>
       </c>
       <c r="E41" s="27">
-        <v>14.98</v>
+        <v>2.14</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -3425,16 +3431,16 @@
         <v>44</v>
       </c>
       <c r="B42" s="24">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C42" s="25">
-        <v>24</v>
+        <v>-14</v>
       </c>
       <c r="D42" s="26">
         <v>2.4500000000000002</v>
       </c>
       <c r="E42" s="27">
-        <v>58.89</v>
+        <v>-34.35</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.25">
@@ -3442,16 +3448,16 @@
         <v>45</v>
       </c>
       <c r="B43" s="24">
-        <v>208</v>
+        <v>216</v>
       </c>
       <c r="C43" s="25">
-        <v>32.5</v>
+        <v>12</v>
       </c>
       <c r="D43" s="26">
         <v>2.4700000000000002</v>
       </c>
       <c r="E43" s="27">
-        <v>80.290000000000006</v>
+        <v>29.64</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -3476,16 +3482,16 @@
         <v>47</v>
       </c>
       <c r="B45" s="24">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="C45" s="25">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D45" s="26">
         <v>2.66</v>
       </c>
       <c r="E45" s="27">
-        <v>10.64</v>
+        <v>5.32</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.25">
@@ -3515,16 +3521,16 @@
         <v>50</v>
       </c>
       <c r="B48" s="24">
-        <v>160</v>
+        <v>164</v>
       </c>
       <c r="C48" s="25">
-        <v>253.5</v>
+        <v>230.5</v>
       </c>
       <c r="D48" s="26">
         <v>1.26</v>
       </c>
       <c r="E48" s="27">
-        <v>319.45</v>
+        <v>290.47000000000003</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.25">
@@ -3566,16 +3572,16 @@
         <v>53</v>
       </c>
       <c r="B51" s="24">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C51" s="25">
-        <v>151</v>
+        <v>141.5</v>
       </c>
       <c r="D51" s="26">
         <v>1.8</v>
       </c>
       <c r="E51" s="27">
-        <v>271.8</v>
+        <v>254.7</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.25">
@@ -3583,16 +3589,16 @@
         <v>54</v>
       </c>
       <c r="B52" s="24">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C52" s="25">
-        <v>63.5</v>
+        <v>54.5</v>
       </c>
       <c r="D52" s="26">
         <v>2.5</v>
       </c>
       <c r="E52" s="27">
-        <v>158.75</v>
+        <v>136.25</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.25">
@@ -3600,16 +3606,16 @@
         <v>55</v>
       </c>
       <c r="B53" s="24">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C53" s="25">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D53" s="26">
         <v>2.5</v>
       </c>
       <c r="E53" s="27">
-        <v>565</v>
+        <v>560</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -3617,16 +3623,16 @@
         <v>56</v>
       </c>
       <c r="B54" s="24">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="C54" s="25">
-        <v>63</v>
+        <v>57.5</v>
       </c>
       <c r="D54" s="26">
         <v>2.75</v>
       </c>
       <c r="E54" s="27">
-        <v>173.25</v>
+        <v>158.13</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.25">
@@ -3634,16 +3640,16 @@
         <v>57</v>
       </c>
       <c r="B55" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C55" s="25">
-        <v>176.15</v>
+        <v>168.15</v>
       </c>
       <c r="D55" s="26">
         <v>2.75</v>
       </c>
       <c r="E55" s="27">
-        <v>484.41</v>
+        <v>462.41</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.25">
@@ -3668,16 +3674,16 @@
         <v>59</v>
       </c>
       <c r="B57" s="24">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C57" s="25">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="D57" s="26">
         <v>1.9</v>
       </c>
       <c r="E57" s="27">
-        <v>119.7</v>
+        <v>108.3</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.25">
@@ -3696,16 +3702,16 @@
         <v>61</v>
       </c>
       <c r="B59" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C59" s="25">
-        <v>16.25</v>
+        <v>14.25</v>
       </c>
       <c r="D59" s="26">
         <v>1.9</v>
       </c>
       <c r="E59" s="27">
-        <v>30.88</v>
+        <v>27.08</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.25">
@@ -3730,16 +3736,16 @@
         <v>63</v>
       </c>
       <c r="B61" s="24">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="C61" s="25">
-        <v>526.5</v>
+        <v>519.5</v>
       </c>
       <c r="D61" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E61" s="27">
-        <v>599.86</v>
+        <v>591.89</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -3792,16 +3798,16 @@
         <v>67</v>
       </c>
       <c r="B65" s="24">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="C65" s="25">
-        <v>469</v>
+        <v>459</v>
       </c>
       <c r="D65" s="26">
         <v>1.65</v>
       </c>
       <c r="E65" s="27">
-        <v>773.85</v>
+        <v>757.35</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.25">
@@ -3837,16 +3843,16 @@
         <v>70</v>
       </c>
       <c r="B68" s="24">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="C68" s="25">
-        <v>317</v>
+        <v>290</v>
       </c>
       <c r="D68" s="26">
         <v>1.65</v>
       </c>
       <c r="E68" s="27">
-        <v>523.04999999999995</v>
+        <v>478.5</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -3865,16 +3871,16 @@
         <v>72</v>
       </c>
       <c r="B70" s="24">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="C70" s="25">
-        <v>353.5</v>
+        <v>331.5</v>
       </c>
       <c r="D70" s="26">
         <v>1.4</v>
       </c>
       <c r="E70" s="27">
-        <v>494.9</v>
+        <v>464.1</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
@@ -3882,16 +3888,16 @@
         <v>73</v>
       </c>
       <c r="B71" s="24">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="C71" s="25">
-        <v>565</v>
+        <v>494</v>
       </c>
       <c r="D71" s="26">
         <v>1.4</v>
       </c>
       <c r="E71" s="27">
-        <v>791</v>
+        <v>691.6</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -3899,16 +3905,16 @@
         <v>74</v>
       </c>
       <c r="B72" s="24">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C72" s="25">
-        <v>422.5</v>
+        <v>367</v>
       </c>
       <c r="D72" s="26">
         <v>1.4</v>
       </c>
       <c r="E72" s="27">
-        <v>591.5</v>
+        <v>513.79999999999995</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.25">
@@ -3916,16 +3922,16 @@
         <v>75</v>
       </c>
       <c r="B73" s="24">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="C73" s="25">
-        <v>423</v>
+        <v>358</v>
       </c>
       <c r="D73" s="26">
         <v>1.4</v>
       </c>
       <c r="E73" s="27">
-        <v>592.20000000000005</v>
+        <v>501.2</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.25">
@@ -3933,16 +3939,16 @@
         <v>76</v>
       </c>
       <c r="B74" s="24">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="C74" s="25">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="D74" s="26">
         <v>1.2</v>
       </c>
       <c r="E74" s="27">
-        <v>115.2</v>
+        <v>112.8</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -3967,16 +3973,16 @@
         <v>78</v>
       </c>
       <c r="B76" s="24">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C76" s="25">
-        <v>354.5</v>
+        <v>279.5</v>
       </c>
       <c r="D76" s="26">
         <v>1.2</v>
       </c>
       <c r="E76" s="27">
-        <v>425.4</v>
+        <v>335.4</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
@@ -4001,16 +4007,16 @@
         <v>80</v>
       </c>
       <c r="B78" s="24">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="C78" s="25">
-        <v>272.5</v>
+        <v>217.5</v>
       </c>
       <c r="D78" s="26">
         <v>1.2</v>
       </c>
       <c r="E78" s="27">
-        <v>327</v>
+        <v>261</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
@@ -4018,16 +4024,16 @@
         <v>81</v>
       </c>
       <c r="B79" s="24">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C79" s="25">
-        <v>331</v>
+        <v>281</v>
       </c>
       <c r="D79" s="26">
         <v>1.2</v>
       </c>
       <c r="E79" s="27">
-        <v>397.2</v>
+        <v>337.2</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.25">
@@ -4035,16 +4041,16 @@
         <v>82</v>
       </c>
       <c r="B80" s="24">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C80" s="25">
-        <v>297.5</v>
+        <v>213.5</v>
       </c>
       <c r="D80" s="26">
         <v>1.2</v>
       </c>
       <c r="E80" s="27">
-        <v>357</v>
+        <v>256.2</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.25">
@@ -4052,16 +4058,16 @@
         <v>83</v>
       </c>
       <c r="B81" s="24">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C81" s="25">
-        <v>367.5</v>
+        <v>277.5</v>
       </c>
       <c r="D81" s="26">
         <v>1.2</v>
       </c>
       <c r="E81" s="27">
-        <v>441</v>
+        <v>333</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -4069,16 +4075,16 @@
         <v>84</v>
       </c>
       <c r="B82" s="24">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C82" s="25">
-        <v>162.5</v>
+        <v>120.5</v>
       </c>
       <c r="D82" s="26">
         <v>1.2</v>
       </c>
       <c r="E82" s="27">
-        <v>195</v>
+        <v>144.6</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.25">
@@ -4086,16 +4092,16 @@
         <v>85</v>
       </c>
       <c r="B83" s="24">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C83" s="25">
-        <v>446.5</v>
+        <v>441.5</v>
       </c>
       <c r="D83" s="26">
         <v>1.2</v>
       </c>
       <c r="E83" s="27">
-        <v>535.79999999999995</v>
+        <v>529.79999999999995</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
@@ -4103,16 +4109,16 @@
         <v>86</v>
       </c>
       <c r="B84" s="24">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="C84" s="25">
-        <v>362</v>
+        <v>320</v>
       </c>
       <c r="D84" s="26">
         <v>1.3</v>
       </c>
       <c r="E84" s="27">
-        <v>470.6</v>
+        <v>416</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
@@ -4120,16 +4126,16 @@
         <v>87</v>
       </c>
       <c r="B85" s="24">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="C85" s="25">
-        <v>854.5</v>
+        <v>829.5</v>
       </c>
       <c r="D85" s="26">
         <v>1.3</v>
       </c>
       <c r="E85" s="27">
-        <v>1110.8499999999999</v>
+        <v>1078.3499999999999</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
@@ -4137,16 +4143,16 @@
         <v>88</v>
       </c>
       <c r="B86" s="24">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="C86" s="25">
-        <v>873</v>
+        <v>851</v>
       </c>
       <c r="D86" s="26">
         <v>1.7</v>
       </c>
       <c r="E86" s="27">
-        <v>1484.1</v>
+        <v>1446.7</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.25">
@@ -4154,16 +4160,16 @@
         <v>89</v>
       </c>
       <c r="B87" s="24">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C87" s="25">
-        <v>418.5</v>
+        <v>402.5</v>
       </c>
       <c r="D87" s="26">
         <v>1.7</v>
       </c>
       <c r="E87" s="27">
-        <v>711.45</v>
+        <v>684.25</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -4171,16 +4177,16 @@
         <v>90</v>
       </c>
       <c r="B88" s="24">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C88" s="25">
-        <v>887.5</v>
+        <v>879.5</v>
       </c>
       <c r="D88" s="26">
         <v>1.7</v>
       </c>
       <c r="E88" s="27">
-        <v>1508.75</v>
+        <v>1495.15</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.25">
@@ -4188,16 +4194,16 @@
         <v>91</v>
       </c>
       <c r="B89" s="24">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="C89" s="25">
-        <v>-112</v>
+        <v>-34</v>
       </c>
       <c r="D89" s="26">
-        <v>1.47</v>
+        <v>1.49</v>
       </c>
       <c r="E89" s="27">
-        <v>-164.8</v>
+        <v>-50.55</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.25">
@@ -4205,16 +4211,16 @@
         <v>92</v>
       </c>
       <c r="B90" s="24">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C90" s="25">
-        <v>69.7</v>
+        <v>59.7</v>
       </c>
       <c r="D90" s="26">
         <v>1.28</v>
       </c>
       <c r="E90" s="27">
-        <v>89.4</v>
+        <v>76.58</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.25">
@@ -4222,16 +4228,16 @@
         <v>93</v>
       </c>
       <c r="B91" s="24">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C91" s="25">
-        <v>15.5</v>
+        <v>7</v>
       </c>
       <c r="D91" s="26">
         <v>1.22</v>
       </c>
       <c r="E91" s="27">
-        <v>18.91</v>
+        <v>8.5399999999999991</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.25">
@@ -4286,16 +4292,16 @@
         <v>97</v>
       </c>
       <c r="B95" s="24">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C95" s="25">
-        <v>87.5</v>
+        <v>80.5</v>
       </c>
       <c r="D95" s="26">
         <v>0.9</v>
       </c>
       <c r="E95" s="27">
-        <v>78.75</v>
+        <v>72.45</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.25">
@@ -4354,16 +4360,16 @@
         <v>101</v>
       </c>
       <c r="B99" s="24">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="C99" s="25">
-        <v>167</v>
+        <v>142</v>
       </c>
       <c r="D99" s="26">
         <v>1.65</v>
       </c>
       <c r="E99" s="27">
-        <v>275.55</v>
+        <v>234.3</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.25">
@@ -4480,16 +4486,16 @@
         <v>109</v>
       </c>
       <c r="B107" s="24">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C107" s="25">
-        <v>84.5</v>
+        <v>80.5</v>
       </c>
       <c r="D107" s="26">
         <v>2.5</v>
       </c>
       <c r="E107" s="27">
-        <v>211.25</v>
+        <v>201.25</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.25">
@@ -4497,16 +4503,16 @@
         <v>110</v>
       </c>
       <c r="B108" s="24">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C108" s="25">
-        <v>87</v>
+        <v>67</v>
       </c>
       <c r="D108" s="26">
         <v>2.5</v>
       </c>
       <c r="E108" s="27">
-        <v>217.5</v>
+        <v>167.5</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.25">
@@ -4514,10 +4520,10 @@
         <v>111</v>
       </c>
       <c r="B109" s="24">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C109" s="25">
-        <v>18</v>
+        <v>15.5</v>
       </c>
       <c r="D109" s="29"/>
       <c r="E109" s="28"/>
@@ -4601,10 +4607,10 @@
         <v>118</v>
       </c>
       <c r="B116" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C116" s="25">
-        <v>-2</v>
+        <v>-12</v>
       </c>
       <c r="D116" s="29"/>
       <c r="E116" s="28"/>
@@ -4653,10 +4659,10 @@
         <v>122</v>
       </c>
       <c r="B120" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C120" s="25">
-        <v>-62</v>
+        <v>40.5</v>
       </c>
       <c r="D120" s="29"/>
       <c r="E120" s="28"/>
@@ -4692,10 +4698,10 @@
         <v>125</v>
       </c>
       <c r="B123" s="24">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C123" s="25">
-        <v>-56</v>
+        <v>-76</v>
       </c>
       <c r="D123" s="29"/>
       <c r="E123" s="28"/>
@@ -4738,13 +4744,13 @@
         <v>84</v>
       </c>
       <c r="C126" s="25">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D126" s="26">
         <v>1.1499999999999999</v>
       </c>
       <c r="E126" s="27">
-        <v>4.5999999999999996</v>
+        <v>5.75</v>
       </c>
     </row>
     <row r="127" spans="1:5" x14ac:dyDescent="0.25">
@@ -4932,16 +4938,16 @@
         <v>143</v>
       </c>
       <c r="B141" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C141" s="25">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="D141" s="26">
         <v>12.5</v>
       </c>
       <c r="E141" s="27">
-        <v>31.25</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.25">
@@ -5016,16 +5022,16 @@
         <v>149</v>
       </c>
       <c r="B147" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C147" s="25">
-        <v>7</v>
+        <v>6.5</v>
       </c>
       <c r="D147" s="26">
         <v>12.5</v>
       </c>
       <c r="E147" s="27">
-        <v>87.5</v>
+        <v>81.25</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.25">
@@ -5101,16 +5107,16 @@
         <v>154</v>
       </c>
       <c r="B152" s="24">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C152" s="25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D152" s="26">
         <v>18.5</v>
       </c>
       <c r="E152" s="27">
-        <v>55.5</v>
+        <v>18.5</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.25">
@@ -5270,17 +5276,11 @@
         <v>165</v>
       </c>
       <c r="B163" s="24">
-        <v>38</v>
-      </c>
-      <c r="C163" s="25">
-        <v>-1</v>
-      </c>
-      <c r="D163" s="26">
-        <v>11.5</v>
-      </c>
-      <c r="E163" s="27">
-        <v>-11.5</v>
-      </c>
+        <v>37</v>
+      </c>
+      <c r="C163" s="28"/>
+      <c r="D163" s="29"/>
+      <c r="E163" s="28"/>
     </row>
     <row r="164" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A164" s="23" t="s">
@@ -5478,16 +5478,16 @@
         <v>179</v>
       </c>
       <c r="B177" s="24">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C177" s="25">
-        <v>92</v>
+        <v>82</v>
       </c>
       <c r="D177" s="26">
         <v>0.92</v>
       </c>
       <c r="E177" s="27">
-        <v>84.99</v>
+        <v>75.75</v>
       </c>
     </row>
     <row r="178" spans="1:5" x14ac:dyDescent="0.25">
@@ -5564,16 +5564,16 @@
         <v>185</v>
       </c>
       <c r="B183" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C183" s="25">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D183" s="26">
         <v>3.25</v>
       </c>
       <c r="E183" s="27">
-        <v>74.75</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="184" spans="1:5" x14ac:dyDescent="0.25">
@@ -5658,16 +5658,16 @@
         <v>191</v>
       </c>
       <c r="B189" s="24">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="C189" s="25">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D189" s="26">
         <v>2.8</v>
       </c>
       <c r="E189" s="27">
-        <v>280.18</v>
+        <v>271.77</v>
       </c>
     </row>
     <row r="190" spans="1:5" x14ac:dyDescent="0.25">
@@ -5692,16 +5692,16 @@
         <v>193</v>
       </c>
       <c r="B191" s="24">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="C191" s="25">
-        <v>13.5</v>
+        <v>2.5</v>
       </c>
       <c r="D191" s="26">
         <v>3.33</v>
       </c>
       <c r="E191" s="27">
-        <v>44.96</v>
+        <v>8.33</v>
       </c>
     </row>
     <row r="192" spans="1:5" x14ac:dyDescent="0.25">
@@ -5776,16 +5776,16 @@
         <v>199</v>
       </c>
       <c r="B197" s="24">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C197" s="25">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D197" s="26">
         <v>2.78</v>
       </c>
       <c r="E197" s="27">
-        <v>11.11</v>
+        <v>2.78</v>
       </c>
     </row>
     <row r="198" spans="1:5" x14ac:dyDescent="0.25">
@@ -5793,16 +5793,16 @@
         <v>200</v>
       </c>
       <c r="B198" s="24">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="C198" s="25">
-        <v>31.81</v>
+        <v>102.31</v>
       </c>
       <c r="D198" s="26">
         <v>2.65</v>
       </c>
       <c r="E198" s="27">
-        <v>84.3</v>
+        <v>271.12</v>
       </c>
     </row>
     <row r="199" spans="1:5" x14ac:dyDescent="0.25">
@@ -5849,16 +5849,16 @@
         <v>204</v>
       </c>
       <c r="B202" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C202" s="25">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="D202" s="26">
         <v>5</v>
       </c>
       <c r="E202" s="27">
-        <v>130</v>
+        <v>120</v>
       </c>
     </row>
     <row r="203" spans="1:5" x14ac:dyDescent="0.25">
@@ -5928,17 +5928,11 @@
         <v>209</v>
       </c>
       <c r="B207" s="24">
-        <v>74</v>
-      </c>
-      <c r="C207" s="25">
-        <v>-1</v>
-      </c>
-      <c r="D207" s="26">
-        <v>4.5</v>
-      </c>
-      <c r="E207" s="27">
-        <v>-4.5</v>
-      </c>
+        <v>75</v>
+      </c>
+      <c r="C207" s="28"/>
+      <c r="D207" s="29"/>
+      <c r="E207" s="28"/>
     </row>
     <row r="208" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A208" s="23" t="s">
@@ -5973,16 +5967,16 @@
         <v>212</v>
       </c>
       <c r="B210" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C210" s="25">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D210" s="26">
         <v>4.5</v>
       </c>
       <c r="E210" s="27">
-        <v>36</v>
+        <v>31.5</v>
       </c>
     </row>
     <row r="211" spans="1:5" x14ac:dyDescent="0.25">
@@ -6018,16 +6012,16 @@
         <v>215</v>
       </c>
       <c r="B213" s="24">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C213" s="25">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="D213" s="26">
         <v>2.7</v>
       </c>
       <c r="E213" s="27">
-        <v>318.60000000000002</v>
+        <v>288.89999999999998</v>
       </c>
     </row>
     <row r="214" spans="1:5" x14ac:dyDescent="0.25">
@@ -6035,16 +6029,16 @@
         <v>216</v>
       </c>
       <c r="B214" s="24">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="C214" s="25">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="D214" s="26">
         <v>2.6</v>
       </c>
       <c r="E214" s="27">
-        <v>101.4</v>
+        <v>75.400000000000006</v>
       </c>
     </row>
     <row r="215" spans="1:5" x14ac:dyDescent="0.25">
@@ -6103,16 +6097,16 @@
         <v>220</v>
       </c>
       <c r="B218" s="24">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C218" s="25">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D218" s="26">
         <v>3.5</v>
       </c>
       <c r="E218" s="27">
-        <v>38.5</v>
+        <v>28</v>
       </c>
     </row>
     <row r="219" spans="1:5" x14ac:dyDescent="0.25">
@@ -6171,16 +6165,16 @@
         <v>224</v>
       </c>
       <c r="B222" s="24">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C222" s="25">
-        <v>1</v>
+        <v>213.5</v>
       </c>
       <c r="D222" s="26">
         <v>2.7</v>
       </c>
       <c r="E222" s="27">
-        <v>2.7</v>
+        <v>576.45000000000005</v>
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.25">
@@ -6222,16 +6216,16 @@
         <v>227</v>
       </c>
       <c r="B225" s="24">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C225" s="25">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D225" s="26">
         <v>4.5</v>
       </c>
       <c r="E225" s="27">
-        <v>45</v>
+        <v>40.5</v>
       </c>
     </row>
     <row r="226" spans="1:5" x14ac:dyDescent="0.25">
@@ -6273,16 +6267,16 @@
         <v>230</v>
       </c>
       <c r="B228" s="24">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C228" s="25">
-        <v>85.5</v>
+        <v>52.5</v>
       </c>
       <c r="D228" s="26">
         <v>3.93</v>
       </c>
       <c r="E228" s="27">
-        <v>336.33</v>
+        <v>206.52</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.25">
@@ -6290,33 +6284,27 @@
         <v>231</v>
       </c>
       <c r="B229" s="24">
-        <v>175</v>
-      </c>
-      <c r="C229" s="25">
-        <v>2.25</v>
-      </c>
-      <c r="D229" s="26">
-        <v>3.25</v>
-      </c>
-      <c r="E229" s="27">
-        <v>7.31</v>
-      </c>
+        <v>176</v>
+      </c>
+      <c r="C229" s="28"/>
+      <c r="D229" s="29"/>
+      <c r="E229" s="28"/>
     </row>
     <row r="230" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A230" s="23" t="s">
         <v>232</v>
       </c>
       <c r="B230" s="24">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="C230" s="25">
-        <v>24.75</v>
+        <v>9.75</v>
       </c>
       <c r="D230" s="26">
         <v>3.65</v>
       </c>
       <c r="E230" s="27">
-        <v>90.43</v>
+        <v>35.630000000000003</v>
       </c>
     </row>
     <row r="231" spans="1:5" x14ac:dyDescent="0.25">
@@ -6369,16 +6357,16 @@
         <v>236</v>
       </c>
       <c r="B234" s="24">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="C234" s="25">
-        <v>8.5</v>
+        <v>3</v>
       </c>
       <c r="D234" s="26">
         <v>2.66</v>
       </c>
       <c r="E234" s="27">
-        <v>22.61</v>
+        <v>7.98</v>
       </c>
     </row>
     <row r="235" spans="1:5" x14ac:dyDescent="0.25">
@@ -6454,16 +6442,16 @@
         <v>241</v>
       </c>
       <c r="B239" s="24">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C239" s="25">
-        <v>77</v>
+        <v>70.5</v>
       </c>
       <c r="D239" s="26">
         <v>3.96</v>
       </c>
       <c r="E239" s="27">
-        <v>304.68</v>
+        <v>278.95999999999998</v>
       </c>
     </row>
     <row r="240" spans="1:5" x14ac:dyDescent="0.25">
@@ -6471,16 +6459,16 @@
         <v>242</v>
       </c>
       <c r="B240" s="24">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C240" s="25">
-        <v>-5.5</v>
+        <v>1</v>
       </c>
       <c r="D240" s="26">
         <v>3.5</v>
       </c>
       <c r="E240" s="27">
-        <v>-19.25</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="241" spans="1:5" x14ac:dyDescent="0.25">
@@ -6499,16 +6487,16 @@
         <v>244</v>
       </c>
       <c r="B242" s="24">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="C242" s="25">
-        <v>82.38</v>
+        <v>73.38</v>
       </c>
       <c r="D242" s="26">
         <v>3.25</v>
       </c>
       <c r="E242" s="27">
-        <v>267.74</v>
+        <v>238.49</v>
       </c>
     </row>
     <row r="243" spans="1:5" x14ac:dyDescent="0.25">
@@ -6727,16 +6715,16 @@
         <v>260</v>
       </c>
       <c r="B258" s="24">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C258" s="25">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="D258" s="26">
         <v>3.8</v>
       </c>
       <c r="E258" s="27">
-        <v>15.2</v>
+        <v>26.6</v>
       </c>
     </row>
     <row r="259" spans="1:5" x14ac:dyDescent="0.25">
@@ -6744,16 +6732,16 @@
         <v>261</v>
       </c>
       <c r="B259" s="24">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="C259" s="25">
-        <v>50.5</v>
+        <v>35.5</v>
       </c>
       <c r="D259" s="26">
         <v>3.9</v>
       </c>
       <c r="E259" s="27">
-        <v>196.95</v>
+        <v>138.44999999999999</v>
       </c>
     </row>
     <row r="260" spans="1:5" x14ac:dyDescent="0.25">
@@ -6817,16 +6805,16 @@
         <v>266</v>
       </c>
       <c r="B264" s="24">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="C264" s="25">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D264" s="26">
         <v>3.5</v>
       </c>
       <c r="E264" s="27">
-        <v>28</v>
+        <v>21</v>
       </c>
     </row>
     <row r="265" spans="1:5" x14ac:dyDescent="0.25">
@@ -6834,16 +6822,16 @@
         <v>267</v>
       </c>
       <c r="B265" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C265" s="25">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="D265" s="26">
         <v>4.25</v>
       </c>
       <c r="E265" s="27">
-        <v>42.5</v>
+        <v>21.25</v>
       </c>
     </row>
     <row r="266" spans="1:5" x14ac:dyDescent="0.25">
@@ -6957,16 +6945,16 @@
         <v>276</v>
       </c>
       <c r="B274" s="24">
-        <v>421</v>
+        <v>422</v>
       </c>
       <c r="C274" s="25">
-        <v>-5.5</v>
+        <v>-5</v>
       </c>
       <c r="D274" s="26">
         <v>4.28</v>
       </c>
       <c r="E274" s="27">
-        <v>-23.54</v>
+        <v>-21.4</v>
       </c>
     </row>
     <row r="275" spans="1:5" x14ac:dyDescent="0.25">
@@ -7019,11 +7007,17 @@
         <v>280</v>
       </c>
       <c r="B278" s="24">
-        <v>144</v>
-      </c>
-      <c r="C278" s="28"/>
-      <c r="D278" s="29"/>
-      <c r="E278" s="28"/>
+        <v>146</v>
+      </c>
+      <c r="C278" s="25">
+        <v>-5</v>
+      </c>
+      <c r="D278" s="26">
+        <v>3.1</v>
+      </c>
+      <c r="E278" s="27">
+        <v>-15.5</v>
+      </c>
     </row>
     <row r="279" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A279" s="23" t="s">
@@ -7058,16 +7052,16 @@
         <v>283</v>
       </c>
       <c r="B281" s="24">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C281" s="25">
-        <v>1</v>
+        <v>15</v>
       </c>
       <c r="D281" s="26">
         <v>6.25</v>
       </c>
       <c r="E281" s="27">
-        <v>6.25</v>
+        <v>93.75</v>
       </c>
     </row>
     <row r="282" spans="1:5" x14ac:dyDescent="0.25">
@@ -7075,16 +7069,16 @@
         <v>284</v>
       </c>
       <c r="B282" s="24">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C282" s="25">
-        <v>2.37</v>
+        <v>1.37</v>
       </c>
       <c r="D282" s="26">
         <v>4.25</v>
       </c>
       <c r="E282" s="27">
-        <v>10.07</v>
+        <v>5.82</v>
       </c>
     </row>
     <row r="283" spans="1:5" x14ac:dyDescent="0.25">
@@ -7159,17 +7153,11 @@
         <v>290</v>
       </c>
       <c r="B288" s="24">
-        <v>48</v>
-      </c>
-      <c r="C288" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="D288" s="26">
-        <v>6.5</v>
-      </c>
-      <c r="E288" s="27">
-        <v>3.25</v>
-      </c>
+        <v>49</v>
+      </c>
+      <c r="C288" s="28"/>
+      <c r="D288" s="29"/>
+      <c r="E288" s="28"/>
     </row>
     <row r="289" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A289" s="23" t="s">
@@ -7193,16 +7181,16 @@
         <v>292</v>
       </c>
       <c r="B290" s="24">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="C290" s="25">
-        <v>18.5</v>
+        <v>6.5</v>
       </c>
       <c r="D290" s="26">
         <v>4.8499999999999996</v>
       </c>
       <c r="E290" s="27">
-        <v>89.78</v>
+        <v>31.55</v>
       </c>
     </row>
     <row r="291" spans="1:5" x14ac:dyDescent="0.25">
@@ -7289,16 +7277,16 @@
         <v>298</v>
       </c>
       <c r="B296" s="24">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C296" s="25">
-        <v>2.5</v>
+        <v>0.5</v>
       </c>
       <c r="D296" s="26">
         <v>5</v>
       </c>
       <c r="E296" s="27">
-        <v>12.5</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="297" spans="1:5" x14ac:dyDescent="0.25">
@@ -7309,13 +7297,13 @@
         <v>27</v>
       </c>
       <c r="C297" s="25">
-        <v>3.5</v>
+        <v>103.5</v>
       </c>
       <c r="D297" s="26">
         <v>6</v>
       </c>
       <c r="E297" s="27">
-        <v>21</v>
+        <v>621</v>
       </c>
     </row>
     <row r="298" spans="1:5" x14ac:dyDescent="0.25">
@@ -7340,16 +7328,16 @@
         <v>301</v>
       </c>
       <c r="B299" s="24">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="C299" s="25">
-        <v>19.5</v>
+        <v>18.5</v>
       </c>
       <c r="D299" s="26">
         <v>4.66</v>
       </c>
       <c r="E299" s="27">
-        <v>90.8</v>
+        <v>86.14</v>
       </c>
     </row>
     <row r="300" spans="1:5" x14ac:dyDescent="0.25">
@@ -7391,17 +7379,11 @@
         <v>304</v>
       </c>
       <c r="B302" s="24">
-        <v>46</v>
-      </c>
-      <c r="C302" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="D302" s="26">
-        <v>3.8</v>
-      </c>
-      <c r="E302" s="27">
-        <v>1.9</v>
-      </c>
+        <v>47</v>
+      </c>
+      <c r="C302" s="28"/>
+      <c r="D302" s="29"/>
+      <c r="E302" s="28"/>
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A303" s="23" t="s">
@@ -7442,16 +7424,16 @@
         <v>307</v>
       </c>
       <c r="B305" s="24">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C305" s="25">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D305" s="26">
         <v>3.15</v>
       </c>
       <c r="E305" s="27">
-        <v>163.80000000000001</v>
+        <v>160.65</v>
       </c>
     </row>
     <row r="306" spans="1:5" x14ac:dyDescent="0.25">
@@ -7459,16 +7441,16 @@
         <v>308</v>
       </c>
       <c r="B306" s="24">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="C306" s="25">
-        <v>38</v>
+        <v>17</v>
       </c>
       <c r="D306" s="26">
-        <v>6.38</v>
+        <v>6.83</v>
       </c>
       <c r="E306" s="27">
-        <v>242.43</v>
+        <v>116.08</v>
       </c>
     </row>
     <row r="307" spans="1:5" x14ac:dyDescent="0.25">
@@ -7493,16 +7475,16 @@
         <v>310</v>
       </c>
       <c r="B308" s="24">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C308" s="25">
-        <v>170</v>
+        <v>162</v>
       </c>
       <c r="D308" s="26">
         <v>4.2699999999999996</v>
       </c>
       <c r="E308" s="27">
-        <v>725.72</v>
+        <v>691.57</v>
       </c>
     </row>
     <row r="309" spans="1:5" x14ac:dyDescent="0.25">
@@ -7538,16 +7520,16 @@
         <v>313</v>
       </c>
       <c r="B311" s="24">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C311" s="25">
-        <v>27</v>
+        <v>23.5</v>
       </c>
       <c r="D311" s="26">
         <v>4.5</v>
       </c>
       <c r="E311" s="27">
-        <v>121.5</v>
+        <v>105.75</v>
       </c>
     </row>
     <row r="312" spans="1:5" x14ac:dyDescent="0.25">
@@ -7555,16 +7537,16 @@
         <v>314</v>
       </c>
       <c r="B312" s="24">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="C312" s="25">
-        <v>240.25</v>
+        <v>236.25</v>
       </c>
       <c r="D312" s="26">
         <v>4.3</v>
       </c>
       <c r="E312" s="27">
-        <v>1032.7</v>
+        <v>1015.5</v>
       </c>
     </row>
     <row r="313" spans="1:5" x14ac:dyDescent="0.25">
@@ -7600,16 +7582,16 @@
         <v>317</v>
       </c>
       <c r="B315" s="24">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C315" s="25">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D315" s="26">
         <v>5.13</v>
       </c>
       <c r="E315" s="27">
-        <v>184.68</v>
+        <v>179.55</v>
       </c>
     </row>
     <row r="316" spans="1:5" x14ac:dyDescent="0.25">
@@ -7662,16 +7644,16 @@
         <v>321</v>
       </c>
       <c r="B319" s="24">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="C319" s="25">
-        <v>15.5</v>
+        <v>14.5</v>
       </c>
       <c r="D319" s="26">
         <v>11.5</v>
       </c>
       <c r="E319" s="27">
-        <v>178.25</v>
+        <v>166.75</v>
       </c>
     </row>
     <row r="320" spans="1:5" x14ac:dyDescent="0.25">
@@ -7731,13 +7713,13 @@
         <v>54</v>
       </c>
       <c r="C323" s="25">
-        <v>11.45</v>
+        <v>14.45</v>
       </c>
       <c r="D323" s="26">
         <v>9.4499999999999993</v>
       </c>
       <c r="E323" s="27">
-        <v>108.2</v>
+        <v>136.55000000000001</v>
       </c>
     </row>
     <row r="324" spans="1:5" x14ac:dyDescent="0.25">
@@ -7952,16 +7934,16 @@
         <v>341</v>
       </c>
       <c r="B339" s="24">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C339" s="25">
-        <v>31.41</v>
+        <v>25.41</v>
       </c>
       <c r="D339" s="26">
         <v>4.28</v>
       </c>
       <c r="E339" s="27">
-        <v>134.43</v>
+        <v>108.75</v>
       </c>
     </row>
     <row r="340" spans="1:5" x14ac:dyDescent="0.25">
@@ -7969,16 +7951,16 @@
         <v>342</v>
       </c>
       <c r="B340" s="24">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C340" s="25">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="D340" s="26">
         <v>4.28</v>
       </c>
       <c r="E340" s="27">
-        <v>273.92</v>
+        <v>252.52</v>
       </c>
     </row>
     <row r="341" spans="1:5" x14ac:dyDescent="0.25">
@@ -8042,16 +8024,16 @@
         <v>347</v>
       </c>
       <c r="B345" s="24">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="C345" s="25">
-        <v>6.5</v>
+        <v>5.5</v>
       </c>
       <c r="D345" s="26">
         <v>9</v>
       </c>
       <c r="E345" s="27">
-        <v>58.5</v>
+        <v>49.5</v>
       </c>
     </row>
     <row r="346" spans="1:5" x14ac:dyDescent="0.25">
@@ -8104,17 +8086,11 @@
         <v>351</v>
       </c>
       <c r="B349" s="24">
-        <v>45</v>
-      </c>
-      <c r="C349" s="25">
-        <v>1.5</v>
-      </c>
-      <c r="D349" s="26">
-        <v>9</v>
-      </c>
-      <c r="E349" s="27">
-        <v>13.5</v>
-      </c>
+        <v>46</v>
+      </c>
+      <c r="C349" s="28"/>
+      <c r="D349" s="29"/>
+      <c r="E349" s="28"/>
     </row>
     <row r="350" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A350" s="23" t="s">
@@ -8288,16 +8264,16 @@
         <v>363</v>
       </c>
       <c r="B361" s="24">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C361" s="25">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D361" s="26">
         <v>6.4</v>
       </c>
       <c r="E361" s="27">
-        <v>32</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="362" spans="1:5" x14ac:dyDescent="0.25">
@@ -8333,17 +8309,11 @@
         <v>366</v>
       </c>
       <c r="B364" s="24">
-        <v>32</v>
-      </c>
-      <c r="C364" s="25">
-        <v>4.5</v>
-      </c>
-      <c r="D364" s="26">
-        <v>9.1999999999999993</v>
-      </c>
-      <c r="E364" s="27">
-        <v>41.4</v>
-      </c>
+        <v>33</v>
+      </c>
+      <c r="C364" s="28"/>
+      <c r="D364" s="29"/>
+      <c r="E364" s="28"/>
     </row>
     <row r="365" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A365" s="23" t="s">
@@ -8382,16 +8352,16 @@
         <v>369</v>
       </c>
       <c r="B367" s="24">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C367" s="25">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="D367" s="26">
         <v>8</v>
       </c>
       <c r="E367" s="27">
-        <v>95.97</v>
+        <v>47.99</v>
       </c>
     </row>
     <row r="368" spans="1:5" x14ac:dyDescent="0.25">
@@ -8500,16 +8470,16 @@
         <v>377</v>
       </c>
       <c r="B375" s="24">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C375" s="25">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D375" s="26">
         <v>7.2</v>
       </c>
       <c r="E375" s="27">
-        <v>10.8</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="376" spans="1:5" x14ac:dyDescent="0.25">
@@ -8647,16 +8617,16 @@
         <v>386</v>
       </c>
       <c r="B384" s="24">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="C384" s="25">
-        <v>0.16</v>
+        <v>50.66</v>
       </c>
       <c r="D384" s="26">
         <v>4.5</v>
       </c>
       <c r="E384" s="27">
-        <v>0.72</v>
+        <v>227.97</v>
       </c>
     </row>
     <row r="385" spans="1:5" x14ac:dyDescent="0.25">
@@ -8664,16 +8634,16 @@
         <v>387</v>
       </c>
       <c r="B385" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C385" s="25">
-        <v>25.5</v>
+        <v>24.5</v>
       </c>
       <c r="D385" s="26">
         <v>8.08</v>
       </c>
       <c r="E385" s="27">
-        <v>206.04</v>
+        <v>197.96</v>
       </c>
     </row>
     <row r="386" spans="1:5" x14ac:dyDescent="0.25">
@@ -8698,16 +8668,16 @@
         <v>389</v>
       </c>
       <c r="B387" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C387" s="25">
-        <v>18</v>
+        <v>16.5</v>
       </c>
       <c r="D387" s="26">
         <v>8.25</v>
       </c>
       <c r="E387" s="27">
-        <v>148.5</v>
+        <v>136.13</v>
       </c>
     </row>
     <row r="388" spans="1:5" x14ac:dyDescent="0.25">
@@ -8754,16 +8724,16 @@
         <v>393</v>
       </c>
       <c r="B391" s="24">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C391" s="25">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="D391" s="26">
         <v>6</v>
       </c>
       <c r="E391" s="27">
-        <v>150</v>
+        <v>126</v>
       </c>
     </row>
     <row r="392" spans="1:5" x14ac:dyDescent="0.25">
@@ -8884,16 +8854,16 @@
         <v>401</v>
       </c>
       <c r="B399" s="24">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C399" s="25">
-        <v>4.5</v>
+        <v>1.5</v>
       </c>
       <c r="D399" s="26">
         <v>5.7</v>
       </c>
       <c r="E399" s="27">
-        <v>25.65</v>
+        <v>8.5500000000000007</v>
       </c>
     </row>
     <row r="400" spans="1:5" x14ac:dyDescent="0.25">
@@ -8901,16 +8871,16 @@
         <v>402</v>
       </c>
       <c r="B400" s="24">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C400" s="25">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="D400" s="26">
         <v>5.7</v>
       </c>
       <c r="E400" s="27">
-        <v>34.200000000000003</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="401" spans="1:5" x14ac:dyDescent="0.25">
@@ -8997,16 +8967,16 @@
         <v>408</v>
       </c>
       <c r="B406" s="24">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C406" s="25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D406" s="26">
         <v>8.5500000000000007</v>
       </c>
       <c r="E406" s="27">
-        <v>25.65</v>
+        <v>8.5500000000000007</v>
       </c>
     </row>
     <row r="407" spans="1:5" x14ac:dyDescent="0.25">
@@ -9042,16 +9012,16 @@
         <v>411</v>
       </c>
       <c r="B409" s="24">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C409" s="25">
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="D409" s="26">
         <v>6.18</v>
       </c>
       <c r="E409" s="27">
-        <v>6.18</v>
+        <v>-6.18</v>
       </c>
     </row>
     <row r="410" spans="1:5" x14ac:dyDescent="0.25">
@@ -9087,16 +9057,16 @@
         <v>414</v>
       </c>
       <c r="B412" s="24">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C412" s="25">
-        <v>2</v>
+        <v>-2</v>
       </c>
       <c r="D412" s="26">
         <v>6.65</v>
       </c>
       <c r="E412" s="27">
-        <v>13.3</v>
+        <v>-13.3</v>
       </c>
     </row>
     <row r="413" spans="1:5" x14ac:dyDescent="0.25">
@@ -9946,16 +9916,16 @@
         <v>473</v>
       </c>
       <c r="B471" s="24">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C471" s="25">
-        <v>11</v>
+        <v>9.5</v>
       </c>
       <c r="D471" s="26">
         <v>10.5</v>
       </c>
       <c r="E471" s="27">
-        <v>115.5</v>
+        <v>99.75</v>
       </c>
     </row>
     <row r="472" spans="1:5" x14ac:dyDescent="0.25">
@@ -9991,16 +9961,16 @@
         <v>476</v>
       </c>
       <c r="B474" s="24">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C474" s="25">
-        <v>4.4000000000000004</v>
+        <v>2.4</v>
       </c>
       <c r="D474" s="26">
         <v>8.5500000000000007</v>
       </c>
       <c r="E474" s="27">
-        <v>37.619999999999997</v>
+        <v>20.52</v>
       </c>
     </row>
     <row r="475" spans="1:5" x14ac:dyDescent="0.25">
@@ -10008,16 +9978,16 @@
         <v>477</v>
       </c>
       <c r="B475" s="24">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C475" s="25">
-        <v>15.16</v>
+        <v>7.16</v>
       </c>
       <c r="D475" s="26">
         <v>8.5500000000000007</v>
       </c>
       <c r="E475" s="27">
-        <v>129.62</v>
+        <v>61.22</v>
       </c>
     </row>
     <row r="476" spans="1:5" x14ac:dyDescent="0.25">
@@ -10128,16 +10098,16 @@
         <v>485</v>
       </c>
       <c r="B483" s="24">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C483" s="25">
-        <v>1</v>
+        <v>1.5</v>
       </c>
       <c r="D483" s="26">
         <v>10</v>
       </c>
       <c r="E483" s="27">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="484" spans="1:5" x14ac:dyDescent="0.25">
@@ -10148,13 +10118,13 @@
         <v>107</v>
       </c>
       <c r="C484" s="25">
-        <v>3.5</v>
+        <v>4</v>
       </c>
       <c r="D484" s="26">
         <v>9.5</v>
       </c>
       <c r="E484" s="27">
-        <v>33.25</v>
+        <v>38</v>
       </c>
     </row>
     <row r="485" spans="1:5" x14ac:dyDescent="0.25">
@@ -10460,16 +10430,16 @@
         <v>507</v>
       </c>
       <c r="B505" s="24">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="C505" s="25">
-        <v>13.38</v>
+        <v>9.8800000000000008</v>
       </c>
       <c r="D505" s="26">
         <v>11.26</v>
       </c>
       <c r="E505" s="27">
-        <v>150.69999999999999</v>
+        <v>111.28</v>
       </c>
     </row>
     <row r="506" spans="1:5" x14ac:dyDescent="0.25">
@@ -10779,16 +10749,16 @@
         <v>528</v>
       </c>
       <c r="B526" s="24">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C526" s="25">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D526" s="26">
         <v>2.6</v>
       </c>
       <c r="E526" s="27">
-        <v>52</v>
+        <v>46.8</v>
       </c>
     </row>
     <row r="527" spans="1:5" x14ac:dyDescent="0.25">
@@ -10943,16 +10913,16 @@
         <v>538</v>
       </c>
       <c r="B536" s="24">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C536" s="25">
-        <v>1.5</v>
+        <v>0.5</v>
       </c>
       <c r="D536" s="26">
         <v>1.4</v>
       </c>
       <c r="E536" s="27">
-        <v>2.1</v>
+        <v>0.7</v>
       </c>
     </row>
     <row r="537" spans="1:5" x14ac:dyDescent="0.25">
@@ -10960,16 +10930,16 @@
         <v>539</v>
       </c>
       <c r="B537" s="24">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="C537" s="25">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D537" s="26">
         <v>1.4</v>
       </c>
       <c r="E537" s="27">
-        <v>18.2</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="538" spans="1:5" x14ac:dyDescent="0.25">
@@ -11260,16 +11230,16 @@
         <v>557</v>
       </c>
       <c r="B555" s="24">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C555" s="25">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
       <c r="D555" s="26">
         <v>4.5</v>
       </c>
       <c r="E555" s="27">
-        <v>6.3</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="556" spans="1:5" x14ac:dyDescent="0.25">
@@ -11362,16 +11332,16 @@
         <v>563</v>
       </c>
       <c r="B561" s="24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C561" s="25">
-        <v>72.5</v>
+        <v>70.5</v>
       </c>
       <c r="D561" s="26">
         <v>3.45</v>
       </c>
       <c r="E561" s="27">
-        <v>250.13</v>
+        <v>243.23</v>
       </c>
     </row>
     <row r="562" spans="1:5" x14ac:dyDescent="0.25">
@@ -11398,15 +11368,9 @@
       <c r="B563" s="24">
         <v>49</v>
       </c>
-      <c r="C563" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="D563" s="26">
-        <v>9.5</v>
-      </c>
-      <c r="E563" s="27">
-        <v>4.75</v>
-      </c>
+      <c r="C563" s="28"/>
+      <c r="D563" s="29"/>
+      <c r="E563" s="28"/>
     </row>
     <row r="564" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A564" s="23" t="s">
@@ -11447,16 +11411,16 @@
         <v>568</v>
       </c>
       <c r="B566" s="24">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="C566" s="25">
-        <v>0.71</v>
+        <v>82.71</v>
       </c>
       <c r="D566" s="26">
         <v>3.9</v>
       </c>
       <c r="E566" s="27">
-        <v>2.77</v>
+        <v>322.57</v>
       </c>
     </row>
     <row r="567" spans="1:5" x14ac:dyDescent="0.25">
@@ -11651,16 +11615,16 @@
         <v>580</v>
       </c>
       <c r="B578" s="24">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="C578" s="25">
-        <v>10.5</v>
+        <v>4.5</v>
       </c>
       <c r="D578" s="26">
         <v>5.7</v>
       </c>
       <c r="E578" s="27">
-        <v>59.85</v>
+        <v>25.65</v>
       </c>
     </row>
     <row r="579" spans="1:5" x14ac:dyDescent="0.25">
@@ -11764,17 +11728,11 @@
         <v>587</v>
       </c>
       <c r="B585" s="24">
-        <v>31</v>
-      </c>
-      <c r="C585" s="25">
-        <v>1</v>
-      </c>
-      <c r="D585" s="26">
-        <v>2.74</v>
-      </c>
-      <c r="E585" s="27">
-        <v>2.74</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="C585" s="28"/>
+      <c r="D585" s="29"/>
+      <c r="E585" s="28"/>
     </row>
     <row r="586" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A586" s="23" t="s">
@@ -11832,16 +11790,16 @@
         <v>591</v>
       </c>
       <c r="B589" s="24">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C589" s="25">
-        <v>107.5</v>
+        <v>104.5</v>
       </c>
       <c r="D589" s="26">
         <v>1.8</v>
       </c>
       <c r="E589" s="27">
-        <v>193.5</v>
+        <v>188.1</v>
       </c>
     </row>
     <row r="590" spans="1:5" x14ac:dyDescent="0.25">
@@ -11866,16 +11824,16 @@
         <v>593</v>
       </c>
       <c r="B591" s="24">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C591" s="25">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="D591" s="26">
         <v>1.2</v>
       </c>
       <c r="E591" s="27">
-        <v>177.6</v>
+        <v>172.8</v>
       </c>
     </row>
     <row r="592" spans="1:5" x14ac:dyDescent="0.25">
@@ -11883,16 +11841,16 @@
         <v>594</v>
       </c>
       <c r="B592" s="24">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C592" s="25">
-        <v>228</v>
+        <v>222</v>
       </c>
       <c r="D592" s="26">
         <v>1.2</v>
       </c>
       <c r="E592" s="27">
-        <v>273.60000000000002</v>
+        <v>266.39999999999998</v>
       </c>
     </row>
     <row r="593" spans="1:5" x14ac:dyDescent="0.25">
@@ -11900,16 +11858,16 @@
         <v>595</v>
       </c>
       <c r="B593" s="24">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C593" s="25">
-        <v>186</v>
+        <v>180</v>
       </c>
       <c r="D593" s="26">
         <v>1.2</v>
       </c>
       <c r="E593" s="27">
-        <v>223.2</v>
+        <v>216</v>
       </c>
     </row>
     <row r="594" spans="1:5" x14ac:dyDescent="0.25">
@@ -11917,10 +11875,10 @@
         <v>596</v>
       </c>
       <c r="B594" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C594" s="25">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="D594" s="29"/>
       <c r="E594" s="28"/>
@@ -11982,16 +11940,16 @@
         <v>601</v>
       </c>
       <c r="B599" s="24">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C599" s="25">
-        <v>239.5</v>
+        <v>236</v>
       </c>
       <c r="D599" s="26">
         <v>1.5</v>
       </c>
       <c r="E599" s="27">
-        <v>359.25</v>
+        <v>354</v>
       </c>
     </row>
     <row r="600" spans="1:5" x14ac:dyDescent="0.25">
@@ -11999,10 +11957,10 @@
         <v>602</v>
       </c>
       <c r="B600" s="24">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="C600" s="25">
-        <v>-259.5</v>
+        <v>-280.5</v>
       </c>
       <c r="D600" s="29"/>
       <c r="E600" s="28"/>
@@ -12012,10 +11970,10 @@
         <v>603</v>
       </c>
       <c r="B601" s="24">
-        <v>167</v>
+        <v>171</v>
       </c>
       <c r="C601" s="25">
-        <v>-105.5</v>
+        <v>-115.5</v>
       </c>
       <c r="D601" s="29"/>
       <c r="E601" s="28"/>
@@ -12038,10 +11996,10 @@
         <v>605</v>
       </c>
       <c r="B603" s="24">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C603" s="25">
-        <v>-45</v>
+        <v>-53</v>
       </c>
       <c r="D603" s="29"/>
       <c r="E603" s="28"/>
@@ -12064,16 +12022,16 @@
         <v>607</v>
       </c>
       <c r="B605" s="24">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="C605" s="25">
-        <v>75.5</v>
+        <v>68.5</v>
       </c>
       <c r="D605" s="26">
         <v>0.87</v>
       </c>
       <c r="E605" s="27">
-        <v>65.69</v>
+        <v>59.6</v>
       </c>
     </row>
     <row r="606" spans="1:5" x14ac:dyDescent="0.25">
@@ -12081,16 +12039,16 @@
         <v>608</v>
       </c>
       <c r="B606" s="24">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="C606" s="25">
-        <v>334.5</v>
+        <v>170.5</v>
       </c>
       <c r="D606" s="26">
         <v>0.57999999999999996</v>
       </c>
       <c r="E606" s="27">
-        <v>194.01</v>
+        <v>98.89</v>
       </c>
     </row>
     <row r="607" spans="1:5" x14ac:dyDescent="0.25">
@@ -12098,16 +12056,16 @@
         <v>609</v>
       </c>
       <c r="B607" s="24">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="C607" s="25">
-        <v>892</v>
+        <v>872</v>
       </c>
       <c r="D607" s="26">
         <v>0.85</v>
       </c>
       <c r="E607" s="27">
-        <v>758.2</v>
+        <v>741.2</v>
       </c>
     </row>
     <row r="608" spans="1:5" x14ac:dyDescent="0.25">
@@ -12199,10 +12157,10 @@
         <v>616</v>
       </c>
       <c r="B614" s="24">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C614" s="25">
-        <v>-160</v>
+        <v>-100</v>
       </c>
       <c r="D614" s="29"/>
       <c r="E614" s="28"/>
@@ -12215,7 +12173,7 @@
         <v>41</v>
       </c>
       <c r="C615" s="25">
-        <v>-105</v>
+        <v>-49</v>
       </c>
       <c r="D615" s="29"/>
       <c r="E615" s="28"/>
@@ -12228,7 +12186,7 @@
         <v>41</v>
       </c>
       <c r="C616" s="25">
-        <v>-146</v>
+        <v>-82</v>
       </c>
       <c r="D616" s="29"/>
       <c r="E616" s="28"/>
@@ -12618,16 +12576,16 @@
         <v>643</v>
       </c>
       <c r="B641" s="24">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C641" s="25">
-        <v>-2.65</v>
+        <v>-3.65</v>
       </c>
       <c r="D641" s="26">
         <v>4</v>
       </c>
       <c r="E641" s="27">
-        <v>-10.6</v>
+        <v>-14.6</v>
       </c>
     </row>
     <row r="642" spans="1:5" x14ac:dyDescent="0.25">
@@ -12714,16 +12672,16 @@
         <v>649</v>
       </c>
       <c r="B647" s="24">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C647" s="25">
-        <v>4.5</v>
+        <v>3</v>
       </c>
       <c r="D647" s="26">
         <v>2.76</v>
       </c>
       <c r="E647" s="27">
-        <v>12.41</v>
+        <v>8.27</v>
       </c>
     </row>
     <row r="648" spans="1:5" x14ac:dyDescent="0.25">
@@ -12731,16 +12689,16 @@
         <v>650</v>
       </c>
       <c r="B648" s="24">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C648" s="25">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D648" s="26">
         <v>4</v>
       </c>
       <c r="E648" s="27">
-        <v>12</v>
+        <v>4</v>
       </c>
     </row>
     <row r="649" spans="1:5" x14ac:dyDescent="0.25">
@@ -12759,16 +12717,16 @@
         <v>652</v>
       </c>
       <c r="B650" s="24">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C650" s="25">
-        <v>0.5</v>
+        <v>-7.5</v>
       </c>
       <c r="D650" s="26">
         <v>1.5</v>
       </c>
       <c r="E650" s="27">
-        <v>0.75</v>
+        <v>-11.25</v>
       </c>
     </row>
     <row r="651" spans="1:5" x14ac:dyDescent="0.25">
@@ -12810,16 +12768,16 @@
         <v>655</v>
       </c>
       <c r="B653" s="24">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="C653" s="25">
-        <v>43.5</v>
+        <v>40</v>
       </c>
       <c r="D653" s="26">
         <v>2.2799999999999998</v>
       </c>
       <c r="E653" s="27">
-        <v>99.18</v>
+        <v>91.2</v>
       </c>
     </row>
     <row r="654" spans="1:5" x14ac:dyDescent="0.25">
@@ -13002,16 +12960,16 @@
         <v>667</v>
       </c>
       <c r="B665" s="24">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="C665" s="25">
-        <v>137.36000000000001</v>
+        <v>129.36000000000001</v>
       </c>
       <c r="D665" s="26">
         <v>1.7</v>
       </c>
       <c r="E665" s="27">
-        <v>233.51</v>
+        <v>219.91</v>
       </c>
     </row>
     <row r="666" spans="1:5" x14ac:dyDescent="0.25">
@@ -13053,16 +13011,16 @@
         <v>670</v>
       </c>
       <c r="B668" s="24">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C668" s="25">
-        <v>8.5</v>
+        <v>7.5</v>
       </c>
       <c r="D668" s="26">
         <v>3.5</v>
       </c>
       <c r="E668" s="27">
-        <v>29.75</v>
+        <v>26.25</v>
       </c>
     </row>
     <row r="669" spans="1:5" x14ac:dyDescent="0.25">
@@ -13121,16 +13079,16 @@
         <v>674</v>
       </c>
       <c r="B672" s="24">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="C672" s="25">
-        <v>23</v>
+        <v>16.5</v>
       </c>
       <c r="D672" s="26">
         <v>2.85</v>
       </c>
       <c r="E672" s="27">
-        <v>65.55</v>
+        <v>47.03</v>
       </c>
     </row>
     <row r="673" spans="1:5" x14ac:dyDescent="0.25">
@@ -13188,16 +13146,16 @@
         <v>679</v>
       </c>
       <c r="B677" s="24">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="C677" s="25">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="D677" s="26">
         <v>3.1</v>
       </c>
       <c r="E677" s="27">
-        <v>62</v>
+        <v>74.400000000000006</v>
       </c>
     </row>
     <row r="678" spans="1:5" x14ac:dyDescent="0.25">
@@ -13239,16 +13197,16 @@
         <v>682</v>
       </c>
       <c r="B680" s="24">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C680" s="25">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="D680" s="26">
         <v>4.8</v>
       </c>
       <c r="E680" s="27">
-        <v>36</v>
+        <v>31.2</v>
       </c>
     </row>
     <row r="681" spans="1:5" x14ac:dyDescent="0.25">
@@ -13340,16 +13298,16 @@
         <v>689</v>
       </c>
       <c r="B687" s="24">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="C687" s="25">
-        <v>119.5</v>
+        <v>118.5</v>
       </c>
       <c r="D687" s="26">
         <v>3.1</v>
       </c>
       <c r="E687" s="27">
-        <v>370.45</v>
+        <v>367.35</v>
       </c>
     </row>
     <row r="688" spans="1:5" x14ac:dyDescent="0.25">
@@ -13376,9 +13334,15 @@
       <c r="B689" s="24">
         <v>66</v>
       </c>
-      <c r="C689" s="28"/>
-      <c r="D689" s="29"/>
-      <c r="E689" s="28"/>
+      <c r="C689" s="25">
+        <v>20</v>
+      </c>
+      <c r="D689" s="26">
+        <v>3.5</v>
+      </c>
+      <c r="E689" s="27">
+        <v>70</v>
+      </c>
     </row>
     <row r="690" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A690" s="23" t="s">
@@ -13405,13 +13369,13 @@
         <v>86</v>
       </c>
       <c r="C691" s="25">
-        <v>-10</v>
+        <v>10</v>
       </c>
       <c r="D691" s="26">
         <v>3.75</v>
       </c>
       <c r="E691" s="27">
-        <v>-37.5</v>
+        <v>37.5</v>
       </c>
     </row>
     <row r="692" spans="1:5" x14ac:dyDescent="0.25">
@@ -13498,16 +13462,16 @@
         <v>699</v>
       </c>
       <c r="B697" s="24">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C697" s="25">
-        <v>19</v>
+        <v>15</v>
       </c>
       <c r="D697" s="26">
         <v>2.25</v>
       </c>
       <c r="E697" s="27">
-        <v>42.75</v>
+        <v>33.75</v>
       </c>
     </row>
     <row r="698" spans="1:5" x14ac:dyDescent="0.25">
@@ -13785,10 +13749,10 @@
         <v>718</v>
       </c>
       <c r="B716" s="24">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C716" s="25">
-        <v>-93</v>
+        <v>-94</v>
       </c>
       <c r="D716" s="29"/>
       <c r="E716" s="28"/>
@@ -13798,10 +13762,10 @@
         <v>719</v>
       </c>
       <c r="B717" s="24">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C717" s="25">
-        <v>-52.5</v>
+        <v>-54</v>
       </c>
       <c r="D717" s="29"/>
       <c r="E717" s="28"/>
@@ -13811,10 +13775,10 @@
         <v>720</v>
       </c>
       <c r="B718" s="24">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C718" s="25">
-        <v>1.5</v>
+        <v>-2.5</v>
       </c>
       <c r="D718" s="29"/>
       <c r="E718" s="28"/>
@@ -14196,16 +14160,16 @@
         <v>749</v>
       </c>
       <c r="B747" s="24">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="C747" s="25">
-        <v>21.75</v>
+        <v>15.75</v>
       </c>
       <c r="D747" s="26">
         <v>2.5</v>
       </c>
       <c r="E747" s="27">
-        <v>54.38</v>
+        <v>39.380000000000003</v>
       </c>
     </row>
     <row r="748" spans="1:5" x14ac:dyDescent="0.25">
@@ -14281,10 +14245,10 @@
         <v>754</v>
       </c>
       <c r="B752" s="24">
-        <v>317</v>
+        <v>322</v>
       </c>
       <c r="C752" s="25">
-        <v>-938.7</v>
+        <v>-950.7</v>
       </c>
       <c r="D752" s="29"/>
       <c r="E752" s="28"/>
@@ -14295,11 +14259,11 @@
       </c>
       <c r="B753" s="31"/>
       <c r="C753" s="32">
-        <v>23733.33</v>
+        <v>23047.08</v>
       </c>
       <c r="D753" s="33"/>
       <c r="E753" s="34">
-        <v>52725.43</v>
+        <v>51977.919999999998</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nikhil @830 on 5may pm
</commit_message>
<xml_diff>
--- a/data/website stock.xlsx
+++ b/data/website stock.xlsx
@@ -3436,16 +3436,16 @@
         <v>45</v>
       </c>
       <c r="B43" s="24">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="C43" s="25">
-        <v>30.5</v>
+        <v>33</v>
       </c>
       <c r="D43" s="26">
         <v>2.4700000000000002</v>
       </c>
       <c r="E43" s="27">
-        <v>75.38</v>
+        <v>81.56</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.25">
@@ -3453,16 +3453,16 @@
         <v>46</v>
       </c>
       <c r="B44" s="24">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C44" s="25">
-        <v>6.32</v>
+        <v>8.82</v>
       </c>
       <c r="D44" s="26">
         <v>2.71</v>
       </c>
       <c r="E44" s="27">
-        <v>17.12</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.25">
@@ -3500,9 +3500,15 @@
       <c r="B47" s="24">
         <v>120</v>
       </c>
-      <c r="C47" s="28"/>
-      <c r="D47" s="29"/>
-      <c r="E47" s="28"/>
+      <c r="C47" s="25">
+        <v>1</v>
+      </c>
+      <c r="D47" s="26">
+        <v>1.27</v>
+      </c>
+      <c r="E47" s="27">
+        <v>1.27</v>
+      </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A48" s="23" t="s">
@@ -3522,16 +3528,16 @@
         <v>51</v>
       </c>
       <c r="B49" s="24">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C49" s="25">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D49" s="26">
         <v>1.4</v>
       </c>
       <c r="E49" s="27">
-        <v>74.2</v>
+        <v>63</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.25">
@@ -3590,16 +3596,16 @@
         <v>55</v>
       </c>
       <c r="B53" s="24">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C53" s="25">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="D53" s="26">
         <v>2.5</v>
       </c>
       <c r="E53" s="27">
-        <v>452.5</v>
+        <v>442.5</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.25">
@@ -3641,16 +3647,16 @@
         <v>58</v>
       </c>
       <c r="B56" s="24">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C56" s="25">
-        <v>127</v>
+        <v>123</v>
       </c>
       <c r="D56" s="26">
         <v>1.8</v>
       </c>
       <c r="E56" s="27">
-        <v>228.6</v>
+        <v>221.4</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.25">
@@ -3714,16 +3720,16 @@
         <v>63</v>
       </c>
       <c r="B61" s="24">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="C61" s="25">
-        <v>379</v>
+        <v>377</v>
       </c>
       <c r="D61" s="26">
         <v>1.1399999999999999</v>
       </c>
       <c r="E61" s="27">
-        <v>431.81</v>
+        <v>429.53</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.25">
@@ -3818,13 +3824,13 @@
         <v>195</v>
       </c>
       <c r="C68" s="25">
-        <v>-11</v>
+        <v>-10</v>
       </c>
       <c r="D68" s="26">
         <v>1.65</v>
       </c>
       <c r="E68" s="27">
-        <v>-18.149999999999999</v>
+        <v>-16.5</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
@@ -3860,16 +3866,16 @@
         <v>73</v>
       </c>
       <c r="B71" s="24">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C71" s="25">
-        <v>120.5</v>
+        <v>107</v>
       </c>
       <c r="D71" s="26">
         <v>1.4</v>
       </c>
       <c r="E71" s="27">
-        <v>168.7</v>
+        <v>149.80000000000001</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
@@ -3914,13 +3920,13 @@
         <v>202</v>
       </c>
       <c r="C74" s="25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D74" s="26">
         <v>1.2</v>
       </c>
       <c r="E74" s="27">
-        <v>1.2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.25">
@@ -4024,16 +4030,16 @@
         <v>83</v>
       </c>
       <c r="B81" s="24">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="C81" s="25">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="D81" s="26">
         <v>1.2</v>
       </c>
       <c r="E81" s="27">
-        <v>13.2</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.25">
@@ -4058,11 +4064,17 @@
         <v>85</v>
       </c>
       <c r="B83" s="24">
-        <v>110</v>
-      </c>
-      <c r="C83" s="28"/>
-      <c r="D83" s="29"/>
-      <c r="E83" s="28"/>
+        <v>111</v>
+      </c>
+      <c r="C83" s="25">
+        <v>-10</v>
+      </c>
+      <c r="D83" s="26">
+        <v>1.2</v>
+      </c>
+      <c r="E83" s="27">
+        <v>-12</v>
+      </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="23" t="s">
@@ -4114,16 +4126,16 @@
         <v>89</v>
       </c>
       <c r="B87" s="24">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="C87" s="25">
-        <v>216.5</v>
+        <v>208.5</v>
       </c>
       <c r="D87" s="26">
         <v>1.7</v>
       </c>
       <c r="E87" s="27">
-        <v>368.05</v>
+        <v>354.45</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.25">
@@ -4199,16 +4211,16 @@
         <v>94</v>
       </c>
       <c r="B92" s="24">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C92" s="25">
-        <v>670</v>
+        <v>654</v>
       </c>
       <c r="D92" s="26">
         <v>1.83</v>
       </c>
       <c r="E92" s="27">
-        <v>1225.07</v>
+        <v>1195.82</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.25">
@@ -4280,16 +4292,16 @@
         <v>99</v>
       </c>
       <c r="B97" s="24">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C97" s="25">
-        <v>21.5</v>
+        <v>18.5</v>
       </c>
       <c r="D97" s="26">
         <v>0.9</v>
       </c>
       <c r="E97" s="27">
-        <v>19.350000000000001</v>
+        <v>16.649999999999999</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.25">
@@ -4330,15 +4342,17 @@
       <c r="A100" s="23" t="s">
         <v>102</v>
       </c>
-      <c r="B100" s="24"/>
+      <c r="B100" s="24">
+        <v>1</v>
+      </c>
       <c r="C100" s="25">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D100" s="26">
         <v>0.85</v>
       </c>
       <c r="E100" s="27">
-        <v>7.65</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.25">
@@ -4406,16 +4420,16 @@
         <v>107</v>
       </c>
       <c r="B105" s="24">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C105" s="25">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D105" s="26">
         <v>2.5</v>
       </c>
       <c r="E105" s="27">
-        <v>90</v>
+        <v>87.5</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.25">
@@ -4556,10 +4570,10 @@
         <v>119</v>
       </c>
       <c r="B117" s="24">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C117" s="25">
-        <v>55</v>
+        <v>35</v>
       </c>
       <c r="D117" s="29"/>
       <c r="E117" s="28"/>
@@ -4636,16 +4650,16 @@
         <v>125</v>
       </c>
       <c r="B123" s="24">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C123" s="25">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="D123" s="26">
         <v>0.87</v>
       </c>
       <c r="E123" s="27">
-        <v>29.58</v>
+        <v>20.88</v>
       </c>
     </row>
     <row r="124" spans="1:5" x14ac:dyDescent="0.25">
@@ -4855,16 +4869,16 @@
         <v>142</v>
       </c>
       <c r="B140" s="24">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C140" s="25">
-        <v>10</v>
+        <v>8.5</v>
       </c>
       <c r="D140" s="26">
         <v>12.5</v>
       </c>
       <c r="E140" s="27">
-        <v>125</v>
+        <v>106.25</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.25">
@@ -4909,13 +4923,13 @@
         <v>12</v>
       </c>
       <c r="C143" s="25">
-        <v>10</v>
+        <v>10.5</v>
       </c>
       <c r="D143" s="26">
         <v>12.5</v>
       </c>
       <c r="E143" s="27">
-        <v>125</v>
+        <v>131.25</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.25">
@@ -5015,9 +5029,15 @@
       <c r="B150" s="24">
         <v>50</v>
       </c>
-      <c r="C150" s="28"/>
-      <c r="D150" s="29"/>
-      <c r="E150" s="28"/>
+      <c r="C150" s="25">
+        <v>0.5</v>
+      </c>
+      <c r="D150" s="26">
+        <v>18.5</v>
+      </c>
+      <c r="E150" s="27">
+        <v>9.25</v>
+      </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A151" s="23" t="s">
@@ -5075,16 +5095,16 @@
         <v>156</v>
       </c>
       <c r="B154" s="24">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C154" s="25">
-        <v>1.27</v>
+        <v>0.27</v>
       </c>
       <c r="D154" s="26">
-        <v>18.5</v>
+        <v>18.52</v>
       </c>
       <c r="E154" s="27">
-        <v>23.5</v>
+        <v>5</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.25">
@@ -5217,9 +5237,15 @@
       <c r="B164" s="24">
         <v>37</v>
       </c>
-      <c r="C164" s="28"/>
-      <c r="D164" s="29"/>
-      <c r="E164" s="28"/>
+      <c r="C164" s="25">
+        <v>0.5</v>
+      </c>
+      <c r="D164" s="26">
+        <v>11.5</v>
+      </c>
+      <c r="E164" s="27">
+        <v>5.75</v>
+      </c>
     </row>
     <row r="165" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A165" s="23" t="s">
@@ -5243,16 +5269,16 @@
         <v>168</v>
       </c>
       <c r="B166" s="24">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C166" s="25">
-        <v>0.5</v>
+        <v>2</v>
       </c>
       <c r="D166" s="26">
         <v>11.5</v>
       </c>
       <c r="E166" s="27">
-        <v>5.75</v>
+        <v>23</v>
       </c>
     </row>
     <row r="167" spans="1:5" x14ac:dyDescent="0.25">
@@ -5405,16 +5431,16 @@
         <v>180</v>
       </c>
       <c r="B178" s="24">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="C178" s="25">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="D178" s="26">
         <v>0.97</v>
       </c>
       <c r="E178" s="27">
-        <v>36.99</v>
+        <v>27.25</v>
       </c>
     </row>
     <row r="179" spans="1:5" x14ac:dyDescent="0.25">
@@ -6016,16 +6042,16 @@
         <v>223</v>
       </c>
       <c r="B221" s="24">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C221" s="25">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="D221" s="26">
         <v>3.95</v>
       </c>
       <c r="E221" s="27">
-        <v>-3.95</v>
+        <v>15.8</v>
       </c>
     </row>
     <row r="222" spans="1:5" x14ac:dyDescent="0.25">
@@ -6123,16 +6149,16 @@
         <v>230</v>
       </c>
       <c r="B228" s="24">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C228" s="25">
-        <v>5.5</v>
+        <v>3</v>
       </c>
       <c r="D228" s="26">
         <v>3</v>
       </c>
       <c r="E228" s="27">
-        <v>16.5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="229" spans="1:5" x14ac:dyDescent="0.25">
@@ -6766,16 +6792,16 @@
         <v>277</v>
       </c>
       <c r="B275" s="24">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C275" s="25">
-        <v>46.5</v>
+        <v>45.5</v>
       </c>
       <c r="D275" s="26">
         <v>6.18</v>
       </c>
       <c r="E275" s="27">
-        <v>287.56</v>
+        <v>281.37</v>
       </c>
     </row>
     <row r="276" spans="1:5" x14ac:dyDescent="0.25">
@@ -7029,16 +7055,16 @@
         <v>296</v>
       </c>
       <c r="B294" s="24">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C294" s="25">
-        <v>15.58</v>
+        <v>11.58</v>
       </c>
       <c r="D294" s="26">
         <v>4.76</v>
       </c>
       <c r="E294" s="27">
-        <v>74.11</v>
+        <v>55.08</v>
       </c>
     </row>
     <row r="295" spans="1:5" x14ac:dyDescent="0.25">
@@ -7238,16 +7264,16 @@
         <v>309</v>
       </c>
       <c r="B307" s="24">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C307" s="25">
-        <v>4.78</v>
+        <v>6.78</v>
       </c>
       <c r="D307" s="26">
         <v>3.15</v>
       </c>
       <c r="E307" s="27">
-        <v>15.06</v>
+        <v>21.36</v>
       </c>
     </row>
     <row r="308" spans="1:5" x14ac:dyDescent="0.25">
@@ -7743,16 +7769,16 @@
         <v>344</v>
       </c>
       <c r="B342" s="24">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C342" s="25">
-        <v>40.5</v>
+        <v>39.5</v>
       </c>
       <c r="D342" s="26">
         <v>4.28</v>
       </c>
       <c r="E342" s="27">
-        <v>173.34</v>
+        <v>169.06</v>
       </c>
     </row>
     <row r="343" spans="1:5" x14ac:dyDescent="0.25">
@@ -8434,13 +8460,13 @@
         <v>72</v>
       </c>
       <c r="C392" s="25">
-        <v>4.5</v>
+        <v>5.5</v>
       </c>
       <c r="D392" s="26">
         <v>3.6</v>
       </c>
       <c r="E392" s="27">
-        <v>16.2</v>
+        <v>19.8</v>
       </c>
     </row>
     <row r="393" spans="1:5" x14ac:dyDescent="0.25">
@@ -8622,16 +8648,16 @@
         <v>407</v>
       </c>
       <c r="B405" s="24">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C405" s="25">
-        <v>0.5</v>
+        <v>1.5</v>
       </c>
       <c r="D405" s="26">
         <v>8.6999999999999993</v>
       </c>
       <c r="E405" s="27">
-        <v>4.3499999999999996</v>
+        <v>13.05</v>
       </c>
     </row>
     <row r="406" spans="1:5" x14ac:dyDescent="0.25">
@@ -9736,16 +9762,16 @@
         <v>485</v>
       </c>
       <c r="B483" s="24">
+        <v>6</v>
+      </c>
+      <c r="C483" s="25">
         <v>7</v>
-      </c>
-      <c r="C483" s="25">
-        <v>3.5</v>
       </c>
       <c r="D483" s="26">
         <v>11.2</v>
       </c>
       <c r="E483" s="27">
-        <v>39.200000000000003</v>
+        <v>78.400000000000006</v>
       </c>
     </row>
     <row r="484" spans="1:5" x14ac:dyDescent="0.25">
@@ -10610,16 +10636,16 @@
         <v>543</v>
       </c>
       <c r="B541" s="24">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C541" s="25">
-        <v>5.5</v>
+        <v>9.5</v>
       </c>
       <c r="D541" s="26">
         <v>1.95</v>
       </c>
       <c r="E541" s="27">
-        <v>10.73</v>
+        <v>18.53</v>
       </c>
     </row>
     <row r="542" spans="1:5" x14ac:dyDescent="0.25">
@@ -10661,16 +10687,16 @@
         <v>546</v>
       </c>
       <c r="B544" s="24">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C544" s="25">
-        <v>22.5</v>
+        <v>21.5</v>
       </c>
       <c r="D544" s="26">
         <v>3</v>
       </c>
       <c r="E544" s="27">
-        <v>67.5</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="545" spans="1:5" x14ac:dyDescent="0.25">
@@ -10678,16 +10704,16 @@
         <v>547</v>
       </c>
       <c r="B545" s="24">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C545" s="25">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="D545" s="26">
         <v>3.8</v>
       </c>
       <c r="E545" s="27">
-        <v>19</v>
+        <v>11.4</v>
       </c>
     </row>
     <row r="546" spans="1:5" x14ac:dyDescent="0.25">
@@ -10831,16 +10857,16 @@
         <v>556</v>
       </c>
       <c r="B554" s="24">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C554" s="25">
-        <v>7</v>
+        <v>10.5</v>
       </c>
       <c r="D554" s="26">
         <v>4.28</v>
       </c>
       <c r="E554" s="27">
-        <v>29.96</v>
+        <v>44.94</v>
       </c>
     </row>
     <row r="555" spans="1:5" x14ac:dyDescent="0.25">
@@ -11057,16 +11083,16 @@
         <v>570</v>
       </c>
       <c r="B568" s="24">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C568" s="25">
-        <v>7.06</v>
+        <v>10.06</v>
       </c>
       <c r="D568" s="26">
         <v>3.9</v>
       </c>
       <c r="E568" s="27">
-        <v>27.53</v>
+        <v>39.229999999999997</v>
       </c>
     </row>
     <row r="569" spans="1:5" x14ac:dyDescent="0.25">
@@ -11257,13 +11283,13 @@
         <v>11</v>
       </c>
       <c r="C581" s="25">
-        <v>2.5</v>
+        <v>2.44</v>
       </c>
       <c r="D581" s="26">
         <v>3.6</v>
       </c>
       <c r="E581" s="27">
-        <v>9</v>
+        <v>8.7799999999999994</v>
       </c>
     </row>
     <row r="582" spans="1:5" x14ac:dyDescent="0.25">
@@ -11282,16 +11308,16 @@
         <v>585</v>
       </c>
       <c r="B583" s="24">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C583" s="25">
-        <v>5.5</v>
+        <v>4.5</v>
       </c>
       <c r="D583" s="26">
         <v>2.66</v>
       </c>
       <c r="E583" s="27">
-        <v>14.63</v>
+        <v>11.97</v>
       </c>
     </row>
     <row r="584" spans="1:5" x14ac:dyDescent="0.25">
@@ -11670,16 +11696,16 @@
         <v>611</v>
       </c>
       <c r="B609" s="24">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="C609" s="25">
-        <v>627.5</v>
+        <v>624.5</v>
       </c>
       <c r="D609" s="26">
         <v>0.85</v>
       </c>
       <c r="E609" s="27">
-        <v>533.38</v>
+        <v>530.83000000000004</v>
       </c>
     </row>
     <row r="610" spans="1:5" x14ac:dyDescent="0.25">
@@ -12752,16 +12778,16 @@
         <v>681</v>
       </c>
       <c r="B679" s="24">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C679" s="25">
-        <v>15.5</v>
+        <v>14.5</v>
       </c>
       <c r="D679" s="26">
         <v>3.1</v>
       </c>
       <c r="E679" s="27">
-        <v>48.05</v>
+        <v>44.95</v>
       </c>
     </row>
     <row r="680" spans="1:5" x14ac:dyDescent="0.25">
@@ -12769,16 +12795,16 @@
         <v>682</v>
       </c>
       <c r="B680" s="24">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C680" s="25">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="D680" s="26">
         <v>5.73</v>
       </c>
       <c r="E680" s="27">
-        <v>77.38</v>
+        <v>71.650000000000006</v>
       </c>
     </row>
     <row r="681" spans="1:5" x14ac:dyDescent="0.25">
@@ -12904,16 +12930,16 @@
         <v>691</v>
       </c>
       <c r="B689" s="24">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C689" s="25">
-        <v>87.5</v>
+        <v>88</v>
       </c>
       <c r="D689" s="26">
         <v>3.1</v>
       </c>
       <c r="E689" s="27">
-        <v>271.25</v>
+        <v>272.8</v>
       </c>
     </row>
     <row r="690" spans="1:5" x14ac:dyDescent="0.25">
@@ -12975,13 +13001,13 @@
         <v>96</v>
       </c>
       <c r="C693" s="25">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="D693" s="26">
         <v>3.75</v>
       </c>
       <c r="E693" s="27">
-        <v>52.5</v>
+        <v>75</v>
       </c>
     </row>
     <row r="694" spans="1:5" x14ac:dyDescent="0.25">
@@ -13090,16 +13116,16 @@
         <v>703</v>
       </c>
       <c r="B701" s="24">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C701" s="25">
-        <v>-0.5</v>
+        <v>0.5</v>
       </c>
       <c r="D701" s="26">
         <v>2.76</v>
       </c>
       <c r="E701" s="27">
-        <v>-1.38</v>
+        <v>1.38</v>
       </c>
     </row>
     <row r="702" spans="1:5" x14ac:dyDescent="0.25">
@@ -13141,17 +13167,11 @@
         <v>706</v>
       </c>
       <c r="B704" s="24">
-        <v>54</v>
-      </c>
-      <c r="C704" s="25">
-        <v>0.5</v>
-      </c>
-      <c r="D704" s="26">
-        <v>4</v>
-      </c>
-      <c r="E704" s="27">
-        <v>2</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="C704" s="28"/>
+      <c r="D704" s="29"/>
+      <c r="E704" s="28"/>
     </row>
     <row r="705" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A705" s="23" t="s">
@@ -13721,16 +13741,16 @@
         <v>750</v>
       </c>
       <c r="B748" s="24">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C748" s="25">
-        <v>3.75</v>
+        <v>2.75</v>
       </c>
       <c r="D748" s="26">
         <v>2.5</v>
       </c>
       <c r="E748" s="27">
-        <v>9.3800000000000008</v>
+        <v>6.88</v>
       </c>
     </row>
     <row r="749" spans="1:5" x14ac:dyDescent="0.25">
@@ -13805,10 +13825,10 @@
         <v>756</v>
       </c>
       <c r="B754" s="24">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C754" s="25">
-        <v>-1030.2</v>
+        <v>-1027.2</v>
       </c>
       <c r="D754" s="29"/>
       <c r="E754" s="28"/>
@@ -13819,11 +13839,11 @@
       </c>
       <c r="B755" s="31"/>
       <c r="C755" s="32">
-        <v>15983.49</v>
+        <v>15885.93</v>
       </c>
       <c r="D755" s="33"/>
       <c r="E755" s="34">
-        <v>34435.31</v>
+        <v>34385.199999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>